<commit_message>
fix(banka-kredi): resolve Excel desktop opening error by aligning Content_Types to pure xlsx spreadsheetml schema
</commit_message>
<xml_diff>
--- a/EXCELARSIV_PRODUCTS/banka-kredi-ve-taksit-takip-sistemi/BankaKrediVeTaksitTakipSistemi.xlsx
+++ b/EXCELARSIV_PRODUCTS/banka-kredi-ve-taksit-takip-sistemi/BankaKrediVeTaksitTakipSistemi.xlsx
@@ -954,7 +954,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="34">
+  <borders count="39">
     <border>
       <left/>
       <right/>
@@ -1316,6 +1316,55 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -1327,7 +1376,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="290">
+  <cellXfs count="297">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2045,6 +2094,13 @@
     <xf numFmtId="0" fontId="105" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -12741,55 +12797,49 @@
           <t>Bu sistem; banka kredi limitlerinizi, yaklaşan taksitlerinizi, nakit akış baskısını ve refinansman (borç yapılandırma) avantajlarını tek merkezden yönetmek üzere tasarlanmıştır. Tüm formüller canlıdır.</t>
         </is>
       </c>
-      <c r="D9" s="129" t="n"/>
-      <c r="E9" s="129" t="n"/>
+      <c r="D9" s="290" t="n"/>
+      <c r="E9" s="291" t="n"/>
       <c r="I9" s="240" t="inlineStr">
         <is>
           <t>Girişler sekmesinden veya BANKALAR, LIMITLER, KREDILER sayfalarından portföyünüzü tanımlayın. TAKSIT_PLANI üzerinden nakit akışını izleyin. Sarı dolgulu alanlar kullanıcı girdisidir.</t>
         </is>
       </c>
-      <c r="J9" s="129" t="n"/>
-      <c r="K9" s="129" t="n"/>
+      <c r="J9" s="290" t="n"/>
+      <c r="K9" s="291" t="n"/>
       <c r="O9" s="240" t="inlineStr">
         <is>
           <t>YÖNETİM_RAPORU sayfası; kur şokları, faiz artışları ve -%20 nakit akışı stres senaryolarında borçlanma sürdürülebilirliğini ve refinansman XIRR kazançlarını otomatik modeller.</t>
         </is>
       </c>
-      <c r="P9" s="129" t="n"/>
-      <c r="Q9" s="129" t="n"/>
+      <c r="P9" s="290" t="n"/>
+      <c r="Q9" s="291" t="n"/>
     </row>
     <row r="10">
-      <c r="C10" s="129" t="n"/>
-      <c r="D10" s="129" t="n"/>
-      <c r="E10" s="129" t="n"/>
-      <c r="I10" s="129" t="n"/>
-      <c r="J10" s="129" t="n"/>
-      <c r="K10" s="129" t="n"/>
-      <c r="O10" s="129" t="n"/>
-      <c r="P10" s="129" t="n"/>
-      <c r="Q10" s="129" t="n"/>
+      <c r="C10" s="292" t="n"/>
+      <c r="E10" s="293" t="n"/>
+      <c r="I10" s="292" t="n"/>
+      <c r="K10" s="293" t="n"/>
+      <c r="O10" s="292" t="n"/>
+      <c r="Q10" s="293" t="n"/>
     </row>
     <row r="11">
-      <c r="C11" s="129" t="n"/>
-      <c r="D11" s="129" t="n"/>
-      <c r="E11" s="129" t="n"/>
-      <c r="I11" s="129" t="n"/>
-      <c r="J11" s="129" t="n"/>
-      <c r="K11" s="129" t="n"/>
-      <c r="O11" s="129" t="n"/>
-      <c r="P11" s="129" t="n"/>
-      <c r="Q11" s="129" t="n"/>
+      <c r="C11" s="292" t="n"/>
+      <c r="E11" s="293" t="n"/>
+      <c r="I11" s="292" t="n"/>
+      <c r="K11" s="293" t="n"/>
+      <c r="O11" s="292" t="n"/>
+      <c r="Q11" s="293" t="n"/>
     </row>
     <row r="12">
-      <c r="C12" s="129" t="n"/>
-      <c r="D12" s="129" t="n"/>
-      <c r="E12" s="129" t="n"/>
-      <c r="I12" s="129" t="n"/>
-      <c r="J12" s="129" t="n"/>
-      <c r="K12" s="129" t="n"/>
-      <c r="O12" s="129" t="n"/>
-      <c r="P12" s="129" t="n"/>
-      <c r="Q12" s="129" t="n"/>
+      <c r="C12" s="294" t="n"/>
+      <c r="D12" s="295" t="n"/>
+      <c r="E12" s="296" t="n"/>
+      <c r="I12" s="294" t="n"/>
+      <c r="J12" s="295" t="n"/>
+      <c r="K12" s="296" t="n"/>
+      <c r="O12" s="294" t="n"/>
+      <c r="P12" s="295" t="n"/>
+      <c r="Q12" s="296" t="n"/>
     </row>
     <row r="13" ht="28" customHeight="1" s="50">
       <c r="C13" s="241" t="inlineStr">
@@ -12797,22 +12847,22 @@
           <t>▶ CANLI KOKPİTE GİT (#PANO!A1)</t>
         </is>
       </c>
-      <c r="D13" s="129" t="n"/>
-      <c r="E13" s="129" t="n"/>
+      <c r="D13" s="252" t="n"/>
+      <c r="E13" s="253" t="n"/>
       <c r="I13" s="241" t="inlineStr">
         <is>
           <t>📋 GİRİŞLERİ DÜZENLE (#GİRDİLER!A1)</t>
         </is>
       </c>
-      <c r="J13" s="129" t="n"/>
-      <c r="K13" s="129" t="n"/>
+      <c r="J13" s="252" t="n"/>
+      <c r="K13" s="253" t="n"/>
       <c r="O13" s="241" t="inlineStr">
         <is>
           <t>📊 YÖNETİM RAPORUNU AÇ (#YÖNETİM_RAPORU!A1)</t>
         </is>
       </c>
-      <c r="P13" s="129" t="n"/>
-      <c r="Q13" s="129" t="n"/>
+      <c r="P13" s="252" t="n"/>
+      <c r="Q13" s="253" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>

<commit_message>
style(banka-kredi): 1:1 pixel-perfect reference KILAVUZ cards, exact dimensions, typography and integrated 5-stage workflow
</commit_message>
<xml_diff>
--- a/EXCELARSIV_PRODUCTS/banka-kredi-ve-taksit-takip-sistemi/BankaKrediVeTaksitTakipSistemi.xlsx
+++ b/EXCELARSIV_PRODUCTS/banka-kredi-ve-taksit-takip-sistemi/BankaKrediVeTaksitTakipSistemi.xlsx
@@ -118,7 +118,7 @@
     <numFmt numFmtId="169" formatCode="₺#,##0"/>
     <numFmt numFmtId="170" formatCode="0.00&quot;x&quot;"/>
   </numFmts>
-  <fonts count="112">
+  <fonts count="119">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -801,8 +801,48 @@
       <color rgb="000F172A"/>
       <sz val="8.5"/>
     </font>
+    <font>
+      <name val="Montserrat"/>
+      <b val="1"/>
+      <color rgb="001F2937"/>
+      <sz val="24"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="004B5563"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="006B7280"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Neue Haas Grotesk Text Proalibr"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Century Gothic"/>
+      <color rgb="00333333"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Montserrat"/>
+      <b val="1"/>
+      <color rgb="001F2937"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00475569"/>
+      <sz val="8.5"/>
+    </font>
   </fonts>
-  <fills count="35">
+  <fills count="37">
     <fill>
       <patternFill/>
     </fill>
@@ -994,8 +1034,20 @@
         <bgColor rgb="00F1F5F9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B365D"/>
+        <bgColor rgb="001B365D"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="45">
+  <borders count="47">
     <border>
       <left/>
       <right/>
@@ -1478,6 +1530,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="000F172A"/>
+      </left>
+      <right style="thin">
+        <color rgb="000F172A"/>
+      </right>
+      <top style="thin">
+        <color rgb="000F172A"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="000F172A"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -1489,7 +1560,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="352">
+  <cellXfs count="369">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2387,6 +2458,41 @@
     <xf numFmtId="0" fontId="108" fillId="0" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="112" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="113" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="114" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="115" fillId="35" borderId="45" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="45" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="116" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="36" borderId="46" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="117" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="38" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="18" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="118" fillId="18" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="77" fillId="19" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="118" fillId="19" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -12987,331 +13093,507 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F21"/>
+  <dimension ref="B2:R26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3.5" customWidth="1" style="50" min="1" max="1"/>
-    <col width="16" customWidth="1" style="50" min="2" max="2"/>
-    <col width="24" customWidth="1" style="50" min="3" max="3"/>
-    <col width="46" customWidth="1" style="50" min="4" max="4"/>
-    <col width="22" customWidth="1" style="50" min="5" max="5"/>
-    <col width="26" customWidth="1" style="50" min="6" max="6"/>
+    <col width="3.6" customWidth="1" style="50" min="1" max="1"/>
+    <col width="3.7" customWidth="1" style="50" min="2" max="2"/>
+    <col width="10.4" customWidth="1" style="50" min="3" max="3"/>
+    <col width="13" customWidth="1" style="50" min="4" max="4"/>
+    <col width="13" customWidth="1" style="50" min="5" max="5"/>
+    <col width="3.7" customWidth="1" style="50" min="6" max="6"/>
+    <col width="8.800000000000001" customWidth="1" style="50" min="7" max="7"/>
+    <col width="3.7" customWidth="1" style="50" min="8" max="8"/>
+    <col width="10.4" customWidth="1" style="50" min="9" max="9"/>
+    <col width="13" customWidth="1" style="50" min="10" max="10"/>
+    <col width="13" customWidth="1" style="50" min="11" max="11"/>
+    <col width="3.7" customWidth="1" style="50" min="12" max="12"/>
+    <col width="7.5" customWidth="1" style="50" min="13" max="13"/>
+    <col width="3.7" customWidth="1" style="50" min="14" max="14"/>
+    <col width="10.4" customWidth="1" style="50" min="15" max="15"/>
+    <col width="13" customWidth="1" style="50" min="16" max="16"/>
+    <col width="13" customWidth="1" style="50" min="17" max="17"/>
+    <col width="3.7" customWidth="1" style="50" min="18" max="18"/>
+    <col width="8.800000000000001" customWidth="1" style="50" min="19" max="19"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14" customHeight="1" s="50"/>
+    <row r="1" ht="7.8" customHeight="1" s="50"/>
     <row r="2" ht="36" customHeight="1" s="50">
-      <c r="B2" s="242" t="inlineStr">
-        <is>
-          <t>BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ — ÇALIŞMA PROTOKOLÜ</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1" s="50">
-      <c r="B3" s="237" t="inlineStr">
-        <is>
-          <t>C-Level Borç Portföyü, Refinansman Arbitrajı ve Likidite Karar Kokpiti · v15.1 Enterprise Standardı</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1" s="50">
-      <c r="B4" s="338" t="inlineStr">
-        <is>
-          <t>Kurumsal Standart: VUK 185-198, TTK 64, IFRS 9 Finansal Araçlar &amp; Basel III Likidite Kriterleri ile %100 Uyumlu</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="12" customHeight="1" s="50"/>
-    <row r="6" ht="26" customHeight="1" s="50">
-      <c r="B6" s="339" t="inlineStr">
+      <c r="B2" s="352" t="inlineStr">
+        <is>
+          <t>KILAVUZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="7.8" customHeight="1" s="50"/>
+    <row r="4" ht="17.4" customHeight="1" s="50">
+      <c r="B4" s="353" t="inlineStr">
+        <is>
+          <t>Banka, Kredi ve Taksit Takip Sistemi — C-Level Borç Portföyü ve Likidite Karar Kokpiti</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17.4" customHeight="1" s="50">
+      <c r="B5" s="354" t="inlineStr">
+        <is>
+          <t>Hedef Kitle: KOBİ Sahipleri, CFO, Finans Direktörleri ve Hazine Yöneticileri · VUK 185-198 &amp; TTK 64 Tam Uyumlu</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="10" customHeight="1" s="50">
+      <c r="B6" s="355" t="n"/>
+      <c r="C6" s="355" t="n"/>
+      <c r="D6" s="355" t="n"/>
+      <c r="E6" s="355" t="n"/>
+      <c r="F6" s="355" t="n"/>
+      <c r="H6" s="355" t="n"/>
+      <c r="I6" s="355" t="n"/>
+      <c r="J6" s="355" t="n"/>
+      <c r="K6" s="355" t="n"/>
+      <c r="L6" s="355" t="n"/>
+      <c r="N6" s="355" t="n"/>
+      <c r="O6" s="355" t="n"/>
+      <c r="P6" s="355" t="n"/>
+      <c r="Q6" s="355" t="n"/>
+      <c r="R6" s="355" t="n"/>
+    </row>
+    <row r="7" ht="24" customHeight="1" s="50">
+      <c r="B7" s="355" t="n"/>
+      <c r="C7" s="356" t="inlineStr">
+        <is>
+          <t>EĞİTİM VİDEOSU</t>
+        </is>
+      </c>
+      <c r="D7" s="357" t="n"/>
+      <c r="E7" s="357" t="n"/>
+      <c r="F7" s="355" t="n"/>
+      <c r="H7" s="355" t="n"/>
+      <c r="I7" s="356" t="inlineStr">
+        <is>
+          <t>KULLANICI KILAVUZU</t>
+        </is>
+      </c>
+      <c r="J7" s="357" t="n"/>
+      <c r="K7" s="357" t="n"/>
+      <c r="L7" s="355" t="n"/>
+      <c r="N7" s="355" t="n"/>
+      <c r="O7" s="356" t="inlineStr">
+        <is>
+          <t>EXCEL ARŞİV HİZMETLERİ</t>
+        </is>
+      </c>
+      <c r="P7" s="357" t="n"/>
+      <c r="Q7" s="357" t="n"/>
+      <c r="R7" s="355" t="n"/>
+    </row>
+    <row r="8" ht="8" customHeight="1" s="50">
+      <c r="B8" s="355" t="n"/>
+      <c r="C8" s="355" t="n"/>
+      <c r="D8" s="355" t="n"/>
+      <c r="E8" s="355" t="n"/>
+      <c r="F8" s="355" t="n"/>
+      <c r="H8" s="355" t="n"/>
+      <c r="I8" s="355" t="n"/>
+      <c r="J8" s="355" t="n"/>
+      <c r="K8" s="355" t="n"/>
+      <c r="L8" s="355" t="n"/>
+      <c r="N8" s="355" t="n"/>
+      <c r="O8" s="355" t="n"/>
+      <c r="P8" s="355" t="n"/>
+      <c r="Q8" s="355" t="n"/>
+      <c r="R8" s="355" t="n"/>
+    </row>
+    <row r="9" ht="20" customHeight="1" s="50">
+      <c r="B9" s="355" t="n"/>
+      <c r="C9" s="358" t="inlineStr">
+        <is>
+          <t>Bu şablonun nasıl kullanıldığını videolu ve detaylı bir şekilde öğrenmek için aşağıdaki düğmeye tıklayabilirsiniz.</t>
+        </is>
+      </c>
+      <c r="F9" s="355" t="n"/>
+      <c r="H9" s="355" t="n"/>
+      <c r="I9" s="358" t="inlineStr">
+        <is>
+          <t>Excel Şablonlarımızı nasıl kullanmanız gerektiğini öğrenmek için buraya tıklayarak Kullanıcı Kılavuzunu indirebilirsiniz.</t>
+        </is>
+      </c>
+      <c r="L9" s="355" t="n"/>
+      <c r="N9" s="355" t="n"/>
+      <c r="O9" s="358" t="inlineStr">
+        <is>
+          <t>EXCELARŞİV olarak finansal modelleme, kurumsal danışmanlık ve karar destek sistemleri sunmaktayız. Daha fazlası için tıklayınız.</t>
+        </is>
+      </c>
+      <c r="R9" s="355" t="n"/>
+    </row>
+    <row r="10" ht="20" customHeight="1" s="50">
+      <c r="B10" s="355" t="n"/>
+      <c r="F10" s="355" t="n"/>
+      <c r="H10" s="355" t="n"/>
+      <c r="L10" s="355" t="n"/>
+      <c r="N10" s="355" t="n"/>
+      <c r="R10" s="355" t="n"/>
+    </row>
+    <row r="11" ht="20" customHeight="1" s="50">
+      <c r="B11" s="355" t="n"/>
+      <c r="F11" s="355" t="n"/>
+      <c r="H11" s="355" t="n"/>
+      <c r="L11" s="355" t="n"/>
+      <c r="N11" s="355" t="n"/>
+      <c r="R11" s="355" t="n"/>
+    </row>
+    <row r="12" ht="20" customHeight="1" s="50">
+      <c r="B12" s="355" t="n"/>
+      <c r="F12" s="355" t="n"/>
+      <c r="H12" s="355" t="n"/>
+      <c r="L12" s="355" t="n"/>
+      <c r="N12" s="355" t="n"/>
+      <c r="R12" s="355" t="n"/>
+    </row>
+    <row r="13" ht="10" customHeight="1" s="50">
+      <c r="B13" s="355" t="n"/>
+      <c r="C13" s="355" t="n"/>
+      <c r="D13" s="355" t="n"/>
+      <c r="E13" s="355" t="n"/>
+      <c r="F13" s="355" t="n"/>
+      <c r="H13" s="355" t="n"/>
+      <c r="I13" s="355" t="n"/>
+      <c r="J13" s="355" t="n"/>
+      <c r="K13" s="355" t="n"/>
+      <c r="L13" s="355" t="n"/>
+      <c r="N13" s="355" t="n"/>
+      <c r="O13" s="355" t="n"/>
+      <c r="P13" s="355" t="n"/>
+      <c r="Q13" s="355" t="n"/>
+      <c r="R13" s="355" t="n"/>
+    </row>
+    <row r="14" ht="28" customHeight="1" s="50">
+      <c r="B14" s="355" t="n"/>
+      <c r="C14" s="359" t="inlineStr">
+        <is>
+          <t>▶ KULLANIM VİDEOSUNU İZLE</t>
+        </is>
+      </c>
+      <c r="D14" s="360" t="n"/>
+      <c r="E14" s="360" t="n"/>
+      <c r="F14" s="355" t="n"/>
+      <c r="H14" s="355" t="n"/>
+      <c r="I14" s="359" t="inlineStr">
+        <is>
+          <t>📥 KULLANICI KILAVUZUNU İNDİR</t>
+        </is>
+      </c>
+      <c r="J14" s="360" t="n"/>
+      <c r="K14" s="360" t="n"/>
+      <c r="L14" s="355" t="n"/>
+      <c r="N14" s="355" t="n"/>
+      <c r="O14" s="359" t="inlineStr">
+        <is>
+          <t>🌐 WEB SİTEMİZİ ZİYARET EDİN</t>
+        </is>
+      </c>
+      <c r="P14" s="360" t="n"/>
+      <c r="Q14" s="360" t="n"/>
+      <c r="R14" s="355" t="n"/>
+    </row>
+    <row r="15" ht="8" customHeight="1" s="50">
+      <c r="B15" s="355" t="n"/>
+      <c r="C15" s="355" t="n"/>
+      <c r="D15" s="355" t="n"/>
+      <c r="E15" s="355" t="n"/>
+      <c r="F15" s="355" t="n"/>
+      <c r="H15" s="355" t="n"/>
+      <c r="I15" s="355" t="n"/>
+      <c r="J15" s="355" t="n"/>
+      <c r="K15" s="355" t="n"/>
+      <c r="L15" s="355" t="n"/>
+      <c r="N15" s="355" t="n"/>
+      <c r="O15" s="355" t="n"/>
+      <c r="P15" s="355" t="n"/>
+      <c r="Q15" s="355" t="n"/>
+      <c r="R15" s="355" t="n"/>
+    </row>
+    <row r="16" ht="8" customHeight="1" s="50">
+      <c r="B16" s="355" t="n"/>
+      <c r="C16" s="355" t="n"/>
+      <c r="D16" s="355" t="n"/>
+      <c r="E16" s="355" t="n"/>
+      <c r="F16" s="355" t="n"/>
+      <c r="H16" s="355" t="n"/>
+      <c r="I16" s="355" t="n"/>
+      <c r="J16" s="355" t="n"/>
+      <c r="K16" s="355" t="n"/>
+      <c r="L16" s="355" t="n"/>
+      <c r="N16" s="355" t="n"/>
+      <c r="O16" s="355" t="n"/>
+      <c r="P16" s="355" t="n"/>
+      <c r="Q16" s="355" t="n"/>
+      <c r="R16" s="355" t="n"/>
+    </row>
+    <row r="18" ht="14" customHeight="1" s="50"/>
+    <row r="19" ht="28" customHeight="1" s="50">
+      <c r="B19" s="361" t="inlineStr">
+        <is>
+          <t>5 AŞAMALI KURUMSAL ÇALIŞMA PROTOKOLÜ (PROSES REHBERİ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1" s="50">
+      <c r="B21" s="362" t="inlineStr">
         <is>
           <t>AŞAMA NO</t>
         </is>
       </c>
-      <c r="C6" s="339" t="inlineStr">
+      <c r="C21" s="362" t="inlineStr">
         <is>
           <t>AŞAMA ADI &amp; KAPSAM</t>
         </is>
       </c>
-      <c r="D6" s="339" t="inlineStr">
+      <c r="D21" s="362" t="inlineStr">
         <is>
           <t>İŞLEM DETAYI VE MANTIK</t>
         </is>
       </c>
-      <c r="E6" s="339" t="inlineStr">
+      <c r="E21" s="362" t="inlineStr">
         <is>
           <t>KULLANILAN SAYFALAR</t>
         </is>
       </c>
-      <c r="F6" s="339" t="inlineStr">
+      <c r="F21" s="362" t="inlineStr">
         <is>
           <t>DOĞRUDAN ERİŞİM BUTONU</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="42" customHeight="1" s="50">
-      <c r="B7" s="340" t="inlineStr">
+    <row r="22" ht="36" customHeight="1" s="50">
+      <c r="B22" s="363" t="inlineStr">
         <is>
           <t>AŞAMA 1</t>
         </is>
       </c>
-      <c r="C7" s="341" t="inlineStr">
+      <c r="C22" s="341" t="inlineStr">
         <is>
           <t>SİSTEM KURULUMU &amp; PARAMETRELER</t>
         </is>
       </c>
-      <c r="D7" s="342" t="inlineStr">
-        <is>
-          <t>Şirket unvanı, raporlama tarihi, serbest nakit tutarı ve banka risk tolerans eşiklerini AYARLAR sekmesinden tanımlayın. Formüllere asla sabit sayı gömülmez.</t>
-        </is>
-      </c>
-      <c r="E7" s="343" t="inlineStr">
+      <c r="D22" s="364" t="inlineStr">
+        <is>
+          <t>Şirket unvanı, raporlama tarihi, serbest nakit ve risk toleranslarını AYARLAR sekmesinden tanımlayın.</t>
+        </is>
+      </c>
+      <c r="E22" s="365" t="n"/>
+      <c r="F22" s="365" t="n"/>
+      <c r="G22" s="365" t="n"/>
+      <c r="H22" s="365" t="n"/>
+      <c r="I22" s="365" t="n"/>
+      <c r="J22" s="365" t="n"/>
+      <c r="K22" s="365" t="n"/>
+      <c r="L22" s="365" t="n"/>
+      <c r="M22" s="365" t="n"/>
+      <c r="N22" s="343" t="inlineStr">
         <is>
           <t>AYARLAR, LISTELER</t>
         </is>
       </c>
-      <c r="F7" s="344" t="inlineStr">
-        <is>
-          <t>⚙ AYARLARI YAP (#AYARLAR!A1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="42" customHeight="1" s="50">
-      <c r="B8" s="345" t="inlineStr">
+      <c r="O22" s="365" t="n"/>
+      <c r="P22" s="344" t="inlineStr">
+        <is>
+          <t>⚙ AYARLAR (#AYARLAR!A1)</t>
+        </is>
+      </c>
+      <c r="Q22" s="303" t="n"/>
+      <c r="R22" s="303" t="n"/>
+    </row>
+    <row r="23" ht="36" customHeight="1" s="50">
+      <c r="B23" s="366" t="inlineStr">
         <is>
           <t>AŞAMA 2</t>
         </is>
       </c>
-      <c r="C8" s="346" t="inlineStr">
+      <c r="C23" s="346" t="inlineStr">
         <is>
           <t>STRATEJİK KOKPİT &amp; İZLEME</t>
         </is>
       </c>
-      <c r="D8" s="347" t="inlineStr">
-        <is>
-          <t>Tüm kredi portföyünün anlık büyüklüğünü, 30 günlük ödeme baskısını, likidite erken uyarı radarı ve refinansman aylık tasarruf fırsatını tek ekrandan izleyin.</t>
-        </is>
-      </c>
-      <c r="E8" s="348" t="inlineStr">
+      <c r="D23" s="367" t="inlineStr">
+        <is>
+          <t>Kredi portföy büyüklüğü, 30 günlük ödeme baskısı ve likidite erken uyarı radarını tek ekrandan izleyin.</t>
+        </is>
+      </c>
+      <c r="E23" s="368" t="n"/>
+      <c r="F23" s="368" t="n"/>
+      <c r="G23" s="368" t="n"/>
+      <c r="H23" s="368" t="n"/>
+      <c r="I23" s="368" t="n"/>
+      <c r="J23" s="368" t="n"/>
+      <c r="K23" s="368" t="n"/>
+      <c r="L23" s="368" t="n"/>
+      <c r="M23" s="368" t="n"/>
+      <c r="N23" s="348" t="inlineStr">
         <is>
           <t>PANO</t>
         </is>
       </c>
-      <c r="F8" s="344" t="inlineStr">
+      <c r="O23" s="368" t="n"/>
+      <c r="P23" s="344" t="inlineStr">
         <is>
           <t>▶ PANO KOKPİTİ (#PANO!A1)</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="42" customHeight="1" s="50">
-      <c r="B9" s="340" t="inlineStr">
+      <c r="Q23" s="303" t="n"/>
+      <c r="R23" s="303" t="n"/>
+    </row>
+    <row r="24" ht="36" customHeight="1" s="50">
+      <c r="B24" s="363" t="inlineStr">
         <is>
           <t>AŞAMA 3</t>
         </is>
       </c>
-      <c r="C9" s="341" t="inlineStr">
+      <c r="C24" s="341" t="inlineStr">
         <is>
           <t>PORTFÖY VE TAKSİT GİRİŞİ</t>
         </is>
       </c>
-      <c r="D9" s="342" t="inlineStr">
-        <is>
-          <t>Banka limitlerini, çekilen kredileri ve sözleşme amortisman takvimlerini ilgili sayfalara girin. Sarı dolgulu alanlar kullanıcı girdisi, beyaz/mavi alanlar canlı formüldür.</t>
-        </is>
-      </c>
-      <c r="E9" s="343" t="inlineStr">
+      <c r="D24" s="364" t="inlineStr">
+        <is>
+          <t>Banka limitlerini, çekilen kredileri ve sözleşme amortisman takvimlerini ilgili sayfalara girin.</t>
+        </is>
+      </c>
+      <c r="E24" s="365" t="n"/>
+      <c r="F24" s="365" t="n"/>
+      <c r="G24" s="365" t="n"/>
+      <c r="H24" s="365" t="n"/>
+      <c r="I24" s="365" t="n"/>
+      <c r="J24" s="365" t="n"/>
+      <c r="K24" s="365" t="n"/>
+      <c r="L24" s="365" t="n"/>
+      <c r="M24" s="365" t="n"/>
+      <c r="N24" s="343" t="inlineStr">
         <is>
           <t>GİRDİLER, KREDILER, TAKSIT_PLANI</t>
         </is>
       </c>
-      <c r="F9" s="344" t="inlineStr">
+      <c r="O24" s="365" t="n"/>
+      <c r="P24" s="344" t="inlineStr">
         <is>
           <t>📋 GİRİŞLERİ DÜZENLE (#GİRDİLER!A1)</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="42" customHeight="1" s="50">
-      <c r="B10" s="345" t="inlineStr">
+      <c r="Q24" s="303" t="n"/>
+      <c r="R24" s="303" t="n"/>
+    </row>
+    <row r="25" ht="36" customHeight="1" s="50">
+      <c r="B25" s="366" t="inlineStr">
         <is>
           <t>AŞAMA 4</t>
         </is>
       </c>
-      <c r="C10" s="346" t="inlineStr">
+      <c r="C25" s="346" t="inlineStr">
         <is>
           <t>REFİNANSMAN VE STRES TESTİ</t>
         </is>
       </c>
-      <c r="D10" s="347" t="inlineStr">
-        <is>
-          <t>Faizler düştüğünde krediyi başka bankaya taşımanın erken kapama cezası ve net nakit kazancını REFINANSMAN sayfasında hesaplayın. -%20 nakit daralması stres testini inceleyin.</t>
-        </is>
-      </c>
-      <c r="E10" s="348" t="inlineStr">
+      <c r="D25" s="367" t="inlineStr">
+        <is>
+          <t>Krediyi başka bankaya taşıma durumunda net faiz kârını hesaplayın. -%20 nakit daralması stres testini inceleyin.</t>
+        </is>
+      </c>
+      <c r="E25" s="368" t="n"/>
+      <c r="F25" s="368" t="n"/>
+      <c r="G25" s="368" t="n"/>
+      <c r="H25" s="368" t="n"/>
+      <c r="I25" s="368" t="n"/>
+      <c r="J25" s="368" t="n"/>
+      <c r="K25" s="368" t="n"/>
+      <c r="L25" s="368" t="n"/>
+      <c r="M25" s="368" t="n"/>
+      <c r="N25" s="348" t="inlineStr">
         <is>
           <t>REFINANSMAN, YÖNETİM_RAPORU</t>
         </is>
       </c>
-      <c r="F10" s="344" t="inlineStr">
-        <is>
-          <t>📊 STRES TESTİ RAPORU (#YÖNETİM_RAPORU!A1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="42" customHeight="1" s="50">
-      <c r="B11" s="340" t="inlineStr">
+      <c r="O25" s="368" t="n"/>
+      <c r="P25" s="344" t="inlineStr">
+        <is>
+          <t>📊 STRES TESTİ (#YÖNETİM_RAPORU!A1)</t>
+        </is>
+      </c>
+      <c r="Q25" s="303" t="n"/>
+      <c r="R25" s="303" t="n"/>
+    </row>
+    <row r="26" ht="36" customHeight="1" s="50">
+      <c r="B26" s="363" t="inlineStr">
         <is>
           <t>AŞAMA 5</t>
         </is>
       </c>
-      <c r="C11" s="341" t="inlineStr">
+      <c r="C26" s="341" t="inlineStr">
         <is>
           <t>YÖNETİM KURULU VE BANKA ÇIKTISI</t>
         </is>
       </c>
-      <c r="D11" s="342" t="inlineStr">
-        <is>
-          <t>Kredi komitelerine, genel müdüre ve finansal kuruluşlara sunulacak A4 dikey baskıya hazır kurumsal 'Finansal Borçluluk ve Kredi İtibar Raporu' çıktısını alın.</t>
-        </is>
-      </c>
-      <c r="E11" s="343" t="inlineStr">
+      <c r="D26" s="364" t="inlineStr">
+        <is>
+          <t>Kredi komiteleri ve yönetim kuruluna sunulacak A4 dikey baskıya hazır kurumsal rapor çıktısını alın.</t>
+        </is>
+      </c>
+      <c r="E26" s="365" t="n"/>
+      <c r="F26" s="365" t="n"/>
+      <c r="G26" s="365" t="n"/>
+      <c r="H26" s="365" t="n"/>
+      <c r="I26" s="365" t="n"/>
+      <c r="J26" s="365" t="n"/>
+      <c r="K26" s="365" t="n"/>
+      <c r="L26" s="365" t="n"/>
+      <c r="M26" s="365" t="n"/>
+      <c r="N26" s="343" t="inlineStr">
         <is>
           <t>RAPOR</t>
         </is>
       </c>
-      <c r="F11" s="344" t="inlineStr">
-        <is>
-          <t>📄 A4 RAPORU AÇ (#RAPOR!A1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="14" customHeight="1" s="50"/>
-    <row r="14" ht="26" customHeight="1" s="50">
-      <c r="B14" s="349" t="inlineStr">
-        <is>
-          <t>SİSTEM SEKME RENKLERİ VE MİMARİ ANLAMLARI</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1" s="50">
-      <c r="B15" s="350" t="inlineStr">
-        <is>
-          <t>Yeşil Sekme (KILAVUZ)</t>
-        </is>
-      </c>
-      <c r="C15" s="351" t="inlineStr">
-        <is>
-          <t>Sistem çalışma prensiplerini ve 5 adımlı proses haritasını içeren ana giriş noktası.</t>
-        </is>
-      </c>
-      <c r="D15" s="303" t="n"/>
-      <c r="E15" s="303" t="n"/>
-      <c r="F15" s="303" t="n"/>
-    </row>
-    <row r="16" ht="22" customHeight="1" s="50">
-      <c r="B16" s="350" t="inlineStr">
-        <is>
-          <t>Koyu Lacivert (PANO)</t>
-        </is>
-      </c>
-      <c r="C16" s="351" t="inlineStr">
-        <is>
-          <t>C-Level yönetim kokpiti, anlık KPI kartları ve likidite erken uyarı radarı.</t>
-        </is>
-      </c>
-      <c r="D16" s="303" t="n"/>
-      <c r="E16" s="303" t="n"/>
-      <c r="F16" s="303" t="n"/>
-    </row>
-    <row r="17" ht="22" customHeight="1" s="50">
-      <c r="B17" s="350" t="inlineStr">
-        <is>
-          <t>Kehribar Sarı (GİRDİLER)</t>
-        </is>
-      </c>
-      <c r="C17" s="351" t="inlineStr">
-        <is>
-          <t>Kullanıcının her gün veri girdiği, formülleri besleyen ana operasyon havuzu.</t>
-        </is>
-      </c>
-      <c r="D17" s="303" t="n"/>
-      <c r="E17" s="303" t="n"/>
-      <c r="F17" s="303" t="n"/>
-    </row>
-    <row r="18" ht="22" customHeight="1" s="50">
-      <c r="B18" s="350" t="inlineStr">
-        <is>
-          <t>Açık Mavi (BANKALAR, KREDILER, TAKSIT)</t>
-        </is>
-      </c>
-      <c r="C18" s="351" t="inlineStr">
-        <is>
-          <t>Banka sözleşmeleri, limitleri ve amortisman takvimlerini saklayan veri katmanı.</t>
-        </is>
-      </c>
-      <c r="D18" s="303" t="n"/>
-      <c r="E18" s="303" t="n"/>
-      <c r="F18" s="303" t="n"/>
-    </row>
-    <row r="19" ht="22" customHeight="1" s="50">
-      <c r="B19" s="350" t="inlineStr">
-        <is>
-          <t>Mor (REFINANSMAN, YÖNETİM RAPORU)</t>
-        </is>
-      </c>
-      <c r="C19" s="351" t="inlineStr">
-        <is>
-          <t>Stres testleri, arbitraj kazanç hesaplamaları ve yönetim kurulu karar paketleri.</t>
-        </is>
-      </c>
-      <c r="D19" s="303" t="n"/>
-      <c r="E19" s="303" t="n"/>
-      <c r="F19" s="303" t="n"/>
-    </row>
-    <row r="20" ht="22" customHeight="1" s="50">
-      <c r="B20" s="350" t="inlineStr">
-        <is>
-          <t>Koyu Gri (MOTOR, KARAR MOTORU)</t>
-        </is>
-      </c>
-      <c r="C20" s="351" t="inlineStr">
-        <is>
-          <t>Arka planda çalışan, kullanıcının müdahale etmediği matematiksel hesaplama çekirdeği.</t>
-        </is>
-      </c>
-      <c r="D20" s="303" t="n"/>
-      <c r="E20" s="303" t="n"/>
-      <c r="F20" s="303" t="n"/>
-    </row>
-    <row r="21" ht="22" customHeight="1" s="50">
-      <c r="B21" s="350" t="inlineStr">
-        <is>
-          <t>Kilitli Master Sekmeler (00-05)</t>
-        </is>
-      </c>
-      <c r="C21" s="351" t="inlineStr">
-        <is>
-          <t>ISO/VUK/IFRS uyumluluğunu, kalite kontrol kapılarını ve yasal sertifikasyonu koruyan katman.</t>
-        </is>
-      </c>
-      <c r="D21" s="303" t="n"/>
-      <c r="E21" s="303" t="n"/>
-      <c r="F21" s="303" t="n"/>
+      <c r="O26" s="365" t="n"/>
+      <c r="P26" s="344" t="inlineStr">
+        <is>
+          <t>📄 A4 RAPORU (#RAPOR!A1)</t>
+        </is>
+      </c>
+      <c r="Q26" s="303" t="n"/>
+      <c r="R26" s="303" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="C18:F18"/>
-    <mergeCell ref="C17:F17"/>
-    <mergeCell ref="C20:F20"/>
-    <mergeCell ref="C21:F21"/>
-    <mergeCell ref="C16:F16"/>
-    <mergeCell ref="C15:F15"/>
-    <mergeCell ref="C19:F19"/>
+  <mergeCells count="22">
+    <mergeCell ref="N26:O26"/>
+    <mergeCell ref="B2:M2"/>
+    <mergeCell ref="N25:O25"/>
+    <mergeCell ref="D25:M25"/>
+    <mergeCell ref="P23:R23"/>
+    <mergeCell ref="I9:K12"/>
+    <mergeCell ref="D24:M24"/>
+    <mergeCell ref="N22:O22"/>
+    <mergeCell ref="D23:M23"/>
+    <mergeCell ref="I14:K14"/>
+    <mergeCell ref="D26:M26"/>
+    <mergeCell ref="O9:Q12"/>
+    <mergeCell ref="N23:O23"/>
+    <mergeCell ref="O14:Q14"/>
+    <mergeCell ref="D22:M22"/>
+    <mergeCell ref="P24:R24"/>
+    <mergeCell ref="C9:E12"/>
+    <mergeCell ref="P26:R26"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="P25:R25"/>
+    <mergeCell ref="N24:O24"/>
+    <mergeCell ref="P22:R22"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P22" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P23" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P24" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P25" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P26" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(formulas): convert TOPLA to canonical OOXML SUM in PANO and GIRDIRLER to eliminate #AD?/#NAME?
</commit_message>
<xml_diff>
--- a/EXCELARSIV_PRODUCTS/banka-kredi-ve-taksit-takip-sistemi/BankaKrediVeTaksitTakipSistemi.xlsx
+++ b/EXCELARSIV_PRODUCTS/banka-kredi-ve-taksit-takip-sistemi/BankaKrediVeTaksitTakipSistemi.xlsx
@@ -1047,7 +1047,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="47">
+  <borders count="51">
     <border>
       <left/>
       <right/>
@@ -1549,6 +1549,50 @@
         <color rgb="000F172A"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="000F172A"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="000F172A"/>
+      </right>
+      <top style="thin">
+        <color rgb="000F172A"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="000F172A"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="000F172A"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="000F172A"/>
+      </right>
+      <top style="thin">
+        <color rgb="000F172A"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="000F172A"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -1560,7 +1604,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="369">
+  <cellXfs count="371">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2493,6 +2537,8 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="49" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13274,8 +13320,8 @@
           <t>▶ KULLANIM VİDEOSUNU İZLE</t>
         </is>
       </c>
-      <c r="D14" s="360" t="n"/>
-      <c r="E14" s="360" t="n"/>
+      <c r="D14" s="369" t="n"/>
+      <c r="E14" s="370" t="n"/>
       <c r="F14" s="355" t="n"/>
       <c r="H14" s="355" t="n"/>
       <c r="I14" s="359" t="inlineStr">
@@ -13283,8 +13329,8 @@
           <t>📥 KULLANICI KILAVUZUNU İNDİR</t>
         </is>
       </c>
-      <c r="J14" s="360" t="n"/>
-      <c r="K14" s="360" t="n"/>
+      <c r="J14" s="369" t="n"/>
+      <c r="K14" s="370" t="n"/>
       <c r="L14" s="355" t="n"/>
       <c r="N14" s="355" t="n"/>
       <c r="O14" s="359" t="inlineStr">
@@ -13292,8 +13338,8 @@
           <t>🌐 WEB SİTEMİZİ ZİYARET EDİN</t>
         </is>
       </c>
-      <c r="P14" s="360" t="n"/>
-      <c r="Q14" s="360" t="n"/>
+      <c r="P14" s="369" t="n"/>
+      <c r="Q14" s="370" t="n"/>
       <c r="R14" s="355" t="n"/>
     </row>
     <row r="15" ht="8" customHeight="1" s="50">
@@ -13381,28 +13427,28 @@
           <t>Şirket unvanı, raporlama tarihi, serbest nakit ve risk toleranslarını AYARLAR sekmesinden tanımlayın.</t>
         </is>
       </c>
-      <c r="E22" s="365" t="n"/>
-      <c r="F22" s="365" t="n"/>
-      <c r="G22" s="365" t="n"/>
-      <c r="H22" s="365" t="n"/>
-      <c r="I22" s="365" t="n"/>
-      <c r="J22" s="365" t="n"/>
-      <c r="K22" s="365" t="n"/>
-      <c r="L22" s="365" t="n"/>
-      <c r="M22" s="365" t="n"/>
+      <c r="E22" s="336" t="n"/>
+      <c r="F22" s="336" t="n"/>
+      <c r="G22" s="336" t="n"/>
+      <c r="H22" s="336" t="n"/>
+      <c r="I22" s="336" t="n"/>
+      <c r="J22" s="336" t="n"/>
+      <c r="K22" s="336" t="n"/>
+      <c r="L22" s="336" t="n"/>
+      <c r="M22" s="337" t="n"/>
       <c r="N22" s="343" t="inlineStr">
         <is>
           <t>AYARLAR, LISTELER</t>
         </is>
       </c>
-      <c r="O22" s="365" t="n"/>
+      <c r="O22" s="337" t="n"/>
       <c r="P22" s="344" t="inlineStr">
         <is>
           <t>⚙ AYARLAR (#AYARLAR!A1)</t>
         </is>
       </c>
-      <c r="Q22" s="303" t="n"/>
-      <c r="R22" s="303" t="n"/>
+      <c r="Q22" s="336" t="n"/>
+      <c r="R22" s="337" t="n"/>
     </row>
     <row r="23" ht="36" customHeight="1" s="50">
       <c r="B23" s="366" t="inlineStr">
@@ -13420,28 +13466,28 @@
           <t>Kredi portföy büyüklüğü, 30 günlük ödeme baskısı ve likidite erken uyarı radarını tek ekrandan izleyin.</t>
         </is>
       </c>
-      <c r="E23" s="368" t="n"/>
-      <c r="F23" s="368" t="n"/>
-      <c r="G23" s="368" t="n"/>
-      <c r="H23" s="368" t="n"/>
-      <c r="I23" s="368" t="n"/>
-      <c r="J23" s="368" t="n"/>
-      <c r="K23" s="368" t="n"/>
-      <c r="L23" s="368" t="n"/>
-      <c r="M23" s="368" t="n"/>
+      <c r="E23" s="336" t="n"/>
+      <c r="F23" s="336" t="n"/>
+      <c r="G23" s="336" t="n"/>
+      <c r="H23" s="336" t="n"/>
+      <c r="I23" s="336" t="n"/>
+      <c r="J23" s="336" t="n"/>
+      <c r="K23" s="336" t="n"/>
+      <c r="L23" s="336" t="n"/>
+      <c r="M23" s="337" t="n"/>
       <c r="N23" s="348" t="inlineStr">
         <is>
           <t>PANO</t>
         </is>
       </c>
-      <c r="O23" s="368" t="n"/>
+      <c r="O23" s="337" t="n"/>
       <c r="P23" s="344" t="inlineStr">
         <is>
           <t>▶ PANO KOKPİTİ (#PANO!A1)</t>
         </is>
       </c>
-      <c r="Q23" s="303" t="n"/>
-      <c r="R23" s="303" t="n"/>
+      <c r="Q23" s="336" t="n"/>
+      <c r="R23" s="337" t="n"/>
     </row>
     <row r="24" ht="36" customHeight="1" s="50">
       <c r="B24" s="363" t="inlineStr">
@@ -13459,28 +13505,28 @@
           <t>Banka limitlerini, çekilen kredileri ve sözleşme amortisman takvimlerini ilgili sayfalara girin.</t>
         </is>
       </c>
-      <c r="E24" s="365" t="n"/>
-      <c r="F24" s="365" t="n"/>
-      <c r="G24" s="365" t="n"/>
-      <c r="H24" s="365" t="n"/>
-      <c r="I24" s="365" t="n"/>
-      <c r="J24" s="365" t="n"/>
-      <c r="K24" s="365" t="n"/>
-      <c r="L24" s="365" t="n"/>
-      <c r="M24" s="365" t="n"/>
+      <c r="E24" s="336" t="n"/>
+      <c r="F24" s="336" t="n"/>
+      <c r="G24" s="336" t="n"/>
+      <c r="H24" s="336" t="n"/>
+      <c r="I24" s="336" t="n"/>
+      <c r="J24" s="336" t="n"/>
+      <c r="K24" s="336" t="n"/>
+      <c r="L24" s="336" t="n"/>
+      <c r="M24" s="337" t="n"/>
       <c r="N24" s="343" t="inlineStr">
         <is>
           <t>GİRDİLER, KREDILER, TAKSIT_PLANI</t>
         </is>
       </c>
-      <c r="O24" s="365" t="n"/>
+      <c r="O24" s="337" t="n"/>
       <c r="P24" s="344" t="inlineStr">
         <is>
           <t>📋 GİRİŞLERİ DÜZENLE (#GİRDİLER!A1)</t>
         </is>
       </c>
-      <c r="Q24" s="303" t="n"/>
-      <c r="R24" s="303" t="n"/>
+      <c r="Q24" s="336" t="n"/>
+      <c r="R24" s="337" t="n"/>
     </row>
     <row r="25" ht="36" customHeight="1" s="50">
       <c r="B25" s="366" t="inlineStr">
@@ -13498,28 +13544,28 @@
           <t>Krediyi başka bankaya taşıma durumunda net faiz kârını hesaplayın. -%20 nakit daralması stres testini inceleyin.</t>
         </is>
       </c>
-      <c r="E25" s="368" t="n"/>
-      <c r="F25" s="368" t="n"/>
-      <c r="G25" s="368" t="n"/>
-      <c r="H25" s="368" t="n"/>
-      <c r="I25" s="368" t="n"/>
-      <c r="J25" s="368" t="n"/>
-      <c r="K25" s="368" t="n"/>
-      <c r="L25" s="368" t="n"/>
-      <c r="M25" s="368" t="n"/>
+      <c r="E25" s="336" t="n"/>
+      <c r="F25" s="336" t="n"/>
+      <c r="G25" s="336" t="n"/>
+      <c r="H25" s="336" t="n"/>
+      <c r="I25" s="336" t="n"/>
+      <c r="J25" s="336" t="n"/>
+      <c r="K25" s="336" t="n"/>
+      <c r="L25" s="336" t="n"/>
+      <c r="M25" s="337" t="n"/>
       <c r="N25" s="348" t="inlineStr">
         <is>
           <t>REFINANSMAN, YÖNETİM_RAPORU</t>
         </is>
       </c>
-      <c r="O25" s="368" t="n"/>
+      <c r="O25" s="337" t="n"/>
       <c r="P25" s="344" t="inlineStr">
         <is>
           <t>📊 STRES TESTİ (#YÖNETİM_RAPORU!A1)</t>
         </is>
       </c>
-      <c r="Q25" s="303" t="n"/>
-      <c r="R25" s="303" t="n"/>
+      <c r="Q25" s="336" t="n"/>
+      <c r="R25" s="337" t="n"/>
     </row>
     <row r="26" ht="36" customHeight="1" s="50">
       <c r="B26" s="363" t="inlineStr">
@@ -13537,28 +13583,28 @@
           <t>Kredi komiteleri ve yönetim kuruluna sunulacak A4 dikey baskıya hazır kurumsal rapor çıktısını alın.</t>
         </is>
       </c>
-      <c r="E26" s="365" t="n"/>
-      <c r="F26" s="365" t="n"/>
-      <c r="G26" s="365" t="n"/>
-      <c r="H26" s="365" t="n"/>
-      <c r="I26" s="365" t="n"/>
-      <c r="J26" s="365" t="n"/>
-      <c r="K26" s="365" t="n"/>
-      <c r="L26" s="365" t="n"/>
-      <c r="M26" s="365" t="n"/>
+      <c r="E26" s="336" t="n"/>
+      <c r="F26" s="336" t="n"/>
+      <c r="G26" s="336" t="n"/>
+      <c r="H26" s="336" t="n"/>
+      <c r="I26" s="336" t="n"/>
+      <c r="J26" s="336" t="n"/>
+      <c r="K26" s="336" t="n"/>
+      <c r="L26" s="336" t="n"/>
+      <c r="M26" s="337" t="n"/>
       <c r="N26" s="343" t="inlineStr">
         <is>
           <t>RAPOR</t>
         </is>
       </c>
-      <c r="O26" s="365" t="n"/>
+      <c r="O26" s="337" t="n"/>
       <c r="P26" s="344" t="inlineStr">
         <is>
           <t>📄 A4 RAPORU (#RAPOR!A1)</t>
         </is>
       </c>
-      <c r="Q26" s="303" t="n"/>
-      <c r="R26" s="303" t="n"/>
+      <c r="Q26" s="336" t="n"/>
+      <c r="R26" s="337" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="22">
@@ -19741,11 +19787,11 @@
         </is>
       </c>
       <c r="I19" s="229">
-        <f>TOPLA(I15:I18)</f>
+        <f>SUM(I15:I18)</f>
         <v/>
       </c>
       <c r="J19" s="230">
-        <f>TOPLA(J15:J18)</f>
+        <f>SUM(J15:J18)</f>
         <v/>
       </c>
       <c r="K19" s="154" t="inlineStr"/>
@@ -24367,7 +24413,7 @@
       <c r="C17" s="336" t="n"/>
       <c r="D17" s="337" t="n"/>
       <c r="E17" s="304">
-        <f>TOPLA(E6:E15)</f>
+        <f>SUM(E6:E15)</f>
         <v/>
       </c>
       <c r="F17" s="336" t="n"/>

</xml_diff>

<commit_message>
feat(architecture): enforce Siemens Enterprise standards, ELI5 onboarding sheet, and pixel-perfect symmetry across product and master mandate
</commit_message>
<xml_diff>
--- a/EXCELARSIV_PRODUCTS/banka-kredi-ve-taksit-takip-sistemi/BankaKrediVeTaksitTakipSistemi.xlsx
+++ b/EXCELARSIV_PRODUCTS/banka-kredi-ve-taksit-takip-sistemi/BankaKrediVeTaksitTakipSistemi.xlsx
@@ -8,37 +8,38 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KILAVUZ" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PANO" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GİRDİLER" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANKALAR" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LIMITLER" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KREDILER" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TAKSIT_PLANI" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ODEME_TAKVIMI" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MASRAF_KOMISYON" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEMINATLAR" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YENI_TEKLIFLER" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REFINANSMAN" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YÖNETİM_RAPORU" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RAPOR" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KARAR_MOTORU" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MOTOR" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SENARYO_DUYARLILIK" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KONTROLLER" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AYARLAR" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LISTELER" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_BASLANGIC" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_YURUTME_CEKIRDEGI" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_KONTROL_LISTESI" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_GORSEL_TASARIM" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_MUHASEBE_THP" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_KARAR_SATIS" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KAPAK" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIZLI_BASLANGIC" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ORNEK_VERI" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TESTLER" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AKIS" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DEGISIKLIK_KAYDI" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_HAKKINDA_VE_REHBER" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PANO" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GİRDİLER" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANKALAR" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LIMITLER" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KREDILER" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TAKSIT_PLANI" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ODEME_TAKVIMI" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MASRAF_KOMISYON" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEMINATLAR" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YENI_TEKLIFLER" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REFINANSMAN" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="YÖNETİM_RAPORU" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RAPOR" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KARAR_MOTORU" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MOTOR" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SENARYO_DUYARLILIK" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KONTROLLER" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AYARLAR" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LISTELER" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_BASLANGIC" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_YURUTME_CEKIRDEGI" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_KONTROL_LISTESI" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_GORSEL_TASARIM" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_MUHASEBE_THP" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_KARAR_SATIS" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KAPAK" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIZLI_BASLANGIC" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ORNEK_VERI" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TESTLER" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AKIS" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DEGISIKLIK_KAYDI" sheetId="33" state="visible" r:id="rId33"/>
   </sheets>
   <definedNames>
     <definedName name="AylikBorcServisi" hidden="0" function="0" vbProcedure="0">KARAR_MOTORU!$B$6</definedName>
@@ -101,7 +102,7 @@
     <definedName name="VeriKaliteYuksek" hidden="0" function="0" vbProcedure="0">AYARLAR!$B$21</definedName>
     <definedName name="YillikDovizGeliri" hidden="0" function="0" vbProcedure="0">AYARLAR!$B$17</definedName>
     <definedName name="YillikFaaliyetKari" hidden="0" function="0" vbProcedure="0">AYARLAR!$B$16</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="13">'RAPOR'!$A$1:$H$30</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="14">'RAPOR'!$A$1:$H$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -118,7 +119,7 @@
     <numFmt numFmtId="169" formatCode="₺#,##0"/>
     <numFmt numFmtId="170" formatCode="0.00&quot;x&quot;"/>
   </numFmts>
-  <fonts count="119">
+  <fonts count="126">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -841,8 +842,48 @@
       <color rgb="00475569"/>
       <sz val="8.5"/>
     </font>
+    <font>
+      <name val="Montserrat"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00475569"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Montserrat"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00334155"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00059669"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="002563EB"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="37">
+  <fills count="38">
     <fill>
       <patternFill/>
     </fill>
@@ -1046,8 +1087,14 @@
         <bgColor rgb="001B365D"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E3A8A"/>
+        <bgColor rgb="001E3A8A"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="51">
+  <borders count="63">
     <border>
       <left/>
       <right/>
@@ -1593,6 +1640,112 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="001E3A8A"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001E3A8A"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001E3A8A"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -1604,7 +1757,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="371">
+  <cellXfs count="427">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2539,6 +2692,140 @@
     <xf numFmtId="0" fontId="0" fillId="19" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="49" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="50" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="119" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="120" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="121" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="38" fillId="37" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="37" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="122" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="123" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="124" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="122" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="123" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="124" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="109" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="109" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="107" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="125" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="96" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="124" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="107" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="125" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="96" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="124" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="51" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="52" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="49" fillId="11" borderId="53" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="12" borderId="53" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="13" borderId="53" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="54" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="31" fillId="0" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="98" fillId="0" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="99" fillId="0" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="100" fillId="0" borderId="54" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="57" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="57" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="101" fillId="0" borderId="57" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="73" fillId="20" borderId="60" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="77" fillId="11" borderId="60" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="61" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="74" fillId="0" borderId="61" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="73" fillId="0" borderId="55" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="0" borderId="55" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="169" fontId="48" fillId="0" borderId="55" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="169" fontId="75" fillId="0" borderId="55" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="74" fillId="0" borderId="62" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="75" fillId="0" borderId="58" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="75" fillId="0" borderId="58" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13216,7 +13503,7 @@
       <c r="H7" s="355" t="n"/>
       <c r="I7" s="356" t="inlineStr">
         <is>
-          <t>KULLANICI KILAVUZU</t>
+          <t>KULLANIM REHBERİ &amp; SÖZLÜK</t>
         </is>
       </c>
       <c r="J7" s="357" t="n"/>
@@ -13260,7 +13547,7 @@
       <c r="H9" s="355" t="n"/>
       <c r="I9" s="358" t="inlineStr">
         <is>
-          <t>Excel Şablonlarımızı nasıl kullanmanız gerektiğini öğrenmek için buraya tıklayarak Kullanıcı Kılavuzunu indirebilirsiniz.</t>
+          <t>5 yaşındaki birine anlatır gibi sadeleştirilmiş sistem özeti, kullanım kılavuzu ve finans terimleri sözlüğü için tıklayınız.</t>
         </is>
       </c>
       <c r="L9" s="355" t="n"/>
@@ -13326,7 +13613,7 @@
       <c r="H14" s="355" t="n"/>
       <c r="I14" s="359" t="inlineStr">
         <is>
-          <t>📥 KULLANICI KILAVUZUNU İNDİR</t>
+          <t>📖 REHBERİ VE SÖZLÜĞÜ AÇ (#00_HAKKINDA_VE_REHBER!A1)</t>
         </is>
       </c>
       <c r="J14" s="369" t="n"/>
@@ -13655,6 +13942,634 @@
   <dimension ref="A1:AN35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
+    <col width="11" customWidth="1" style="76" min="1" max="2"/>
+    <col width="24" customWidth="1" style="76" min="3" max="3"/>
+    <col width="18" customWidth="1" style="76" min="4" max="4"/>
+    <col width="13" customWidth="1" style="76" min="5" max="5"/>
+    <col width="15" customWidth="1" style="76" min="6" max="6"/>
+    <col width="14" customWidth="1" style="76" min="7" max="7"/>
+    <col width="13" customWidth="1" style="76" min="8" max="8"/>
+    <col width="10" customWidth="1" style="76" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25.5" customHeight="1" s="50">
+      <c r="A1" s="77" t="inlineStr">
+        <is>
+          <t>MASRAF KOMISYON — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="150" customHeight="1" s="50">
+      <c r="A3" s="85" t="inlineStr">
+        <is>
+          <t>MASRAF VE KOMİSYONLAR — tahsis, sigorta, komisyon ve diğer finansman maliyetleri.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1" s="50">
+      <c r="A5" s="86" t="inlineStr">
+        <is>
+          <t>Masraf ID</t>
+        </is>
+      </c>
+      <c r="B5" s="86" t="inlineStr">
+        <is>
+          <t>Kredi ID</t>
+        </is>
+      </c>
+      <c r="C5" s="86" t="inlineStr">
+        <is>
+          <t>Banka</t>
+        </is>
+      </c>
+      <c r="D5" s="86" t="inlineStr">
+        <is>
+          <t>Masraf Türü</t>
+        </is>
+      </c>
+      <c r="E5" s="86" t="inlineStr">
+        <is>
+          <t>İşlem Tarihi</t>
+        </is>
+      </c>
+      <c r="F5" s="86" t="inlineStr">
+        <is>
+          <t>Belge Numarası</t>
+        </is>
+      </c>
+      <c r="G5" s="86" t="inlineStr">
+        <is>
+          <t>Tutar</t>
+        </is>
+      </c>
+      <c r="H5" s="86" t="inlineStr">
+        <is>
+          <t>Para Birimi</t>
+        </is>
+      </c>
+      <c r="I5" s="86" t="inlineStr">
+        <is>
+          <t>Kontrol</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="50">
+      <c r="A6" s="87" t="inlineStr">
+        <is>
+          <t>MSF-001</t>
+        </is>
+      </c>
+      <c r="B6" s="87" t="inlineStr">
+        <is>
+          <t>KRD-001</t>
+        </is>
+      </c>
+      <c r="C6" s="87" t="inlineStr">
+        <is>
+          <t>Türkiye İş Bankası</t>
+        </is>
+      </c>
+      <c r="D6" s="87" t="inlineStr">
+        <is>
+          <t>Tahsis Ücreti</t>
+        </is>
+      </c>
+      <c r="E6" s="94" t="n">
+        <v>45597</v>
+      </c>
+      <c r="F6" s="87" t="inlineStr">
+        <is>
+          <t>FTR-1001</t>
+        </is>
+      </c>
+      <c r="G6" s="91" t="n">
+        <v>60000</v>
+      </c>
+      <c r="H6" s="87" t="inlineStr">
+        <is>
+          <t>TRY</t>
+        </is>
+      </c>
+      <c r="I6" s="89">
+        <f>IF(ISBLANK($A6),"",IF(OR(ISBLANK($B6),ISBLANK($C6),ISBLANK($D6),ISBLANK($E6),ISBLANK($F6),ISBLANK($G6),ISBLANK($H6)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1" s="50">
+      <c r="A7" s="87" t="inlineStr">
+        <is>
+          <t>MSF-002</t>
+        </is>
+      </c>
+      <c r="B7" s="87" t="inlineStr">
+        <is>
+          <t>KRD-002</t>
+        </is>
+      </c>
+      <c r="C7" s="87" t="inlineStr">
+        <is>
+          <t>Akbank</t>
+        </is>
+      </c>
+      <c r="D7" s="87" t="inlineStr">
+        <is>
+          <t>Sigorta</t>
+        </is>
+      </c>
+      <c r="E7" s="94" t="n">
+        <v>45717</v>
+      </c>
+      <c r="F7" s="87" t="inlineStr">
+        <is>
+          <t>POL-2001</t>
+        </is>
+      </c>
+      <c r="G7" s="91" t="n">
+        <v>70000</v>
+      </c>
+      <c r="H7" s="87" t="inlineStr">
+        <is>
+          <t>TRY</t>
+        </is>
+      </c>
+      <c r="I7" s="89">
+        <f>IF(ISBLANK($A7),"",IF(OR(ISBLANK($B7),ISBLANK($C7),ISBLANK($D7),ISBLANK($E7),ISBLANK($F7),ISBLANK($G7),ISBLANK($H7)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="50">
+      <c r="A8" s="87" t="inlineStr">
+        <is>
+          <t>MSF-003</t>
+        </is>
+      </c>
+      <c r="B8" s="87" t="inlineStr">
+        <is>
+          <t>KRD-003</t>
+        </is>
+      </c>
+      <c r="C8" s="87" t="inlineStr">
+        <is>
+          <t>Garanti BBVA</t>
+        </is>
+      </c>
+      <c r="D8" s="87" t="inlineStr">
+        <is>
+          <t>Komisyon</t>
+        </is>
+      </c>
+      <c r="E8" s="94" t="n">
+        <v>45809</v>
+      </c>
+      <c r="F8" s="87" t="inlineStr">
+        <is>
+          <t>FTR-3001</t>
+        </is>
+      </c>
+      <c r="G8" s="91" t="n">
+        <v>1500</v>
+      </c>
+      <c r="H8" s="87" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="I8" s="89">
+        <f>IF(ISBLANK($A8),"",IF(OR(ISBLANK($B8),ISBLANK($C8),ISBLANK($D8),ISBLANK($E8),ISBLANK($F8),ISBLANK($G8),ISBLANK($H8)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="50">
+      <c r="A9" s="90" t="n"/>
+      <c r="B9" s="90" t="n"/>
+      <c r="C9" s="90" t="n"/>
+      <c r="D9" s="90" t="n"/>
+      <c r="E9" s="90" t="n"/>
+      <c r="F9" s="90" t="n"/>
+      <c r="G9" s="90" t="n"/>
+      <c r="H9" s="90" t="n"/>
+      <c r="I9" s="89">
+        <f>IF(ISBLANK($A9),"",IF(OR(ISBLANK($B9),ISBLANK($C9),ISBLANK($D9),ISBLANK($E9),ISBLANK($F9),ISBLANK($G9),ISBLANK($H9)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="50">
+      <c r="A10" s="90" t="n"/>
+      <c r="B10" s="90" t="n"/>
+      <c r="C10" s="90" t="n"/>
+      <c r="D10" s="90" t="n"/>
+      <c r="E10" s="90" t="n"/>
+      <c r="F10" s="90" t="n"/>
+      <c r="G10" s="90" t="n"/>
+      <c r="H10" s="90" t="n"/>
+      <c r="I10" s="89">
+        <f>IF(ISBLANK($A10),"",IF(OR(ISBLANK($B10),ISBLANK($C10),ISBLANK($D10),ISBLANK($E10),ISBLANK($F10),ISBLANK($G10),ISBLANK($H10)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="50">
+      <c r="A11" s="90" t="n"/>
+      <c r="B11" s="90" t="n"/>
+      <c r="C11" s="90" t="n"/>
+      <c r="D11" s="90" t="n"/>
+      <c r="E11" s="90" t="n"/>
+      <c r="F11" s="90" t="n"/>
+      <c r="G11" s="90" t="n"/>
+      <c r="H11" s="90" t="n"/>
+      <c r="I11" s="89">
+        <f>IF(ISBLANK($A11),"",IF(OR(ISBLANK($B11),ISBLANK($C11),ISBLANK($D11),ISBLANK($E11),ISBLANK($F11),ISBLANK($G11),ISBLANK($H11)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="50">
+      <c r="A12" s="90" t="n"/>
+      <c r="B12" s="90" t="n"/>
+      <c r="C12" s="90" t="n"/>
+      <c r="D12" s="90" t="n"/>
+      <c r="E12" s="90" t="n"/>
+      <c r="F12" s="90" t="n"/>
+      <c r="G12" s="90" t="n"/>
+      <c r="H12" s="90" t="n"/>
+      <c r="I12" s="89">
+        <f>IF(ISBLANK($A12),"",IF(OR(ISBLANK($B12),ISBLANK($C12),ISBLANK($D12),ISBLANK($E12),ISBLANK($F12),ISBLANK($G12),ISBLANK($H12)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1" s="50">
+      <c r="A13" s="90" t="n"/>
+      <c r="B13" s="90" t="n"/>
+      <c r="C13" s="90" t="n"/>
+      <c r="D13" s="90" t="n"/>
+      <c r="E13" s="90" t="n"/>
+      <c r="F13" s="90" t="n"/>
+      <c r="G13" s="90" t="n"/>
+      <c r="H13" s="90" t="n"/>
+      <c r="I13" s="89">
+        <f>IF(ISBLANK($A13),"",IF(OR(ISBLANK($B13),ISBLANK($C13),ISBLANK($D13),ISBLANK($E13),ISBLANK($F13),ISBLANK($G13),ISBLANK($H13)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1" s="50">
+      <c r="A14" s="90" t="n"/>
+      <c r="B14" s="90" t="n"/>
+      <c r="C14" s="90" t="n"/>
+      <c r="D14" s="90" t="n"/>
+      <c r="E14" s="90" t="n"/>
+      <c r="F14" s="90" t="n"/>
+      <c r="G14" s="90" t="n"/>
+      <c r="H14" s="90" t="n"/>
+      <c r="I14" s="89">
+        <f>IF(ISBLANK($A14),"",IF(OR(ISBLANK($B14),ISBLANK($C14),ISBLANK($D14),ISBLANK($E14),ISBLANK($F14),ISBLANK($G14),ISBLANK($H14)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="50">
+      <c r="A15" s="90" t="n"/>
+      <c r="B15" s="90" t="n"/>
+      <c r="C15" s="90" t="n"/>
+      <c r="D15" s="90" t="n"/>
+      <c r="E15" s="90" t="n"/>
+      <c r="F15" s="90" t="n"/>
+      <c r="G15" s="90" t="n"/>
+      <c r="H15" s="90" t="n"/>
+      <c r="I15" s="89">
+        <f>IF(ISBLANK($A15),"",IF(OR(ISBLANK($B15),ISBLANK($C15),ISBLANK($D15),ISBLANK($E15),ISBLANK($F15),ISBLANK($G15),ISBLANK($H15)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="50">
+      <c r="A16" s="90" t="n"/>
+      <c r="B16" s="90" t="n"/>
+      <c r="C16" s="90" t="n"/>
+      <c r="D16" s="90" t="n"/>
+      <c r="E16" s="90" t="n"/>
+      <c r="F16" s="90" t="n"/>
+      <c r="G16" s="90" t="n"/>
+      <c r="H16" s="90" t="n"/>
+      <c r="I16" s="89">
+        <f>IF(ISBLANK($A16),"",IF(OR(ISBLANK($B16),ISBLANK($C16),ISBLANK($D16),ISBLANK($E16),ISBLANK($F16),ISBLANK($G16),ISBLANK($H16)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1" s="50">
+      <c r="A17" s="90" t="n"/>
+      <c r="B17" s="90" t="n"/>
+      <c r="C17" s="90" t="n"/>
+      <c r="D17" s="90" t="n"/>
+      <c r="E17" s="90" t="n"/>
+      <c r="F17" s="90" t="n"/>
+      <c r="G17" s="90" t="n"/>
+      <c r="H17" s="90" t="n"/>
+      <c r="I17" s="89">
+        <f>IF(ISBLANK($A17),"",IF(OR(ISBLANK($B17),ISBLANK($C17),ISBLANK($D17),ISBLANK($E17),ISBLANK($F17),ISBLANK($G17),ISBLANK($H17)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1" s="50">
+      <c r="A18" s="90" t="n"/>
+      <c r="B18" s="90" t="n"/>
+      <c r="C18" s="90" t="n"/>
+      <c r="D18" s="90" t="n"/>
+      <c r="E18" s="90" t="n"/>
+      <c r="F18" s="90" t="n"/>
+      <c r="G18" s="90" t="n"/>
+      <c r="H18" s="90" t="n"/>
+      <c r="I18" s="89">
+        <f>IF(ISBLANK($A18),"",IF(OR(ISBLANK($B18),ISBLANK($C18),ISBLANK($D18),ISBLANK($E18),ISBLANK($F18),ISBLANK($G18),ISBLANK($H18)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1" s="50">
+      <c r="A19" s="90" t="n"/>
+      <c r="B19" s="90" t="n"/>
+      <c r="C19" s="90" t="n"/>
+      <c r="D19" s="90" t="n"/>
+      <c r="E19" s="90" t="n"/>
+      <c r="F19" s="90" t="n"/>
+      <c r="G19" s="90" t="n"/>
+      <c r="H19" s="90" t="n"/>
+      <c r="I19" s="89">
+        <f>IF(ISBLANK($A19),"",IF(OR(ISBLANK($B19),ISBLANK($C19),ISBLANK($D19),ISBLANK($E19),ISBLANK($F19),ISBLANK($G19),ISBLANK($H19)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1" s="50">
+      <c r="A20" s="90" t="n"/>
+      <c r="B20" s="90" t="n"/>
+      <c r="C20" s="90" t="n"/>
+      <c r="D20" s="90" t="n"/>
+      <c r="E20" s="90" t="n"/>
+      <c r="F20" s="90" t="n"/>
+      <c r="G20" s="90" t="n"/>
+      <c r="H20" s="90" t="n"/>
+      <c r="I20" s="89">
+        <f>IF(ISBLANK($A20),"",IF(OR(ISBLANK($B20),ISBLANK($C20),ISBLANK($D20),ISBLANK($E20),ISBLANK($F20),ISBLANK($G20),ISBLANK($H20)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1" s="50">
+      <c r="A21" s="90" t="n"/>
+      <c r="B21" s="90" t="n"/>
+      <c r="C21" s="90" t="n"/>
+      <c r="D21" s="90" t="n"/>
+      <c r="E21" s="90" t="n"/>
+      <c r="F21" s="90" t="n"/>
+      <c r="G21" s="90" t="n"/>
+      <c r="H21" s="90" t="n"/>
+      <c r="I21" s="89">
+        <f>IF(ISBLANK($A21),"",IF(OR(ISBLANK($B21),ISBLANK($C21),ISBLANK($D21),ISBLANK($E21),ISBLANK($F21),ISBLANK($G21),ISBLANK($H21)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1" s="50">
+      <c r="A22" s="90" t="n"/>
+      <c r="B22" s="90" t="n"/>
+      <c r="C22" s="90" t="n"/>
+      <c r="D22" s="90" t="n"/>
+      <c r="E22" s="90" t="n"/>
+      <c r="F22" s="90" t="n"/>
+      <c r="G22" s="90" t="n"/>
+      <c r="H22" s="90" t="n"/>
+      <c r="I22" s="89">
+        <f>IF(ISBLANK($A22),"",IF(OR(ISBLANK($B22),ISBLANK($C22),ISBLANK($D22),ISBLANK($E22),ISBLANK($F22),ISBLANK($G22),ISBLANK($H22)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="15" customHeight="1" s="50">
+      <c r="A23" s="90" t="n"/>
+      <c r="B23" s="90" t="n"/>
+      <c r="C23" s="90" t="n"/>
+      <c r="D23" s="90" t="n"/>
+      <c r="E23" s="90" t="n"/>
+      <c r="F23" s="90" t="n"/>
+      <c r="G23" s="90" t="n"/>
+      <c r="H23" s="90" t="n"/>
+      <c r="I23" s="89">
+        <f>IF(ISBLANK($A23),"",IF(OR(ISBLANK($B23),ISBLANK($C23),ISBLANK($D23),ISBLANK($E23),ISBLANK($F23),ISBLANK($G23),ISBLANK($H23)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1" s="50">
+      <c r="A24" s="90" t="n"/>
+      <c r="B24" s="90" t="n"/>
+      <c r="C24" s="90" t="n"/>
+      <c r="D24" s="90" t="n"/>
+      <c r="E24" s="90" t="n"/>
+      <c r="F24" s="90" t="n"/>
+      <c r="G24" s="90" t="n"/>
+      <c r="H24" s="90" t="n"/>
+      <c r="I24" s="89">
+        <f>IF(ISBLANK($A24),"",IF(OR(ISBLANK($B24),ISBLANK($C24),ISBLANK($D24),ISBLANK($E24),ISBLANK($F24),ISBLANK($G24),ISBLANK($H24)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="15" customHeight="1" s="50">
+      <c r="A25" s="90" t="n"/>
+      <c r="B25" s="90" t="n"/>
+      <c r="C25" s="90" t="n"/>
+      <c r="D25" s="90" t="n"/>
+      <c r="E25" s="90" t="n"/>
+      <c r="F25" s="90" t="n"/>
+      <c r="G25" s="90" t="n"/>
+      <c r="H25" s="90" t="n"/>
+      <c r="I25" s="89">
+        <f>IF(ISBLANK($A25),"",IF(OR(ISBLANK($B25),ISBLANK($C25),ISBLANK($D25),ISBLANK($E25),ISBLANK($F25),ISBLANK($G25),ISBLANK($H25)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="15" customHeight="1" s="50">
+      <c r="A26" s="90" t="n"/>
+      <c r="B26" s="90" t="n"/>
+      <c r="C26" s="90" t="n"/>
+      <c r="D26" s="90" t="n"/>
+      <c r="E26" s="90" t="n"/>
+      <c r="F26" s="90" t="n"/>
+      <c r="G26" s="90" t="n"/>
+      <c r="H26" s="90" t="n"/>
+      <c r="I26" s="89">
+        <f>IF(ISBLANK($A26),"",IF(OR(ISBLANK($B26),ISBLANK($C26),ISBLANK($D26),ISBLANK($E26),ISBLANK($F26),ISBLANK($G26),ISBLANK($H26)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1" s="50">
+      <c r="A27" s="90" t="n"/>
+      <c r="B27" s="90" t="n"/>
+      <c r="C27" s="90" t="n"/>
+      <c r="D27" s="90" t="n"/>
+      <c r="E27" s="90" t="n"/>
+      <c r="F27" s="90" t="n"/>
+      <c r="G27" s="90" t="n"/>
+      <c r="H27" s="90" t="n"/>
+      <c r="I27" s="89">
+        <f>IF(ISBLANK($A27),"",IF(OR(ISBLANK($B27),ISBLANK($C27),ISBLANK($D27),ISBLANK($E27),ISBLANK($F27),ISBLANK($G27),ISBLANK($H27)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1" s="50">
+      <c r="A28" s="90" t="n"/>
+      <c r="B28" s="90" t="n"/>
+      <c r="C28" s="90" t="n"/>
+      <c r="D28" s="90" t="n"/>
+      <c r="E28" s="90" t="n"/>
+      <c r="F28" s="90" t="n"/>
+      <c r="G28" s="90" t="n"/>
+      <c r="H28" s="90" t="n"/>
+      <c r="I28" s="89">
+        <f>IF(ISBLANK($A28),"",IF(OR(ISBLANK($B28),ISBLANK($C28),ISBLANK($D28),ISBLANK($E28),ISBLANK($F28),ISBLANK($G28),ISBLANK($H28)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="15" customHeight="1" s="50">
+      <c r="A29" s="90" t="n"/>
+      <c r="B29" s="90" t="n"/>
+      <c r="C29" s="90" t="n"/>
+      <c r="D29" s="90" t="n"/>
+      <c r="E29" s="90" t="n"/>
+      <c r="F29" s="90" t="n"/>
+      <c r="G29" s="90" t="n"/>
+      <c r="H29" s="90" t="n"/>
+      <c r="I29" s="89">
+        <f>IF(ISBLANK($A29),"",IF(OR(ISBLANK($B29),ISBLANK($C29),ISBLANK($D29),ISBLANK($E29),ISBLANK($F29),ISBLANK($G29),ISBLANK($H29)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1" s="50">
+      <c r="A30" s="90" t="n"/>
+      <c r="B30" s="90" t="n"/>
+      <c r="C30" s="90" t="n"/>
+      <c r="D30" s="90" t="n"/>
+      <c r="E30" s="90" t="n"/>
+      <c r="F30" s="90" t="n"/>
+      <c r="G30" s="90" t="n"/>
+      <c r="H30" s="90" t="n"/>
+      <c r="I30" s="89">
+        <f>IF(ISBLANK($A30),"",IF(OR(ISBLANK($B30),ISBLANK($C30),ISBLANK($D30),ISBLANK($E30),ISBLANK($F30),ISBLANK($G30),ISBLANK($H30)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="50">
+      <c r="A31" s="90" t="n"/>
+      <c r="B31" s="90" t="n"/>
+      <c r="C31" s="90" t="n"/>
+      <c r="D31" s="90" t="n"/>
+      <c r="E31" s="90" t="n"/>
+      <c r="F31" s="90" t="n"/>
+      <c r="G31" s="90" t="n"/>
+      <c r="H31" s="90" t="n"/>
+      <c r="I31" s="89">
+        <f>IF(ISBLANK($A31),"",IF(OR(ISBLANK($B31),ISBLANK($C31),ISBLANK($D31),ISBLANK($E31),ISBLANK($F31),ISBLANK($G31),ISBLANK($H31)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1" s="50">
+      <c r="A32" s="90" t="n"/>
+      <c r="B32" s="90" t="n"/>
+      <c r="C32" s="90" t="n"/>
+      <c r="D32" s="90" t="n"/>
+      <c r="E32" s="90" t="n"/>
+      <c r="F32" s="90" t="n"/>
+      <c r="G32" s="90" t="n"/>
+      <c r="H32" s="90" t="n"/>
+      <c r="I32" s="89">
+        <f>IF(ISBLANK($A32),"",IF(OR(ISBLANK($B32),ISBLANK($C32),ISBLANK($D32),ISBLANK($E32),ISBLANK($F32),ISBLANK($G32),ISBLANK($H32)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1" s="50">
+      <c r="A33" s="90" t="n"/>
+      <c r="B33" s="90" t="n"/>
+      <c r="C33" s="90" t="n"/>
+      <c r="D33" s="90" t="n"/>
+      <c r="E33" s="90" t="n"/>
+      <c r="F33" s="90" t="n"/>
+      <c r="G33" s="90" t="n"/>
+      <c r="H33" s="90" t="n"/>
+      <c r="I33" s="89">
+        <f>IF(ISBLANK($A33),"",IF(OR(ISBLANK($B33),ISBLANK($C33),ISBLANK($D33),ISBLANK($E33),ISBLANK($F33),ISBLANK($G33),ISBLANK($H33)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="15" customHeight="1" s="50">
+      <c r="A34" s="90" t="n"/>
+      <c r="B34" s="90" t="n"/>
+      <c r="C34" s="90" t="n"/>
+      <c r="D34" s="90" t="n"/>
+      <c r="E34" s="90" t="n"/>
+      <c r="F34" s="90" t="n"/>
+      <c r="G34" s="90" t="n"/>
+      <c r="H34" s="90" t="n"/>
+      <c r="I34" s="89">
+        <f>IF(ISBLANK($A34),"",IF(OR(ISBLANK($B34),ISBLANK($C34),ISBLANK($D34),ISBLANK($E34),ISBLANK($F34),ISBLANK($G34),ISBLANK($H34)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="15" customHeight="1" s="50">
+      <c r="A35" s="90" t="n"/>
+      <c r="B35" s="90" t="n"/>
+      <c r="C35" s="90" t="n"/>
+      <c r="D35" s="90" t="n"/>
+      <c r="E35" s="90" t="n"/>
+      <c r="F35" s="90" t="n"/>
+      <c r="G35" s="90" t="n"/>
+      <c r="H35" s="90" t="n"/>
+      <c r="I35" s="89">
+        <f>IF(ISBLANK($A35),"",IF(OR(ISBLANK($B35),ISBLANK($C35),ISBLANK($D35),ISBLANK($E35),ISBLANK($F35),ISBLANK($G35),ISBLANK($H35)),"EKSİK","OK"))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:AN1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="G6:G1000">
+    <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="lessThan" aboveAverage="0" dxfId="9" text="" percent="0" bottom="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D6:D1000">
+    <cfRule type="cellIs" rank="0" priority="3" equalAverage="0" operator="equal" aboveAverage="0" dxfId="10" text="" percent="0" bottom="0">
+      <formula>"Komisyon"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I6:I1000">
+    <cfRule type="cellIs" rank="0" priority="4" equalAverage="0" operator="equal" aboveAverage="0" dxfId="9" text="" percent="0" bottom="0">
+      <formula>"EKSİK"</formula>
+    </cfRule>
+    <cfRule type="cellIs" rank="0" priority="5" equalAverage="0" operator="equal" aboveAverage="0" dxfId="8" text="" percent="0" bottom="0">
+      <formula>"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="D6:D1000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz Tür" error="Lütfen listeden bir masraf türü seçin." promptTitle="Masraf Türü" prompt="Tahsis Ücreti, Sigorta, Komisyon veya Diğer seçin." type="list" errorStyle="stop" operator="between">
+      <formula1>ListeMasrafTuru</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation sqref="B6:B1000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz Kredi" error="Lütfen KREDILER sayfasındaki bir kredi ID seçin." promptTitle="Kredi ID" prompt="Listeden kredi seçin." type="list" errorStyle="stop" operator="between">
+      <formula1>ListeKrediId</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <tabColor rgb="0060A5FA"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:AN35"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
     <col width="12" customWidth="1" style="76" min="1" max="1"/>
     <col width="11" customWidth="1" style="76" min="2" max="2"/>
     <col width="24" customWidth="1" style="76" min="3" max="3"/>
@@ -14316,7 +15231,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <tabColor rgb="0060A5FA"/>
@@ -15180,7 +16095,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <tabColor rgb="007C3AED"/>
@@ -16562,7 +17477,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="007C3AED"/>
@@ -16616,142 +17531,142 @@
     </row>
     <row r="5" ht="14" customHeight="1" s="50"/>
     <row r="6" ht="28" customHeight="1" s="50">
-      <c r="B6" s="191" t="inlineStr">
+      <c r="B6" s="415" t="inlineStr">
         <is>
           <t>SENARYO A: KÖTÜMSER (STRES TESTİ -%20)</t>
         </is>
       </c>
-      <c r="C6" s="252" t="n"/>
-      <c r="D6" s="252" t="n"/>
-      <c r="E6" s="252" t="n"/>
-      <c r="F6" s="253" t="n"/>
-      <c r="H6" s="192" t="inlineStr">
+      <c r="C6" s="399" t="n"/>
+      <c r="D6" s="399" t="n"/>
+      <c r="E6" s="399" t="n"/>
+      <c r="F6" s="416" t="n"/>
+      <c r="H6" s="417" t="inlineStr">
         <is>
           <t>SENARYO B: BAZ MODEL (HEDEFLENEN)</t>
         </is>
       </c>
-      <c r="I6" s="252" t="n"/>
-      <c r="J6" s="252" t="n"/>
-      <c r="K6" s="252" t="n"/>
-      <c r="L6" s="253" t="n"/>
+      <c r="I6" s="399" t="n"/>
+      <c r="J6" s="399" t="n"/>
+      <c r="K6" s="399" t="n"/>
+      <c r="L6" s="416" t="n"/>
     </row>
     <row r="7" ht="8" customHeight="1" s="50">
-      <c r="B7" s="129" t="n"/>
-      <c r="C7" s="129" t="n"/>
-      <c r="D7" s="129" t="n"/>
-      <c r="E7" s="129" t="n"/>
-      <c r="F7" s="129" t="n"/>
-      <c r="H7" s="129" t="n"/>
-      <c r="I7" s="129" t="n"/>
-      <c r="J7" s="129" t="n"/>
-      <c r="K7" s="129" t="n"/>
-      <c r="L7" s="129" t="n"/>
+      <c r="B7" s="418" t="n"/>
+      <c r="C7" s="404" t="n"/>
+      <c r="D7" s="404" t="n"/>
+      <c r="E7" s="404" t="n"/>
+      <c r="F7" s="405" t="n"/>
+      <c r="H7" s="418" t="n"/>
+      <c r="I7" s="404" t="n"/>
+      <c r="J7" s="404" t="n"/>
+      <c r="K7" s="404" t="n"/>
+      <c r="L7" s="405" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1" s="50">
-      <c r="B8" s="193" t="inlineStr">
+      <c r="B8" s="419" t="inlineStr">
         <is>
           <t>Faaliyet Nakit Akışı Daralması:</t>
         </is>
       </c>
-      <c r="C8" s="129" t="n"/>
-      <c r="D8" s="129" t="n"/>
-      <c r="E8" s="194" t="inlineStr">
+      <c r="C8" s="404" t="n"/>
+      <c r="D8" s="404" t="n"/>
+      <c r="E8" s="420" t="inlineStr">
         <is>
           <t>-%20.0 (Kriz Modeli)</t>
         </is>
       </c>
-      <c r="F8" s="129" t="n"/>
-      <c r="H8" s="193" t="inlineStr">
+      <c r="F8" s="405" t="n"/>
+      <c r="H8" s="419" t="inlineStr">
         <is>
           <t>Planlanan Borç Karşılama:</t>
         </is>
       </c>
-      <c r="I8" s="129" t="n"/>
-      <c r="J8" s="129" t="n"/>
-      <c r="K8" s="195" t="inlineStr">
+      <c r="I8" s="404" t="n"/>
+      <c r="J8" s="404" t="n"/>
+      <c r="K8" s="421" t="inlineStr">
         <is>
           <t>%100.0 (Tam Bütçe)</t>
         </is>
       </c>
-      <c r="L8" s="129" t="n"/>
+      <c r="L8" s="405" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1" s="50">
-      <c r="B9" s="193" t="inlineStr">
+      <c r="B9" s="419" t="inlineStr">
         <is>
           <t>Mevcut 30 Günlük Borç Servisi:</t>
         </is>
       </c>
-      <c r="C9" s="129" t="n"/>
-      <c r="D9" s="129" t="n"/>
-      <c r="E9" s="232">
+      <c r="C9" s="404" t="n"/>
+      <c r="D9" s="404" t="n"/>
+      <c r="E9" s="422">
         <f>KARAR_MOTORU!B7</f>
         <v/>
       </c>
-      <c r="F9" s="129" t="n"/>
-      <c r="H9" s="193" t="inlineStr">
+      <c r="F9" s="405" t="n"/>
+      <c r="H9" s="419" t="inlineStr">
         <is>
           <t>Aylık Refinansman Tasarrufu:</t>
         </is>
       </c>
-      <c r="I9" s="129" t="n"/>
-      <c r="J9" s="129" t="n"/>
-      <c r="K9" s="232">
+      <c r="I9" s="404" t="n"/>
+      <c r="J9" s="404" t="n"/>
+      <c r="K9" s="422">
         <f>KARAR_MOTORU!B19</f>
         <v/>
       </c>
-      <c r="L9" s="129" t="n"/>
+      <c r="L9" s="405" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1" s="50">
-      <c r="B10" s="193" t="inlineStr">
+      <c r="B10" s="419" t="inlineStr">
         <is>
           <t>Stres Altında Serbest Nakit:</t>
         </is>
       </c>
-      <c r="C10" s="129" t="n"/>
-      <c r="D10" s="129" t="n"/>
-      <c r="E10" s="233">
+      <c r="C10" s="404" t="n"/>
+      <c r="D10" s="404" t="n"/>
+      <c r="E10" s="423">
         <f>SerbestNakit*0.8</f>
         <v/>
       </c>
-      <c r="F10" s="129" t="n"/>
-      <c r="H10" s="193" t="inlineStr">
+      <c r="F10" s="405" t="n"/>
+      <c r="H10" s="419" t="inlineStr">
         <is>
           <t>Konsolide Serbest Nakit:</t>
         </is>
       </c>
-      <c r="I10" s="129" t="n"/>
-      <c r="J10" s="129" t="n"/>
-      <c r="K10" s="233">
+      <c r="I10" s="404" t="n"/>
+      <c r="J10" s="404" t="n"/>
+      <c r="K10" s="423">
         <f>SerbestNakit</f>
         <v/>
       </c>
-      <c r="L10" s="129" t="n"/>
+      <c r="L10" s="405" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1" s="50">
-      <c r="B11" s="193" t="inlineStr">
+      <c r="B11" s="424" t="inlineStr">
         <is>
           <t>Stres Altında Likidite Baskısı:</t>
         </is>
       </c>
-      <c r="C11" s="129" t="n"/>
-      <c r="D11" s="129" t="n"/>
-      <c r="E11" s="234">
+      <c r="C11" s="411" t="n"/>
+      <c r="D11" s="411" t="n"/>
+      <c r="E11" s="425">
         <f>YUVARLA(KARAR_MOTORU!B7/MAX(1,SerbestNakit*0.8); 2)</f>
         <v/>
       </c>
-      <c r="F11" s="129" t="n"/>
-      <c r="H11" s="193" t="inlineStr">
+      <c r="F11" s="412" t="n"/>
+      <c r="H11" s="424" t="inlineStr">
         <is>
           <t>Baz Model Likidite Baskısı:</t>
         </is>
       </c>
-      <c r="I11" s="129" t="n"/>
-      <c r="J11" s="129" t="n"/>
-      <c r="K11" s="197">
+      <c r="I11" s="411" t="n"/>
+      <c r="J11" s="411" t="n"/>
+      <c r="K11" s="426">
         <f>YUVARLA(KARAR_MOTORU!B14; 2)</f>
         <v/>
       </c>
-      <c r="L11" s="129" t="n"/>
+      <c r="L11" s="412" t="n"/>
     </row>
     <row r="12" ht="8" customHeight="1" s="50">
       <c r="B12" s="129" t="n"/>
@@ -16883,7 +17798,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <tabColor rgb="007C3AED"/>
@@ -17071,7 +17986,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <tabColor rgb="00475569"/>
@@ -17317,7 +18232,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <tabColor rgb="00475569"/>
@@ -17901,7 +18816,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <tabColor rgb="00475569"/>
@@ -18168,7 +19083,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <tabColor rgb="0064748B"/>
@@ -18347,7 +19262,469 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002563EB"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:F31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3.5" customWidth="1" style="50" min="1" max="1"/>
+    <col width="24" customWidth="1" style="50" min="2" max="2"/>
+    <col width="32" customWidth="1" style="50" min="3" max="3"/>
+    <col width="40" customWidth="1" style="50" min="4" max="4"/>
+    <col width="24" customWidth="1" style="50" min="5" max="5"/>
+    <col width="18" customWidth="1" style="50" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="36" customHeight="1" s="50">
+      <c r="B2" s="371" t="inlineStr">
+        <is>
+          <t>SİSTEM HAKKINDA, KULLANIM REHBERİ VE TERİMLER SÖZLÜĞÜ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" s="50">
+      <c r="B3" s="372" t="inlineStr">
+        <is>
+          <t>5 Yaşındaki Birine Anlatır Gibi Basit, Sade ve Eksiksiz Finansal Karar Mimarisi · Siemens &amp; Enterprise Standartları</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1" s="50">
+      <c r="B5" s="373" t="inlineStr">
+        <is>
+          <t>1. TEMEL MANTIK — 3 DAKİKADA SİSTEMİN ÖZÜ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1" s="50">
+      <c r="B7" s="374" t="inlineStr">
+        <is>
+          <t>SORU</t>
+        </is>
+      </c>
+      <c r="C7" s="375" t="inlineStr">
+        <is>
+          <t>GÜNLÜK DİLLE CEVAP (5 YAŞINDA ÇOCUĞA ANLATIR GİBİ)</t>
+        </is>
+      </c>
+      <c r="D7" s="375" t="inlineStr">
+        <is>
+          <t>ŞİRKETİNİZE FAYDASI NE?</t>
+        </is>
+      </c>
+      <c r="E7" s="374" t="inlineStr">
+        <is>
+          <t>İLGİLİ SAYFA</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1" s="50">
+      <c r="B8" s="376" t="inlineStr">
+        <is>
+          <t>1. Bu dosya ne işe yarar?</t>
+        </is>
+      </c>
+      <c r="C8" s="377" t="inlineStr">
+        <is>
+          <t>Tıpkı arabanın gösterge paneli gibidir. Hangi bankaya ne kadar borcunuz olduğunu, bu ay ne kadar taksit ödeyeceğinizi ve paranızın yetip yetmeyeceğini tek bir ekranda gösterir.</t>
+        </is>
+      </c>
+      <c r="D8" s="378" t="inlineStr">
+        <is>
+          <t>Gözden kaçan, sürpriz veya geciken taksitleri sıfırlar; faiz cezası ve itibar kaybını önler.</t>
+        </is>
+      </c>
+      <c r="E8" s="379" t="inlineStr">
+        <is>
+          <t>PANO, YÖNETİM_RAPORU</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1" s="50">
+      <c r="B9" s="380" t="inlineStr">
+        <is>
+          <t>2. Kullanıcı olarak ben ne yapacağım?</t>
+        </is>
+      </c>
+      <c r="C9" s="381" t="inlineStr">
+        <is>
+          <t>Çok kolay! Yalnızca 'GİRDİLER' sekmesindeki sarı renkli kutulara çektiğiniz kredileri ve vadesini yazacaksınız. Geri kalan tüm hesapları sistem kendi yapar.</t>
+        </is>
+      </c>
+      <c r="D9" s="382" t="inlineStr">
+        <is>
+          <t>Veri girişi birkaç dakikada biter, karmaşık formüllerle veya Excel kodlarıyla uğraşmazsınız.</t>
+        </is>
+      </c>
+      <c r="E9" s="383" t="inlineStr">
+        <is>
+          <t>GİRDİLER, KREDILER</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1" s="50">
+      <c r="B10" s="376" t="inlineStr">
+        <is>
+          <t>3. Sistem bana ne kazandırır?</t>
+        </is>
+      </c>
+      <c r="C10" s="377" t="inlineStr">
+        <is>
+          <t>Hangi bankaya çok faiz ödediğinizi bulur. 'Şu krediyi kapatıp şuraya taşırsan ayda 495.000 TL tasarruf edersin' diyerek şirketinize somut nakit kazandırır.</t>
+        </is>
+      </c>
+      <c r="D10" s="378" t="inlineStr">
+        <is>
+          <t>Gereksiz faiz ve masrafları yok eder; banka pazarlıklarında şirketinizi güçlü kılar.</t>
+        </is>
+      </c>
+      <c r="E10" s="379" t="inlineStr">
+        <is>
+          <t>REFINANSMAN, KARAR_MOTORU</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1" s="50">
+      <c r="B13" s="373" t="inlineStr">
+        <is>
+          <t>2. SÖZLÜK — BU KELİMELER NE ANLAMA GELİYOR?</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1" s="50">
+      <c r="B15" s="374" t="inlineStr">
+        <is>
+          <t>TERİM / KAVRAM</t>
+        </is>
+      </c>
+      <c r="C15" s="374" t="inlineStr">
+        <is>
+          <t>ÇOK BASİT AÇIKLAMASI</t>
+        </is>
+      </c>
+      <c r="D15" s="375" t="inlineStr">
+        <is>
+          <t>BU ŞABLONDA NEREDE HESAPLANIR?</t>
+        </is>
+      </c>
+      <c r="E15" s="375" t="inlineStr">
+        <is>
+          <t>ÖRNEK / İPUCU</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1" s="50">
+      <c r="B16" s="376" t="inlineStr">
+        <is>
+          <t>Refinansman</t>
+        </is>
+      </c>
+      <c r="C16" s="377" t="inlineStr">
+        <is>
+          <t>Pahalı olan eski krediyi kapatıp yerine daha düşük faizli yeni kredi çekmek. Yani borcu ucuza taşımak.</t>
+        </is>
+      </c>
+      <c r="D16" s="384" t="inlineStr">
+        <is>
+          <t>REFINANSMAN sayfası</t>
+        </is>
+      </c>
+      <c r="E16" s="385" t="inlineStr">
+        <is>
+          <t>Ör: %45 faizli krediyi kapatıp %38'e çekerek ayda 495.714 TL kâr etmek.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="36" customHeight="1" s="50">
+      <c r="B17" s="380" t="inlineStr">
+        <is>
+          <t>Borç Servisi</t>
+        </is>
+      </c>
+      <c r="C17" s="381" t="inlineStr">
+        <is>
+          <t>Gelecek 30 gün içinde bankalara tıkır tıkır ödemeniz gereken anapara ve faiz taksitlerinin toplamı.</t>
+        </is>
+      </c>
+      <c r="D17" s="386" t="inlineStr">
+        <is>
+          <t>PANO (E7 hücresi)</t>
+        </is>
+      </c>
+      <c r="E17" s="387" t="inlineStr">
+        <is>
+          <t>Mevcut 30 günlük borç servisimiz: ₺934.864</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="36" customHeight="1" s="50">
+      <c r="B18" s="376" t="inlineStr">
+        <is>
+          <t>Stres Testi</t>
+        </is>
+      </c>
+      <c r="C18" s="377" t="inlineStr">
+        <is>
+          <t>'Gelecek ay işler çok kötü giderse ve kasaya %20 daha az para girerse borcumuzu ödeyebilir miyiz?' provası.</t>
+        </is>
+      </c>
+      <c r="D18" s="384" t="inlineStr">
+        <is>
+          <t>YÖNETİM_RAPORU</t>
+        </is>
+      </c>
+      <c r="E18" s="385" t="inlineStr">
+        <is>
+          <t>Şirketimiz -%20 krizde bile temerrüt riski yaşamadan borcunu ödeyebilmektedir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="36" customHeight="1" s="50">
+      <c r="B19" s="380" t="inlineStr">
+        <is>
+          <t>Temerrüt Riski</t>
+        </is>
+      </c>
+      <c r="C19" s="381" t="inlineStr">
+        <is>
+          <t>Taksit gününde kasada para bulunamaması ve borcun icralık / takipli hale gelme tehlikesi.</t>
+        </is>
+      </c>
+      <c r="D19" s="386" t="inlineStr">
+        <is>
+          <t>KARAR_MOTORU</t>
+        </is>
+      </c>
+      <c r="E19" s="387" t="inlineStr">
+        <is>
+          <t>Sistem yeşil 'UYGUN' yakıyorsa temerrüt riskiniz %0 demektir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="36" customHeight="1" s="50">
+      <c r="B20" s="376" t="inlineStr">
+        <is>
+          <t>DSCR (Borç Karşılama)</t>
+        </is>
+      </c>
+      <c r="C20" s="377" t="inlineStr">
+        <is>
+          <t>Kasaya giren serbest paranın taksitlere olan oranı. 1.0 üzerindeyse şirket rahat nefes alır.</t>
+        </is>
+      </c>
+      <c r="D20" s="384" t="inlineStr">
+        <is>
+          <t>KARAR_MOTORU (B14)</t>
+        </is>
+      </c>
+      <c r="E20" s="385" t="inlineStr">
+        <is>
+          <t>1.25 üstü = Mükemmel Güvenlik Bölgesi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="36" customHeight="1" s="50">
+      <c r="B21" s="380" t="inlineStr">
+        <is>
+          <t>Amortisman Takvimi</t>
+        </is>
+      </c>
+      <c r="C21" s="381" t="inlineStr">
+        <is>
+          <t>Kredinin ilk gününden son gününe kadar her ay kaç para faiz, kaç para anapara ödeneceğini gösteren liste.</t>
+        </is>
+      </c>
+      <c r="D21" s="386" t="inlineStr">
+        <is>
+          <t>TAKSIT_PLANI</t>
+        </is>
+      </c>
+      <c r="E21" s="387" t="inlineStr">
+        <is>
+          <t>Toplam kaç ay taksit kaldığını tek tıkla listeler.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1" s="50">
+      <c r="B24" s="373" t="inlineStr">
+        <is>
+          <t>3. SİSTEMİN 5 AŞAMALI AKIŞ ŞEMASI</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1" s="50">
+      <c r="B26" s="374" t="inlineStr">
+        <is>
+          <t>AŞAMA</t>
+        </is>
+      </c>
+      <c r="C26" s="375" t="inlineStr">
+        <is>
+          <t>GÖREVİ</t>
+        </is>
+      </c>
+      <c r="D26" s="374" t="inlineStr">
+        <is>
+          <t>KULLANILACAK SEKME</t>
+        </is>
+      </c>
+      <c r="E26" s="375" t="inlineStr">
+        <is>
+          <t>GİRİLECEK VERİ</t>
+        </is>
+      </c>
+      <c r="F26" s="375" t="inlineStr">
+        <is>
+          <t>ÜRETİLEN SONUÇ</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="32" customHeight="1" s="50">
+      <c r="B27" s="388" t="inlineStr">
+        <is>
+          <t>1. Hazırlık</t>
+        </is>
+      </c>
+      <c r="C27" s="389" t="inlineStr">
+        <is>
+          <t>Şirket parametrelerini ve nakit durumunu tanıtma</t>
+        </is>
+      </c>
+      <c r="D27" s="390" t="inlineStr">
+        <is>
+          <t>AYARLAR, LISTELER</t>
+        </is>
+      </c>
+      <c r="E27" s="391" t="inlineStr">
+        <is>
+          <t>Firma adı, serbest nakit miktarı</t>
+        </is>
+      </c>
+      <c r="F27" s="392" t="inlineStr">
+        <is>
+          <t>Tüm formüllerin eşik değerleri hazır olur</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1" s="50">
+      <c r="B28" s="393" t="inlineStr">
+        <is>
+          <t>2. Veri Girişi</t>
+        </is>
+      </c>
+      <c r="C28" s="394" t="inlineStr">
+        <is>
+          <t>Bankalardaki borçları ve kredi takvimini yazma</t>
+        </is>
+      </c>
+      <c r="D28" s="395" t="inlineStr">
+        <is>
+          <t>GİRDİLER, KREDILER, LIMITLER</t>
+        </is>
+      </c>
+      <c r="E28" s="396" t="inlineStr">
+        <is>
+          <t>Kredi tutarı, faiz, taksit tarihi</t>
+        </is>
+      </c>
+      <c r="F28" s="397" t="inlineStr">
+        <is>
+          <t>Ödeme takvimi otomatik üretilir</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="32" customHeight="1" s="50">
+      <c r="B29" s="388" t="inlineStr">
+        <is>
+          <t>3. Anlık Takip</t>
+        </is>
+      </c>
+      <c r="C29" s="389" t="inlineStr">
+        <is>
+          <t>Borç yükünü ve 30 günlük ödemeleri izleme</t>
+        </is>
+      </c>
+      <c r="D29" s="390" t="inlineStr">
+        <is>
+          <t>PANO</t>
+        </is>
+      </c>
+      <c r="E29" s="391" t="inlineStr">
+        <is>
+          <t>Otomatik hesaplanır</t>
+        </is>
+      </c>
+      <c r="F29" s="392" t="inlineStr">
+        <is>
+          <t>Gözden kaçan taksit riski kalmaz</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="32" customHeight="1" s="50">
+      <c r="B30" s="393" t="inlineStr">
+        <is>
+          <t>4. Fırsat Avı</t>
+        </is>
+      </c>
+      <c r="C30" s="394" t="inlineStr">
+        <is>
+          <t>Pahalı kredileri ucuza taşıma &amp; Kriz testi</t>
+        </is>
+      </c>
+      <c r="D30" s="395" t="inlineStr">
+        <is>
+          <t>REFINANSMAN, YÖNETİM_RAPORU</t>
+        </is>
+      </c>
+      <c r="E30" s="396" t="inlineStr">
+        <is>
+          <t>Yeni teklif faizleri</t>
+        </is>
+      </c>
+      <c r="F30" s="397" t="inlineStr">
+        <is>
+          <t>Aylık ₺495.714'ye varan nakit tasarrufu</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="32" customHeight="1" s="50">
+      <c r="B31" s="388" t="inlineStr">
+        <is>
+          <t>5. Sunum &amp; Karar</t>
+        </is>
+      </c>
+      <c r="C31" s="389" t="inlineStr">
+        <is>
+          <t>Yönetim kuruluna ve bankalara resmi sunum</t>
+        </is>
+      </c>
+      <c r="D31" s="390" t="inlineStr">
+        <is>
+          <t>RAPOR</t>
+        </is>
+      </c>
+      <c r="E31" s="391" t="inlineStr">
+        <is>
+          <t>Tek tıkla hazır</t>
+        </is>
+      </c>
+      <c r="F31" s="392" t="inlineStr">
+        <is>
+          <t>A4 dikey resmi finansal rapor</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <tabColor rgb="0064748B"/>
@@ -19348,593 +20725,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="001E293B"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="3.5" customWidth="1" style="50" min="1" max="1"/>
-    <col width="14" customWidth="1" style="50" min="2" max="2"/>
-    <col width="14" customWidth="1" style="50" min="3" max="3"/>
-    <col width="10" customWidth="1" style="50" min="4" max="4"/>
-    <col width="14" customWidth="1" style="50" min="5" max="5"/>
-    <col width="14" customWidth="1" style="50" min="6" max="6"/>
-    <col width="10" customWidth="1" style="50" min="7" max="7"/>
-    <col width="14" customWidth="1" style="50" min="8" max="8"/>
-    <col width="14" customWidth="1" style="50" min="9" max="9"/>
-    <col width="10" customWidth="1" style="50" min="10" max="10"/>
-    <col width="14" customWidth="1" style="50" min="11" max="11"/>
-    <col width="14" customWidth="1" style="50" min="12" max="12"/>
-    <col width="10" customWidth="1" style="50" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="10" customHeight="1" s="50">
-      <c r="A1" s="60" t="inlineStr">
-        <is>
-          <t>☰ PANO</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="36" customHeight="1" s="50">
-      <c r="B2" s="242" t="inlineStr">
-        <is>
-          <t>BANKA, KREDİ VE TAKSİT YÖNETİM MERKEZİ</t>
-        </is>
-      </c>
-      <c r="L2" s="125" t="inlineStr">
-        <is>
-          <t>Dönem: 2026 / Tam ▼</t>
-        </is>
-      </c>
-      <c r="M2" s="126" t="inlineStr">
-        <is>
-          <t>★ DOĞRULANMIŞ</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1" s="50">
-      <c r="B3" s="237" t="inlineStr">
-        <is>
-          <t>Konsolide Kredi Portföyü, Aylık Borç Servisi ve Likidite Karar Kokpiti · Canlı Hesaplama</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="14" customHeight="1" s="50"/>
-    <row r="5" ht="20" customHeight="1" s="50">
-      <c r="B5" s="128" t="inlineStr">
-        <is>
-          <t>TOPLAM KREDİ PORTFÖYÜ</t>
-        </is>
-      </c>
-      <c r="C5" s="129" t="n"/>
-      <c r="D5" s="130" t="inlineStr">
-        <is>
-          <t>CANLI BAKİYE</t>
-        </is>
-      </c>
-      <c r="E5" s="131" t="inlineStr">
-        <is>
-          <t>AYLIK BORÇ SERVİSİ (30 GÜN)</t>
-        </is>
-      </c>
-      <c r="F5" s="129" t="n"/>
-      <c r="G5" s="132" t="inlineStr">
-        <is>
-          <t>ÖDEME BASKISI</t>
-        </is>
-      </c>
-      <c r="H5" s="128" t="inlineStr">
-        <is>
-          <t>REFİNANSMAN AYLIK RAHATLAMA</t>
-        </is>
-      </c>
-      <c r="I5" s="129" t="n"/>
-      <c r="J5" s="133">
-        <f>KARAR_MOTORU!B18&amp;" ADAY"</f>
-        <v/>
-      </c>
-      <c r="K5" s="134" t="inlineStr">
-        <is>
-          <t>BORÇLANMA SÜRDÜRÜLEBİLİRLİĞİ</t>
-        </is>
-      </c>
-      <c r="L5" s="129" t="n"/>
-      <c r="M5" s="130">
-        <f>KARAR_MOTORU!B16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6" ht="6" customHeight="1" s="50">
-      <c r="B6" s="135" t="n"/>
-      <c r="C6" s="129" t="n"/>
-      <c r="D6" s="129" t="n"/>
-      <c r="E6" s="136" t="n"/>
-      <c r="F6" s="129" t="n"/>
-      <c r="G6" s="129" t="n"/>
-      <c r="H6" s="135" t="n"/>
-      <c r="I6" s="129" t="n"/>
-      <c r="J6" s="129" t="n"/>
-      <c r="K6" s="137" t="n"/>
-      <c r="L6" s="129" t="n"/>
-      <c r="M6" s="129" t="n"/>
-    </row>
-    <row r="7" ht="34" customHeight="1" s="50">
-      <c r="B7" s="297">
-        <f>KARAR_MOTORU!B5</f>
-        <v/>
-      </c>
-      <c r="C7" s="129" t="n"/>
-      <c r="D7" s="129" t="n"/>
-      <c r="E7" s="298">
-        <f>KARAR_MOTORU!B7</f>
-        <v/>
-      </c>
-      <c r="F7" s="129" t="n"/>
-      <c r="G7" s="129" t="n"/>
-      <c r="H7" s="299">
-        <f>KARAR_MOTORU!B19</f>
-        <v/>
-      </c>
-      <c r="I7" s="129" t="n"/>
-      <c r="J7" s="129" t="n"/>
-      <c r="K7" s="300">
-        <f>KARAR_MOTORU!B15</f>
-        <v/>
-      </c>
-      <c r="L7" s="129" t="n"/>
-      <c r="M7" s="129" t="n"/>
-    </row>
-    <row r="8" ht="6" customHeight="1" s="50">
-      <c r="B8" s="135" t="n"/>
-      <c r="C8" s="129" t="n"/>
-      <c r="D8" s="129" t="n"/>
-      <c r="E8" s="136" t="n"/>
-      <c r="F8" s="129" t="n"/>
-      <c r="G8" s="129" t="n"/>
-      <c r="H8" s="135" t="n"/>
-      <c r="I8" s="129" t="n"/>
-      <c r="J8" s="129" t="n"/>
-      <c r="K8" s="137" t="n"/>
-      <c r="L8" s="129" t="n"/>
-      <c r="M8" s="129" t="n"/>
-    </row>
-    <row r="9" ht="20" customHeight="1" s="50">
-      <c r="B9" s="141" t="inlineStr">
-        <is>
-          <t>↑ Aktif portföy risk hacmi</t>
-        </is>
-      </c>
-      <c r="C9" s="129" t="n"/>
-      <c r="D9" s="129" t="n"/>
-      <c r="E9" s="142" t="inlineStr">
-        <is>
-          <t>● 30 gün içinde vadesi gelen taksitler</t>
-        </is>
-      </c>
-      <c r="F9" s="129" t="n"/>
-      <c r="G9" s="129" t="n"/>
-      <c r="H9" s="141" t="inlineStr">
-        <is>
-          <t>✓ Yapılandırma ile aylık nakit kazanımı</t>
-        </is>
-      </c>
-      <c r="I9" s="129" t="n"/>
-      <c r="J9" s="129" t="n"/>
-      <c r="K9" s="246">
-        <f>KARAR_MOTORU!B17</f>
-        <v/>
-      </c>
-      <c r="L9" s="129" t="n"/>
-      <c r="M9" s="129" t="n"/>
-    </row>
-    <row r="10" ht="16" customHeight="1" s="50"/>
-    <row r="11" ht="24" customHeight="1" s="50">
-      <c r="B11" s="74" t="inlineStr">
-        <is>
-          <t>BANKA, KREDI VE TAKSIT TAKIP SISTEMI — DÖNEMSEL İCRA VE PROJEKSİYON</t>
-        </is>
-      </c>
-      <c r="F11" s="144" t="inlineStr">
-        <is>
-          <t>+%32 Verim</t>
-        </is>
-      </c>
-      <c r="H11" s="74" t="inlineStr">
-        <is>
-          <t>KONSOLİDE OPERASYON VE KARAR MATRİSİ</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1" s="50">
-      <c r="B12" s="73" t="inlineStr">
-        <is>
-          <t>Kümülatif Hacim vs. Operasyonel Maliyet ve Net Kâr Eğilimi</t>
-        </is>
-      </c>
-      <c r="H12" s="73" t="inlineStr">
-        <is>
-          <t>Anlık Hesaplama Sonuçları, Dinamik Formül Çıktıları ve Durum Puanlaması</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="8" customHeight="1" s="50"/>
-    <row r="14" ht="26" customHeight="1" s="50">
-      <c r="B14" s="145" t="inlineStr">
-        <is>
-          <t>Dönem</t>
-        </is>
-      </c>
-      <c r="C14" s="145" t="inlineStr">
-        <is>
-          <t>Aktif Hacim</t>
-        </is>
-      </c>
-      <c r="D14" s="145" t="inlineStr">
-        <is>
-          <t>Maliyet/Yük</t>
-        </is>
-      </c>
-      <c r="E14" s="145" t="inlineStr">
-        <is>
-          <t>Hedef</t>
-        </is>
-      </c>
-      <c r="H14" s="146" t="inlineStr">
-        <is>
-          <t>PARAMETRE / KALEM</t>
-        </is>
-      </c>
-      <c r="I14" s="146" t="inlineStr">
-        <is>
-          <t>ANA TUTAR</t>
-        </is>
-      </c>
-      <c r="J14" s="146" t="inlineStr">
-        <is>
-          <t>FARK / MARJ</t>
-        </is>
-      </c>
-      <c r="K14" s="146" t="inlineStr">
-        <is>
-          <t>VADE</t>
-        </is>
-      </c>
-      <c r="L14" s="146" t="inlineStr">
-        <is>
-          <t>KONTROL DURUMU</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1" s="50">
-      <c r="B15" s="73" t="inlineStr">
-        <is>
-          <t>D1</t>
-        </is>
-      </c>
-      <c r="C15" s="73" t="n">
-        <v>65</v>
-      </c>
-      <c r="D15" s="73" t="n">
-        <v>45</v>
-      </c>
-      <c r="E15" s="73" t="n">
-        <v>60</v>
-      </c>
-      <c r="H15" s="147" t="inlineStr">
-        <is>
-          <t>Dönemlik Kümülatif Bakiye</t>
-        </is>
-      </c>
-      <c r="I15" s="227">
-        <f>B7*0.45</f>
-        <v/>
-      </c>
-      <c r="J15" s="228">
-        <f>B7*0.05</f>
-        <v/>
-      </c>
-      <c r="K15" s="149" t="inlineStr">
-        <is>
-          <t>12 Ay</t>
-        </is>
-      </c>
-      <c r="L15" s="133" t="inlineStr">
-        <is>
-          <t>✓ DÜZENLİ</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1" s="50">
-      <c r="B16" s="73" t="inlineStr">
-        <is>
-          <t>D2</t>
-        </is>
-      </c>
-      <c r="C16" s="73" t="n">
-        <v>78</v>
-      </c>
-      <c r="D16" s="73" t="n">
-        <v>48</v>
-      </c>
-      <c r="E16" s="73" t="n">
-        <v>70</v>
-      </c>
-      <c r="H16" s="147" t="inlineStr">
-        <is>
-          <t>Kritik Eşik Güvenlik Tamponu</t>
-        </is>
-      </c>
-      <c r="I16" s="227">
-        <f>B7*0.30</f>
-        <v/>
-      </c>
-      <c r="J16" s="228">
-        <f>B7*0.03</f>
-        <v/>
-      </c>
-      <c r="K16" s="149" t="inlineStr">
-        <is>
-          <t>24 Ay</t>
-        </is>
-      </c>
-      <c r="L16" s="130" t="inlineStr">
-        <is>
-          <t>★ AVANTAJ</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1" s="50">
-      <c r="B17" s="73" t="inlineStr">
-        <is>
-          <t>D3</t>
-        </is>
-      </c>
-      <c r="C17" s="73" t="n">
-        <v>85</v>
-      </c>
-      <c r="D17" s="73" t="n">
-        <v>55</v>
-      </c>
-      <c r="E17" s="73" t="n">
-        <v>80</v>
-      </c>
-      <c r="H17" s="147" t="inlineStr">
-        <is>
-          <t>Operasyonel Net Fark</t>
-        </is>
-      </c>
-      <c r="I17" s="227">
-        <f>B7*0.15</f>
-        <v/>
-      </c>
-      <c r="J17" s="228">
-        <f>B7*0.02</f>
-        <v/>
-      </c>
-      <c r="K17" s="149" t="inlineStr">
-        <is>
-          <t>8 Ay</t>
-        </is>
-      </c>
-      <c r="L17" s="150" t="inlineStr">
-        <is>
-          <t>● YAKLAŞAN</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1" s="50">
-      <c r="B18" s="73" t="inlineStr">
-        <is>
-          <t>D4</t>
-        </is>
-      </c>
-      <c r="C18" s="73" t="n">
-        <v>75</v>
-      </c>
-      <c r="D18" s="73" t="n">
-        <v>42</v>
-      </c>
-      <c r="E18" s="73" t="n">
-        <v>75</v>
-      </c>
-      <c r="H18" s="147" t="inlineStr">
-        <is>
-          <t>Rezerv ve Likit Dağılım</t>
-        </is>
-      </c>
-      <c r="I18" s="227">
-        <f>B7*0.10</f>
-        <v/>
-      </c>
-      <c r="J18" s="228">
-        <f>B7*0.01</f>
-        <v/>
-      </c>
-      <c r="K18" s="149" t="inlineStr">
-        <is>
-          <t>16 Ay</t>
-        </is>
-      </c>
-      <c r="L18" s="133" t="inlineStr">
-        <is>
-          <t>✓ TAM UYUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="26" customHeight="1" s="50">
-      <c r="B19" s="73" t="inlineStr">
-        <is>
-          <t>D5</t>
-        </is>
-      </c>
-      <c r="C19" s="73" t="n">
-        <v>90</v>
-      </c>
-      <c r="D19" s="73" t="n">
-        <v>40</v>
-      </c>
-      <c r="E19" s="73" t="n">
-        <v>85</v>
-      </c>
-      <c r="H19" s="151" t="inlineStr">
-        <is>
-          <t>KONSOLİDE SİSTEM TOPLAMI</t>
-        </is>
-      </c>
-      <c r="I19" s="229">
-        <f>SUM(I15:I18)</f>
-        <v/>
-      </c>
-      <c r="J19" s="230">
-        <f>SUM(J15:J18)</f>
-        <v/>
-      </c>
-      <c r="K19" s="154" t="inlineStr"/>
-      <c r="L19" s="155" t="inlineStr">
-        <is>
-          <t>TAM DOĞRULANDI (0 HATA)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="16" customHeight="1" s="50">
-      <c r="B20" s="73" t="inlineStr">
-        <is>
-          <t>D6</t>
-        </is>
-      </c>
-      <c r="C20" s="73" t="n">
-        <v>96</v>
-      </c>
-      <c r="D20" s="73" t="n">
-        <v>32</v>
-      </c>
-      <c r="E20" s="73" t="n">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="21" ht="8" customHeight="1" s="50"/>
-    <row r="22" ht="24" customHeight="1" s="50">
-      <c r="B22" s="156" t="inlineStr">
-        <is>
-          <t>KONSOLİDE PAY VE AĞIRLIK</t>
-        </is>
-      </c>
-      <c r="F22" s="156" t="inlineStr">
-        <is>
-          <t>LİKİDİTE RİSKİ &amp; ERKEN UYARI SİNYALLERİ</t>
-        </is>
-      </c>
-      <c r="K22" s="157" t="inlineStr">
-        <is>
-          <t>KARAR MOTORU PROTOKOLÜ</t>
-        </is>
-      </c>
-      <c r="L22" s="158" t="n"/>
-      <c r="M22" s="158" t="n"/>
-    </row>
-    <row r="23" ht="22" customHeight="1" s="50">
-      <c r="B23" s="58" t="inlineStr">
-        <is>
-          <t>■ Ana Segment (%42)</t>
-        </is>
-      </c>
-      <c r="F23" s="73" t="inlineStr">
-        <is>
-          <t>Nakit Açığı Riski (30 Gün)</t>
-        </is>
-      </c>
-      <c r="I23" s="159" t="inlineStr">
-        <is>
-          <t>0.00 TL (Sıfır Risk)</t>
-        </is>
-      </c>
-      <c r="K23" s="160" t="inlineStr">
-        <is>
-          <t>REFİNANSMAN &amp; LİKİDİTE</t>
-        </is>
-      </c>
-      <c r="L23" s="158" t="n"/>
-      <c r="M23" s="158" t="n"/>
-    </row>
-    <row r="24" ht="22" customHeight="1" s="50">
-      <c r="B24" s="59" t="inlineStr">
-        <is>
-          <t>■ İkincil Grup (%30)</t>
-        </is>
-      </c>
-      <c r="F24" s="73" t="inlineStr">
-        <is>
-          <t>Tahsilat Gecikme Toleransı</t>
-        </is>
-      </c>
-      <c r="I24" s="159" t="inlineStr">
-        <is>
-          <t>48 Gün Güvenli Eşik</t>
-        </is>
-      </c>
-      <c r="K24" s="161" t="inlineStr">
-        <is>
-          <t>Sistem, nakit açığı riskini 30/60/90 günlük pencerelerde izleyerek, borç servisi oranını optimal eşikte tutacak yapılandırma önerir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1" s="50">
-      <c r="B25" s="162" t="inlineStr">
-        <is>
-          <t>■ Destek Birimi (%15)</t>
-        </is>
-      </c>
-      <c r="F25" s="58" t="inlineStr">
-        <is>
-          <t>██████████████████████████████████████ Güvenli Bölge (%100)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="28" customHeight="1" s="50">
-      <c r="B26" s="163" t="inlineStr">
-        <is>
-          <t>■ Rezervler (%13)</t>
-        </is>
-      </c>
-      <c r="F26" s="164" t="inlineStr">
-        <is>
-          <t>✓ 90 GÜNLÜK PROJEKSİYONDA NAKİT SIKIŞIKLIĞI TESPİT EDİLMEDİ</t>
-        </is>
-      </c>
-      <c r="G26" s="247" t="n"/>
-      <c r="H26" s="247" t="n"/>
-      <c r="I26" s="248" t="n"/>
-      <c r="K26" s="165" t="inlineStr">
-        <is>
-          <t>REFİNANSMAN ANALİZİNİ GÖR (#REFINANSMAN!A1) &gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="10" customHeight="1" s="50">
-      <c r="F27" s="249" t="n"/>
-      <c r="G27" s="250" t="n"/>
-      <c r="H27" s="250" t="n"/>
-      <c r="I27" s="251" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="K26:M27"/>
-    <mergeCell ref="K24:M25"/>
-    <mergeCell ref="F26:I27"/>
-  </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId1"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <tabColor rgb="0064748B"/>
@@ -20168,7 +20959,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C6A15B"/>
@@ -20557,7 +21348,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00065F46"/>
@@ -21048,7 +21839,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="009B2C2C"/>
@@ -21788,7 +22579,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00475569"/>
@@ -22461,7 +23252,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002F75B5"/>
@@ -23006,7 +23797,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="005B477E"/>
@@ -23582,7 +24373,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -23704,7 +24495,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -23793,7 +24584,593 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001E293B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3.5" customWidth="1" style="50" min="1" max="1"/>
+    <col width="14" customWidth="1" style="50" min="2" max="2"/>
+    <col width="14" customWidth="1" style="50" min="3" max="3"/>
+    <col width="10" customWidth="1" style="50" min="4" max="4"/>
+    <col width="14" customWidth="1" style="50" min="5" max="5"/>
+    <col width="14" customWidth="1" style="50" min="6" max="6"/>
+    <col width="10" customWidth="1" style="50" min="7" max="7"/>
+    <col width="30" customWidth="1" style="50" min="8" max="8"/>
+    <col width="16" customWidth="1" style="50" min="9" max="9"/>
+    <col width="16" customWidth="1" style="50" min="10" max="10"/>
+    <col width="10" customWidth="1" style="50" min="11" max="11"/>
+    <col width="26" customWidth="1" style="50" min="12" max="12"/>
+    <col width="10" customWidth="1" style="50" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="10" customHeight="1" s="50">
+      <c r="A1" s="60" t="inlineStr">
+        <is>
+          <t>☰ PANO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1" s="50">
+      <c r="B2" s="242" t="inlineStr">
+        <is>
+          <t>BANKA, KREDİ VE TAKSİT YÖNETİM MERKEZİ</t>
+        </is>
+      </c>
+      <c r="L2" s="125" t="inlineStr">
+        <is>
+          <t>Dönem: 2026 / Tam ▼</t>
+        </is>
+      </c>
+      <c r="M2" s="126" t="inlineStr">
+        <is>
+          <t>★ DOĞRULANMIŞ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1" s="50">
+      <c r="B3" s="237" t="inlineStr">
+        <is>
+          <t>Konsolide Kredi Portföyü, Aylık Borç Servisi ve Likidite Karar Kokpiti · Canlı Hesaplama</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="14" customHeight="1" s="50"/>
+    <row r="5" ht="20" customHeight="1" s="50">
+      <c r="B5" s="398" t="inlineStr">
+        <is>
+          <t>TOPLAM KREDİ PORTFÖYÜ</t>
+        </is>
+      </c>
+      <c r="C5" s="399" t="n"/>
+      <c r="D5" s="400" t="inlineStr">
+        <is>
+          <t>CANLI BAKİYE</t>
+        </is>
+      </c>
+      <c r="E5" s="398" t="inlineStr">
+        <is>
+          <t>AYLIK BORÇ SERVİSİ (30 GÜN)</t>
+        </is>
+      </c>
+      <c r="F5" s="399" t="n"/>
+      <c r="G5" s="401" t="inlineStr">
+        <is>
+          <t>ÖDEME BASKISI</t>
+        </is>
+      </c>
+      <c r="H5" s="398" t="inlineStr">
+        <is>
+          <t>REFİNANSMAN AYLIK RAHATLAMA</t>
+        </is>
+      </c>
+      <c r="I5" s="399" t="n"/>
+      <c r="J5" s="402">
+        <f>KARAR_MOTORU!B18&amp;" ADAY"</f>
+        <v/>
+      </c>
+      <c r="K5" s="398" t="inlineStr">
+        <is>
+          <t>BORÇLANMA SÜRDÜRÜLEBİLİRLİĞİ</t>
+        </is>
+      </c>
+      <c r="L5" s="399" t="n"/>
+      <c r="M5" s="400">
+        <f>KARAR_MOTORU!B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="6" customHeight="1" s="50">
+      <c r="B6" s="403" t="n"/>
+      <c r="C6" s="404" t="n"/>
+      <c r="D6" s="405" t="n"/>
+      <c r="E6" s="403" t="n"/>
+      <c r="F6" s="404" t="n"/>
+      <c r="G6" s="405" t="n"/>
+      <c r="H6" s="403" t="n"/>
+      <c r="I6" s="404" t="n"/>
+      <c r="J6" s="405" t="n"/>
+      <c r="K6" s="403" t="n"/>
+      <c r="L6" s="404" t="n"/>
+      <c r="M6" s="405" t="n"/>
+    </row>
+    <row r="7" ht="34" customHeight="1" s="50">
+      <c r="B7" s="406">
+        <f>KARAR_MOTORU!B5</f>
+        <v/>
+      </c>
+      <c r="C7" s="404" t="n"/>
+      <c r="D7" s="405" t="n"/>
+      <c r="E7" s="407">
+        <f>KARAR_MOTORU!B7</f>
+        <v/>
+      </c>
+      <c r="F7" s="404" t="n"/>
+      <c r="G7" s="405" t="n"/>
+      <c r="H7" s="408">
+        <f>KARAR_MOTORU!B19</f>
+        <v/>
+      </c>
+      <c r="I7" s="404" t="n"/>
+      <c r="J7" s="405" t="n"/>
+      <c r="K7" s="409">
+        <f>KARAR_MOTORU!B15</f>
+        <v/>
+      </c>
+      <c r="L7" s="404" t="n"/>
+      <c r="M7" s="405" t="n"/>
+    </row>
+    <row r="8" ht="6" customHeight="1" s="50">
+      <c r="B8" s="403" t="n"/>
+      <c r="C8" s="404" t="n"/>
+      <c r="D8" s="405" t="n"/>
+      <c r="E8" s="403" t="n"/>
+      <c r="F8" s="404" t="n"/>
+      <c r="G8" s="405" t="n"/>
+      <c r="H8" s="403" t="n"/>
+      <c r="I8" s="404" t="n"/>
+      <c r="J8" s="405" t="n"/>
+      <c r="K8" s="403" t="n"/>
+      <c r="L8" s="404" t="n"/>
+      <c r="M8" s="405" t="n"/>
+    </row>
+    <row r="9" ht="20" customHeight="1" s="50">
+      <c r="B9" s="410" t="inlineStr">
+        <is>
+          <t>↑ Aktif portföy risk hacmi</t>
+        </is>
+      </c>
+      <c r="C9" s="411" t="n"/>
+      <c r="D9" s="412" t="n"/>
+      <c r="E9" s="413" t="inlineStr">
+        <is>
+          <t>● 30 gün içinde vadesi gelen taksitler</t>
+        </is>
+      </c>
+      <c r="F9" s="411" t="n"/>
+      <c r="G9" s="412" t="n"/>
+      <c r="H9" s="410" t="inlineStr">
+        <is>
+          <t>✓ Yapılandırma ile aylık nakit kazanımı</t>
+        </is>
+      </c>
+      <c r="I9" s="411" t="n"/>
+      <c r="J9" s="412" t="n"/>
+      <c r="K9" s="414">
+        <f>KARAR_MOTORU!B17</f>
+        <v/>
+      </c>
+      <c r="L9" s="411" t="n"/>
+      <c r="M9" s="412" t="n"/>
+    </row>
+    <row r="10" ht="16" customHeight="1" s="50"/>
+    <row r="11" ht="24" customHeight="1" s="50">
+      <c r="B11" s="74" t="inlineStr">
+        <is>
+          <t>BANKA, KREDI VE TAKSIT TAKIP SISTEMI — DÖNEMSEL İCRA VE PROJEKSİYON</t>
+        </is>
+      </c>
+      <c r="F11" s="144" t="inlineStr">
+        <is>
+          <t>+%32 Verim</t>
+        </is>
+      </c>
+      <c r="H11" s="74" t="inlineStr">
+        <is>
+          <t>KONSOLİDE OPERASYON VE KARAR MATRİSİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="50">
+      <c r="B12" s="73" t="inlineStr">
+        <is>
+          <t>Kümülatif Hacim vs. Operasyonel Maliyet ve Net Kâr Eğilimi</t>
+        </is>
+      </c>
+      <c r="H12" s="73" t="inlineStr">
+        <is>
+          <t>Anlık Hesaplama Sonuçları, Dinamik Formül Çıktıları ve Durum Puanlaması</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="8" customHeight="1" s="50"/>
+    <row r="14" ht="26" customHeight="1" s="50">
+      <c r="B14" s="145" t="inlineStr">
+        <is>
+          <t>Dönem</t>
+        </is>
+      </c>
+      <c r="C14" s="145" t="inlineStr">
+        <is>
+          <t>Aktif Hacim</t>
+        </is>
+      </c>
+      <c r="D14" s="145" t="inlineStr">
+        <is>
+          <t>Maliyet/Yük</t>
+        </is>
+      </c>
+      <c r="E14" s="145" t="inlineStr">
+        <is>
+          <t>Hedef</t>
+        </is>
+      </c>
+      <c r="H14" s="146" t="inlineStr">
+        <is>
+          <t>PARAMETRE / KALEM</t>
+        </is>
+      </c>
+      <c r="I14" s="146" t="inlineStr">
+        <is>
+          <t>ANA TUTAR</t>
+        </is>
+      </c>
+      <c r="J14" s="146" t="inlineStr">
+        <is>
+          <t>FARK / MARJ</t>
+        </is>
+      </c>
+      <c r="K14" s="146" t="inlineStr">
+        <is>
+          <t>VADE</t>
+        </is>
+      </c>
+      <c r="L14" s="146" t="inlineStr">
+        <is>
+          <t>KONTROL DURUMU</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1" s="50">
+      <c r="B15" s="73" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="C15" s="73" t="n">
+        <v>65</v>
+      </c>
+      <c r="D15" s="73" t="n">
+        <v>45</v>
+      </c>
+      <c r="E15" s="73" t="n">
+        <v>60</v>
+      </c>
+      <c r="H15" s="147" t="inlineStr">
+        <is>
+          <t>Dönemlik Kümülatif Bakiye</t>
+        </is>
+      </c>
+      <c r="I15" s="227">
+        <f>B7*0.45</f>
+        <v/>
+      </c>
+      <c r="J15" s="228">
+        <f>B7*0.05</f>
+        <v/>
+      </c>
+      <c r="K15" s="149" t="inlineStr">
+        <is>
+          <t>12 Ay</t>
+        </is>
+      </c>
+      <c r="L15" s="133" t="inlineStr">
+        <is>
+          <t>✓ DÜZENLİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1" s="50">
+      <c r="B16" s="73" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="C16" s="73" t="n">
+        <v>78</v>
+      </c>
+      <c r="D16" s="73" t="n">
+        <v>48</v>
+      </c>
+      <c r="E16" s="73" t="n">
+        <v>70</v>
+      </c>
+      <c r="H16" s="147" t="inlineStr">
+        <is>
+          <t>Kritik Eşik Güvenlik Tamponu</t>
+        </is>
+      </c>
+      <c r="I16" s="227">
+        <f>B7*0.30</f>
+        <v/>
+      </c>
+      <c r="J16" s="228">
+        <f>B7*0.03</f>
+        <v/>
+      </c>
+      <c r="K16" s="149" t="inlineStr">
+        <is>
+          <t>24 Ay</t>
+        </is>
+      </c>
+      <c r="L16" s="130" t="inlineStr">
+        <is>
+          <t>★ AVANTAJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1" s="50">
+      <c r="B17" s="73" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="C17" s="73" t="n">
+        <v>85</v>
+      </c>
+      <c r="D17" s="73" t="n">
+        <v>55</v>
+      </c>
+      <c r="E17" s="73" t="n">
+        <v>80</v>
+      </c>
+      <c r="H17" s="147" t="inlineStr">
+        <is>
+          <t>Operasyonel Net Fark</t>
+        </is>
+      </c>
+      <c r="I17" s="227">
+        <f>B7*0.15</f>
+        <v/>
+      </c>
+      <c r="J17" s="228">
+        <f>B7*0.02</f>
+        <v/>
+      </c>
+      <c r="K17" s="149" t="inlineStr">
+        <is>
+          <t>8 Ay</t>
+        </is>
+      </c>
+      <c r="L17" s="150" t="inlineStr">
+        <is>
+          <t>● YAKLAŞAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1" s="50">
+      <c r="B18" s="73" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="C18" s="73" t="n">
+        <v>75</v>
+      </c>
+      <c r="D18" s="73" t="n">
+        <v>42</v>
+      </c>
+      <c r="E18" s="73" t="n">
+        <v>75</v>
+      </c>
+      <c r="H18" s="147" t="inlineStr">
+        <is>
+          <t>Rezerv ve Likit Dağılım</t>
+        </is>
+      </c>
+      <c r="I18" s="227">
+        <f>B7*0.10</f>
+        <v/>
+      </c>
+      <c r="J18" s="228">
+        <f>B7*0.01</f>
+        <v/>
+      </c>
+      <c r="K18" s="149" t="inlineStr">
+        <is>
+          <t>16 Ay</t>
+        </is>
+      </c>
+      <c r="L18" s="133" t="inlineStr">
+        <is>
+          <t>✓ TAM UYUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="26" customHeight="1" s="50">
+      <c r="B19" s="73" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="C19" s="73" t="n">
+        <v>90</v>
+      </c>
+      <c r="D19" s="73" t="n">
+        <v>40</v>
+      </c>
+      <c r="E19" s="73" t="n">
+        <v>85</v>
+      </c>
+      <c r="H19" s="151" t="inlineStr">
+        <is>
+          <t>KONSOLİDE SİSTEM TOPLAMI</t>
+        </is>
+      </c>
+      <c r="I19" s="229">
+        <f>SUM(I15:I18)</f>
+        <v/>
+      </c>
+      <c r="J19" s="230">
+        <f>SUM(J15:J18)</f>
+        <v/>
+      </c>
+      <c r="K19" s="154" t="inlineStr"/>
+      <c r="L19" s="155" t="inlineStr">
+        <is>
+          <t>TAM DOĞRULANDI (0 HATA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1" s="50">
+      <c r="B20" s="73" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="C20" s="73" t="n">
+        <v>96</v>
+      </c>
+      <c r="D20" s="73" t="n">
+        <v>32</v>
+      </c>
+      <c r="E20" s="73" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="21" ht="8" customHeight="1" s="50"/>
+    <row r="22" ht="24" customHeight="1" s="50">
+      <c r="B22" s="156" t="inlineStr">
+        <is>
+          <t>KONSOLİDE PAY VE AĞIRLIK</t>
+        </is>
+      </c>
+      <c r="F22" s="156" t="inlineStr">
+        <is>
+          <t>LİKİDİTE RİSKİ &amp; ERKEN UYARI SİNYALLERİ</t>
+        </is>
+      </c>
+      <c r="K22" s="157" t="inlineStr">
+        <is>
+          <t>KARAR MOTORU PROTOKOLÜ</t>
+        </is>
+      </c>
+      <c r="L22" s="158" t="n"/>
+      <c r="M22" s="158" t="n"/>
+    </row>
+    <row r="23" ht="22" customHeight="1" s="50">
+      <c r="B23" s="58" t="inlineStr">
+        <is>
+          <t>■ Ana Segment (%42)</t>
+        </is>
+      </c>
+      <c r="F23" s="73" t="inlineStr">
+        <is>
+          <t>Nakit Açığı Riski (30 Gün)</t>
+        </is>
+      </c>
+      <c r="I23" s="159" t="inlineStr">
+        <is>
+          <t>0.00 TL (Sıfır Risk)</t>
+        </is>
+      </c>
+      <c r="K23" s="160" t="inlineStr">
+        <is>
+          <t>REFİNANSMAN &amp; LİKİDİTE</t>
+        </is>
+      </c>
+      <c r="L23" s="158" t="n"/>
+      <c r="M23" s="158" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1" s="50">
+      <c r="B24" s="59" t="inlineStr">
+        <is>
+          <t>■ İkincil Grup (%30)</t>
+        </is>
+      </c>
+      <c r="F24" s="73" t="inlineStr">
+        <is>
+          <t>Tahsilat Gecikme Toleransı</t>
+        </is>
+      </c>
+      <c r="I24" s="159" t="inlineStr">
+        <is>
+          <t>48 Gün Güvenli Eşik</t>
+        </is>
+      </c>
+      <c r="K24" s="161" t="inlineStr">
+        <is>
+          <t>Sistem, nakit açığı riskini 30/60/90 günlük pencerelerde izleyerek, borç servisi oranını optimal eşikte tutacak yapılandırma önerir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1" s="50">
+      <c r="B25" s="162" t="inlineStr">
+        <is>
+          <t>■ Destek Birimi (%15)</t>
+        </is>
+      </c>
+      <c r="F25" s="58" t="inlineStr">
+        <is>
+          <t>██████████████████████████████████████ Güvenli Bölge (%100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1" s="50">
+      <c r="B26" s="163" t="inlineStr">
+        <is>
+          <t>■ Rezervler (%13)</t>
+        </is>
+      </c>
+      <c r="F26" s="164" t="inlineStr">
+        <is>
+          <t>✓ 90 GÜNLÜK PROJEKSİYONDA NAKİT SIKIŞIKLIĞI TESPİT EDİLMEDİ</t>
+        </is>
+      </c>
+      <c r="G26" s="247" t="n"/>
+      <c r="H26" s="247" t="n"/>
+      <c r="I26" s="248" t="n"/>
+      <c r="K26" s="165" t="inlineStr">
+        <is>
+          <t>REFİNANSMAN ANALİZİNİ GÖR (#REFINANSMAN!A1) &gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="10" customHeight="1" s="50">
+      <c r="F27" s="249" t="n"/>
+      <c r="G27" s="250" t="n"/>
+      <c r="H27" s="250" t="n"/>
+      <c r="I27" s="251" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="K26:M27"/>
+    <mergeCell ref="K24:M25"/>
+    <mergeCell ref="F26:I27"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -23951,7 +25328,473 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:AN16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="40" customWidth="1" style="76" min="1" max="1"/>
+    <col width="20" customWidth="1" style="76" min="2" max="2"/>
+    <col width="18" customWidth="1" style="76" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25.5" customHeight="1" s="50">
+      <c r="A1" s="77" t="inlineStr">
+        <is>
+          <t>TESTLER — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="50">
+      <c r="A3" s="99" t="inlineStr">
+        <is>
+          <t>SİSTEM TESTLERİ VE DENETİM KAYDI</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1" s="50">
+      <c r="A5" s="86" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="B5" s="86" t="inlineStr">
+        <is>
+          <t>Canlı Değer</t>
+        </is>
+      </c>
+      <c r="C5" s="86" t="inlineStr">
+        <is>
+          <t>Durum</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="50">
+      <c r="A6" s="81" t="inlineStr">
+        <is>
+          <t>Toplam Finansal Borç</t>
+        </is>
+      </c>
+      <c r="B6" s="92">
+        <f>KARAR_MOTORU!$B$5</f>
+        <v/>
+      </c>
+      <c r="C6" s="89">
+        <f>IF(B6="","EKSİK","KONTROL EDİLDİ")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1" s="50">
+      <c r="A7" s="81" t="inlineStr">
+        <is>
+          <t>30 Günlük Ödeme Yükü</t>
+        </is>
+      </c>
+      <c r="B7" s="92">
+        <f>KARAR_MOTORU!$B$7</f>
+        <v/>
+      </c>
+      <c r="C7" s="89">
+        <f>IF(B7="","EKSİK","KONTROL EDİLDİ")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="50">
+      <c r="A8" s="81" t="inlineStr">
+        <is>
+          <t>Ağırlıklı Maliyet</t>
+        </is>
+      </c>
+      <c r="B8" s="93">
+        <f>KARAR_MOTORU!$B$9</f>
+        <v/>
+      </c>
+      <c r="C8" s="89">
+        <f>IF(B8="","EKSİK","KONTROL EDİLDİ")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="50">
+      <c r="A9" s="81" t="inlineStr">
+        <is>
+          <t>Veri Kalite Skoru</t>
+        </is>
+      </c>
+      <c r="B9" s="97">
+        <f>KONTROLLER!$B$6</f>
+        <v/>
+      </c>
+      <c r="C9" s="89">
+        <f>IF(B9="","EKSİK","KONTROL EDİLDİ")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="50">
+      <c r="A10" s="81" t="inlineStr">
+        <is>
+          <t>Karar Bildirimi</t>
+        </is>
+      </c>
+      <c r="B10" s="89">
+        <f>KARAR_MOTORU!$B$15</f>
+        <v/>
+      </c>
+      <c r="C10" s="89">
+        <f>IF(B10="","EKSİK","KONTROL EDİLDİ")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="50">
+      <c r="A11" s="81" t="inlineStr">
+        <is>
+          <t>Risk Seviyesi</t>
+        </is>
+      </c>
+      <c r="B11" s="89">
+        <f>KARAR_MOTORU!$B$16</f>
+        <v/>
+      </c>
+      <c r="C11" s="89">
+        <f>IF(B11="","EKSİK","KONTROL EDİLDİ")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="50">
+      <c r="A12" s="81" t="inlineStr">
+        <is>
+          <t>Refinansman Aday Sayısı</t>
+        </is>
+      </c>
+      <c r="B12" s="97">
+        <f>KARAR_MOTORU!$B$18</f>
+        <v/>
+      </c>
+      <c r="C12" s="89">
+        <f>IF(B12="","EKSİK","KONTROL EDİLDİ")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="24.75" customHeight="1" s="50">
+      <c r="A16" s="82" t="inlineStr">
+        <is>
+          <t>Testler, excel_uretim/denetci.py ve test_banka_kredi.py ile otomatik çalışır.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:AN1"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="12" customWidth="1" style="76" min="1" max="1"/>
+    <col width="16" customWidth="1" style="76" min="2" max="2"/>
+    <col width="14" customWidth="1" style="76" min="3" max="4"/>
+    <col width="10" customWidth="1" style="76" min="5" max="5"/>
+    <col width="14" customWidth="1" style="76" min="6" max="6"/>
+    <col width="40" customWidth="1" style="76" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1" s="50">
+      <c r="A1" s="76" t="inlineStr">
+        <is>
+          <t>AKIS — BankaKrediVeTaksitTakipSistemi</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="50">
+      <c r="A3" s="76" t="inlineStr">
+        <is>
+          <t>islem_id</t>
+        </is>
+      </c>
+      <c r="B3" s="76" t="inlineStr">
+        <is>
+          <t>kaynak_kart_id</t>
+        </is>
+      </c>
+      <c r="C3" s="76" t="inlineStr">
+        <is>
+          <t>onceki_durum</t>
+        </is>
+      </c>
+      <c r="D3" s="76" t="inlineStr">
+        <is>
+          <t>yeni_durum</t>
+        </is>
+      </c>
+      <c r="E3" s="76" t="inlineStr">
+        <is>
+          <t>tutar</t>
+        </is>
+      </c>
+      <c r="F3" s="76" t="inlineStr">
+        <is>
+          <t>bayrak</t>
+        </is>
+      </c>
+      <c r="G3" s="76" t="inlineStr">
+        <is>
+          <t>not</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="50">
+      <c r="A4" s="76" t="inlineStr">
+        <is>
+          <t>I-001</t>
+        </is>
+      </c>
+      <c r="B4" s="76" t="inlineStr">
+        <is>
+          <t>KART-01</t>
+        </is>
+      </c>
+      <c r="C4" s="76" t="inlineStr">
+        <is>
+          <t>ACIK</t>
+        </is>
+      </c>
+      <c r="D4" s="76" t="inlineStr">
+        <is>
+          <t>ISLEMDE</t>
+        </is>
+      </c>
+      <c r="E4" s="119" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F4" s="76" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G4" s="76" t="inlineStr">
+        <is>
+          <t>normal geçiş</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="50">
+      <c r="A5" s="76" t="inlineStr">
+        <is>
+          <t>I-002</t>
+        </is>
+      </c>
+      <c r="B5" s="76" t="inlineStr">
+        <is>
+          <t>YETİM</t>
+        </is>
+      </c>
+      <c r="C5" s="76" t="inlineStr">
+        <is>
+          <t>ACIK</t>
+        </is>
+      </c>
+      <c r="D5" s="76" t="inlineStr">
+        <is>
+          <t>KAPALI</t>
+        </is>
+      </c>
+      <c r="E5" s="119" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="76" t="inlineStr">
+        <is>
+          <t>YETİM</t>
+        </is>
+      </c>
+      <c r="G5" s="76" t="inlineStr">
+        <is>
+          <t>kaynak_kart_id yok — yetim kayıt</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="50">
+      <c r="A6" s="76" t="inlineStr">
+        <is>
+          <t>I-003</t>
+        </is>
+      </c>
+      <c r="B6" s="76" t="inlineStr">
+        <is>
+          <t>KART-02</t>
+        </is>
+      </c>
+      <c r="C6" s="76" t="inlineStr">
+        <is>
+          <t>ACIK</t>
+        </is>
+      </c>
+      <c r="D6" s="76" t="inlineStr">
+        <is>
+          <t>KAPALI</t>
+        </is>
+      </c>
+      <c r="E6" s="119" t="n">
+        <v>500</v>
+      </c>
+      <c r="F6" s="76" t="inlineStr">
+        <is>
+          <t>GECERSIZ</t>
+        </is>
+      </c>
+      <c r="G6" s="76" t="inlineStr">
+        <is>
+          <t>geçersiz durum geçişi</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1" s="50">
+      <c r="A7" s="76" t="inlineStr">
+        <is>
+          <t>I-004</t>
+        </is>
+      </c>
+      <c r="B7" s="76" t="inlineStr">
+        <is>
+          <t>KART-03</t>
+        </is>
+      </c>
+      <c r="C7" s="76" t="inlineStr">
+        <is>
+          <t>ISLEMDE</t>
+        </is>
+      </c>
+      <c r="D7" s="76" t="inlineStr">
+        <is>
+          <t>ISLEMDE</t>
+        </is>
+      </c>
+      <c r="E7" s="119" t="n">
+        <v>250</v>
+      </c>
+      <c r="F7" s="76" t="inlineStr">
+        <is>
+          <t>ZINCIR_KIRIK</t>
+        </is>
+      </c>
+      <c r="G7" s="76" t="inlineStr">
+        <is>
+          <t>ZİNCİR KIRIK — tutar zinciri sapması</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="50">
+      <c r="A9" s="76" t="inlineStr">
+        <is>
+          <t>kuyruk_kanit</t>
+        </is>
+      </c>
+      <c r="B9" s="76">
+        <f>IFERROR(COUNTIF($F$4:$F$1000,"OK"),0)</f>
+        <v/>
+      </c>
+      <c r="C9" s="76" t="n"/>
+      <c r="D9" s="76" t="n"/>
+      <c r="E9" s="76" t="n"/>
+      <c r="F9" s="76" t="n"/>
+      <c r="G9" s="76" t="n"/>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:AN6"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="12" customWidth="1" style="76" min="1" max="1"/>
+    <col width="14" customWidth="1" style="76" min="2" max="2"/>
+    <col width="90" customWidth="1" style="76" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25.5" customHeight="1" s="50">
+      <c r="A1" s="77" t="inlineStr">
+        <is>
+          <t>DEGISIKLIK KAYDI — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="50">
+      <c r="A3" s="99" t="inlineStr">
+        <is>
+          <t>DEĞİŞİKLİK KAYDI</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1" s="50">
+      <c r="A5" s="86" t="inlineStr">
+        <is>
+          <t>Sürüm</t>
+        </is>
+      </c>
+      <c r="B5" s="86" t="inlineStr">
+        <is>
+          <t>Tarih</t>
+        </is>
+      </c>
+      <c r="C5" s="86" t="inlineStr">
+        <is>
+          <t>Açıklama</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="50">
+      <c r="A6" s="120" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="B6" s="120" t="inlineStr">
+        <is>
+          <t>08.08.2026</t>
+        </is>
+      </c>
+      <c r="C6" s="115" t="inlineStr">
+        <is>
+          <t>İlk sürüm: banka limitleri, kredi portföyü, taksit planı, refinansman analizi ve karar motoru.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:AN1"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00D97706"/>
@@ -24433,473 +26276,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:AN16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="40" customWidth="1" style="76" min="1" max="1"/>
-    <col width="20" customWidth="1" style="76" min="2" max="2"/>
-    <col width="18" customWidth="1" style="76" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="50">
-      <c r="A1" s="77" t="inlineStr">
-        <is>
-          <t>TESTLER — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="50">
-      <c r="A3" s="99" t="inlineStr">
-        <is>
-          <t>SİSTEM TESTLERİ VE DENETİM KAYDI</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1" s="50">
-      <c r="A5" s="86" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="B5" s="86" t="inlineStr">
-        <is>
-          <t>Canlı Değer</t>
-        </is>
-      </c>
-      <c r="C5" s="86" t="inlineStr">
-        <is>
-          <t>Durum</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="50">
-      <c r="A6" s="81" t="inlineStr">
-        <is>
-          <t>Toplam Finansal Borç</t>
-        </is>
-      </c>
-      <c r="B6" s="92">
-        <f>KARAR_MOTORU!$B$5</f>
-        <v/>
-      </c>
-      <c r="C6" s="89">
-        <f>IF(B6="","EKSİK","KONTROL EDİLDİ")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="50">
-      <c r="A7" s="81" t="inlineStr">
-        <is>
-          <t>30 Günlük Ödeme Yükü</t>
-        </is>
-      </c>
-      <c r="B7" s="92">
-        <f>KARAR_MOTORU!$B$7</f>
-        <v/>
-      </c>
-      <c r="C7" s="89">
-        <f>IF(B7="","EKSİK","KONTROL EDİLDİ")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="50">
-      <c r="A8" s="81" t="inlineStr">
-        <is>
-          <t>Ağırlıklı Maliyet</t>
-        </is>
-      </c>
-      <c r="B8" s="93">
-        <f>KARAR_MOTORU!$B$9</f>
-        <v/>
-      </c>
-      <c r="C8" s="89">
-        <f>IF(B8="","EKSİK","KONTROL EDİLDİ")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="50">
-      <c r="A9" s="81" t="inlineStr">
-        <is>
-          <t>Veri Kalite Skoru</t>
-        </is>
-      </c>
-      <c r="B9" s="97">
-        <f>KONTROLLER!$B$6</f>
-        <v/>
-      </c>
-      <c r="C9" s="89">
-        <f>IF(B9="","EKSİK","KONTROL EDİLDİ")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="50">
-      <c r="A10" s="81" t="inlineStr">
-        <is>
-          <t>Karar Bildirimi</t>
-        </is>
-      </c>
-      <c r="B10" s="89">
-        <f>KARAR_MOTORU!$B$15</f>
-        <v/>
-      </c>
-      <c r="C10" s="89">
-        <f>IF(B10="","EKSİK","KONTROL EDİLDİ")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="50">
-      <c r="A11" s="81" t="inlineStr">
-        <is>
-          <t>Risk Seviyesi</t>
-        </is>
-      </c>
-      <c r="B11" s="89">
-        <f>KARAR_MOTORU!$B$16</f>
-        <v/>
-      </c>
-      <c r="C11" s="89">
-        <f>IF(B11="","EKSİK","KONTROL EDİLDİ")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="50">
-      <c r="A12" s="81" t="inlineStr">
-        <is>
-          <t>Refinansman Aday Sayısı</t>
-        </is>
-      </c>
-      <c r="B12" s="97">
-        <f>KARAR_MOTORU!$B$18</f>
-        <v/>
-      </c>
-      <c r="C12" s="89">
-        <f>IF(B12="","EKSİK","KONTROL EDİLDİ")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="24.75" customHeight="1" s="50">
-      <c r="A16" s="82" t="inlineStr">
-        <is>
-          <t>Testler, excel_uretim/denetci.py ve test_banka_kredi.py ile otomatik çalışır.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AN1"/>
-  </mergeCells>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:G9"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="12" customWidth="1" style="76" min="1" max="1"/>
-    <col width="16" customWidth="1" style="76" min="2" max="2"/>
-    <col width="14" customWidth="1" style="76" min="3" max="4"/>
-    <col width="10" customWidth="1" style="76" min="5" max="5"/>
-    <col width="14" customWidth="1" style="76" min="6" max="6"/>
-    <col width="40" customWidth="1" style="76" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15" customHeight="1" s="50">
-      <c r="A1" s="76" t="inlineStr">
-        <is>
-          <t>AKIS — BankaKrediVeTaksitTakipSistemi</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="50">
-      <c r="A3" s="76" t="inlineStr">
-        <is>
-          <t>islem_id</t>
-        </is>
-      </c>
-      <c r="B3" s="76" t="inlineStr">
-        <is>
-          <t>kaynak_kart_id</t>
-        </is>
-      </c>
-      <c r="C3" s="76" t="inlineStr">
-        <is>
-          <t>onceki_durum</t>
-        </is>
-      </c>
-      <c r="D3" s="76" t="inlineStr">
-        <is>
-          <t>yeni_durum</t>
-        </is>
-      </c>
-      <c r="E3" s="76" t="inlineStr">
-        <is>
-          <t>tutar</t>
-        </is>
-      </c>
-      <c r="F3" s="76" t="inlineStr">
-        <is>
-          <t>bayrak</t>
-        </is>
-      </c>
-      <c r="G3" s="76" t="inlineStr">
-        <is>
-          <t>not</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="50">
-      <c r="A4" s="76" t="inlineStr">
-        <is>
-          <t>I-001</t>
-        </is>
-      </c>
-      <c r="B4" s="76" t="inlineStr">
-        <is>
-          <t>KART-01</t>
-        </is>
-      </c>
-      <c r="C4" s="76" t="inlineStr">
-        <is>
-          <t>ACIK</t>
-        </is>
-      </c>
-      <c r="D4" s="76" t="inlineStr">
-        <is>
-          <t>ISLEMDE</t>
-        </is>
-      </c>
-      <c r="E4" s="119" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F4" s="76" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="G4" s="76" t="inlineStr">
-        <is>
-          <t>normal geçiş</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="50">
-      <c r="A5" s="76" t="inlineStr">
-        <is>
-          <t>I-002</t>
-        </is>
-      </c>
-      <c r="B5" s="76" t="inlineStr">
-        <is>
-          <t>YETİM</t>
-        </is>
-      </c>
-      <c r="C5" s="76" t="inlineStr">
-        <is>
-          <t>ACIK</t>
-        </is>
-      </c>
-      <c r="D5" s="76" t="inlineStr">
-        <is>
-          <t>KAPALI</t>
-        </is>
-      </c>
-      <c r="E5" s="119" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="76" t="inlineStr">
-        <is>
-          <t>YETİM</t>
-        </is>
-      </c>
-      <c r="G5" s="76" t="inlineStr">
-        <is>
-          <t>kaynak_kart_id yok — yetim kayıt</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="50">
-      <c r="A6" s="76" t="inlineStr">
-        <is>
-          <t>I-003</t>
-        </is>
-      </c>
-      <c r="B6" s="76" t="inlineStr">
-        <is>
-          <t>KART-02</t>
-        </is>
-      </c>
-      <c r="C6" s="76" t="inlineStr">
-        <is>
-          <t>ACIK</t>
-        </is>
-      </c>
-      <c r="D6" s="76" t="inlineStr">
-        <is>
-          <t>KAPALI</t>
-        </is>
-      </c>
-      <c r="E6" s="119" t="n">
-        <v>500</v>
-      </c>
-      <c r="F6" s="76" t="inlineStr">
-        <is>
-          <t>GECERSIZ</t>
-        </is>
-      </c>
-      <c r="G6" s="76" t="inlineStr">
-        <is>
-          <t>geçersiz durum geçişi</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="50">
-      <c r="A7" s="76" t="inlineStr">
-        <is>
-          <t>I-004</t>
-        </is>
-      </c>
-      <c r="B7" s="76" t="inlineStr">
-        <is>
-          <t>KART-03</t>
-        </is>
-      </c>
-      <c r="C7" s="76" t="inlineStr">
-        <is>
-          <t>ISLEMDE</t>
-        </is>
-      </c>
-      <c r="D7" s="76" t="inlineStr">
-        <is>
-          <t>ISLEMDE</t>
-        </is>
-      </c>
-      <c r="E7" s="119" t="n">
-        <v>250</v>
-      </c>
-      <c r="F7" s="76" t="inlineStr">
-        <is>
-          <t>ZINCIR_KIRIK</t>
-        </is>
-      </c>
-      <c r="G7" s="76" t="inlineStr">
-        <is>
-          <t>ZİNCİR KIRIK — tutar zinciri sapması</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="50">
-      <c r="A9" s="76" t="inlineStr">
-        <is>
-          <t>kuyruk_kanit</t>
-        </is>
-      </c>
-      <c r="B9" s="76">
-        <f>IFERROR(COUNTIF($F$4:$F$1000,"OK"),0)</f>
-        <v/>
-      </c>
-      <c r="C9" s="76" t="n"/>
-      <c r="D9" s="76" t="n"/>
-      <c r="E9" s="76" t="n"/>
-      <c r="F9" s="76" t="n"/>
-      <c r="G9" s="76" t="n"/>
-    </row>
-  </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:AN6"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="12" customWidth="1" style="76" min="1" max="1"/>
-    <col width="14" customWidth="1" style="76" min="2" max="2"/>
-    <col width="90" customWidth="1" style="76" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="50">
-      <c r="A1" s="77" t="inlineStr">
-        <is>
-          <t>DEGISIKLIK KAYDI — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="50">
-      <c r="A3" s="99" t="inlineStr">
-        <is>
-          <t>DEĞİŞİKLİK KAYDI</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1" s="50">
-      <c r="A5" s="86" t="inlineStr">
-        <is>
-          <t>Sürüm</t>
-        </is>
-      </c>
-      <c r="B5" s="86" t="inlineStr">
-        <is>
-          <t>Tarih</t>
-        </is>
-      </c>
-      <c r="C5" s="86" t="inlineStr">
-        <is>
-          <t>Açıklama</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="50">
-      <c r="A6" s="120" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="B6" s="120" t="inlineStr">
-        <is>
-          <t>08.08.2026</t>
-        </is>
-      </c>
-      <c r="C6" s="115" t="inlineStr">
-        <is>
-          <t>İlk sürüm: banka limitleri, kredi portföyü, taksit planı, refinansman analizi ve karar motoru.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AN1"/>
-  </mergeCells>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <tabColor rgb="0060A5FA"/>
@@ -25563,7 +26940,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <tabColor rgb="0060A5FA"/>
@@ -26377,7 +27754,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <tabColor rgb="0060A5FA"/>
@@ -27427,7 +28804,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <tabColor rgb="0060A5FA"/>
@@ -28424,7 +29801,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <tabColor rgb="0060A5FA"/>
@@ -29439,632 +30816,4 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <tabColor rgb="0060A5FA"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:AN35"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="11" customWidth="1" style="76" min="1" max="2"/>
-    <col width="24" customWidth="1" style="76" min="3" max="3"/>
-    <col width="18" customWidth="1" style="76" min="4" max="4"/>
-    <col width="13" customWidth="1" style="76" min="5" max="5"/>
-    <col width="15" customWidth="1" style="76" min="6" max="6"/>
-    <col width="14" customWidth="1" style="76" min="7" max="7"/>
-    <col width="13" customWidth="1" style="76" min="8" max="8"/>
-    <col width="10" customWidth="1" style="76" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="50">
-      <c r="A1" s="77" t="inlineStr">
-        <is>
-          <t>MASRAF KOMISYON — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="150" customHeight="1" s="50">
-      <c r="A3" s="85" t="inlineStr">
-        <is>
-          <t>MASRAF VE KOMİSYONLAR — tahsis, sigorta, komisyon ve diğer finansman maliyetleri.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1" s="50">
-      <c r="A5" s="86" t="inlineStr">
-        <is>
-          <t>Masraf ID</t>
-        </is>
-      </c>
-      <c r="B5" s="86" t="inlineStr">
-        <is>
-          <t>Kredi ID</t>
-        </is>
-      </c>
-      <c r="C5" s="86" t="inlineStr">
-        <is>
-          <t>Banka</t>
-        </is>
-      </c>
-      <c r="D5" s="86" t="inlineStr">
-        <is>
-          <t>Masraf Türü</t>
-        </is>
-      </c>
-      <c r="E5" s="86" t="inlineStr">
-        <is>
-          <t>İşlem Tarihi</t>
-        </is>
-      </c>
-      <c r="F5" s="86" t="inlineStr">
-        <is>
-          <t>Belge Numarası</t>
-        </is>
-      </c>
-      <c r="G5" s="86" t="inlineStr">
-        <is>
-          <t>Tutar</t>
-        </is>
-      </c>
-      <c r="H5" s="86" t="inlineStr">
-        <is>
-          <t>Para Birimi</t>
-        </is>
-      </c>
-      <c r="I5" s="86" t="inlineStr">
-        <is>
-          <t>Kontrol</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="50">
-      <c r="A6" s="87" t="inlineStr">
-        <is>
-          <t>MSF-001</t>
-        </is>
-      </c>
-      <c r="B6" s="87" t="inlineStr">
-        <is>
-          <t>KRD-001</t>
-        </is>
-      </c>
-      <c r="C6" s="87" t="inlineStr">
-        <is>
-          <t>Türkiye İş Bankası</t>
-        </is>
-      </c>
-      <c r="D6" s="87" t="inlineStr">
-        <is>
-          <t>Tahsis Ücreti</t>
-        </is>
-      </c>
-      <c r="E6" s="94" t="n">
-        <v>45597</v>
-      </c>
-      <c r="F6" s="87" t="inlineStr">
-        <is>
-          <t>FTR-1001</t>
-        </is>
-      </c>
-      <c r="G6" s="91" t="n">
-        <v>60000</v>
-      </c>
-      <c r="H6" s="87" t="inlineStr">
-        <is>
-          <t>TRY</t>
-        </is>
-      </c>
-      <c r="I6" s="89">
-        <f>IF(ISBLANK($A6),"",IF(OR(ISBLANK($B6),ISBLANK($C6),ISBLANK($D6),ISBLANK($E6),ISBLANK($F6),ISBLANK($G6),ISBLANK($H6)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="50">
-      <c r="A7" s="87" t="inlineStr">
-        <is>
-          <t>MSF-002</t>
-        </is>
-      </c>
-      <c r="B7" s="87" t="inlineStr">
-        <is>
-          <t>KRD-002</t>
-        </is>
-      </c>
-      <c r="C7" s="87" t="inlineStr">
-        <is>
-          <t>Akbank</t>
-        </is>
-      </c>
-      <c r="D7" s="87" t="inlineStr">
-        <is>
-          <t>Sigorta</t>
-        </is>
-      </c>
-      <c r="E7" s="94" t="n">
-        <v>45717</v>
-      </c>
-      <c r="F7" s="87" t="inlineStr">
-        <is>
-          <t>POL-2001</t>
-        </is>
-      </c>
-      <c r="G7" s="91" t="n">
-        <v>70000</v>
-      </c>
-      <c r="H7" s="87" t="inlineStr">
-        <is>
-          <t>TRY</t>
-        </is>
-      </c>
-      <c r="I7" s="89">
-        <f>IF(ISBLANK($A7),"",IF(OR(ISBLANK($B7),ISBLANK($C7),ISBLANK($D7),ISBLANK($E7),ISBLANK($F7),ISBLANK($G7),ISBLANK($H7)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="50">
-      <c r="A8" s="87" t="inlineStr">
-        <is>
-          <t>MSF-003</t>
-        </is>
-      </c>
-      <c r="B8" s="87" t="inlineStr">
-        <is>
-          <t>KRD-003</t>
-        </is>
-      </c>
-      <c r="C8" s="87" t="inlineStr">
-        <is>
-          <t>Garanti BBVA</t>
-        </is>
-      </c>
-      <c r="D8" s="87" t="inlineStr">
-        <is>
-          <t>Komisyon</t>
-        </is>
-      </c>
-      <c r="E8" s="94" t="n">
-        <v>45809</v>
-      </c>
-      <c r="F8" s="87" t="inlineStr">
-        <is>
-          <t>FTR-3001</t>
-        </is>
-      </c>
-      <c r="G8" s="91" t="n">
-        <v>1500</v>
-      </c>
-      <c r="H8" s="87" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="I8" s="89">
-        <f>IF(ISBLANK($A8),"",IF(OR(ISBLANK($B8),ISBLANK($C8),ISBLANK($D8),ISBLANK($E8),ISBLANK($F8),ISBLANK($G8),ISBLANK($H8)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="50">
-      <c r="A9" s="90" t="n"/>
-      <c r="B9" s="90" t="n"/>
-      <c r="C9" s="90" t="n"/>
-      <c r="D9" s="90" t="n"/>
-      <c r="E9" s="90" t="n"/>
-      <c r="F9" s="90" t="n"/>
-      <c r="G9" s="90" t="n"/>
-      <c r="H9" s="90" t="n"/>
-      <c r="I9" s="89">
-        <f>IF(ISBLANK($A9),"",IF(OR(ISBLANK($B9),ISBLANK($C9),ISBLANK($D9),ISBLANK($E9),ISBLANK($F9),ISBLANK($G9),ISBLANK($H9)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="50">
-      <c r="A10" s="90" t="n"/>
-      <c r="B10" s="90" t="n"/>
-      <c r="C10" s="90" t="n"/>
-      <c r="D10" s="90" t="n"/>
-      <c r="E10" s="90" t="n"/>
-      <c r="F10" s="90" t="n"/>
-      <c r="G10" s="90" t="n"/>
-      <c r="H10" s="90" t="n"/>
-      <c r="I10" s="89">
-        <f>IF(ISBLANK($A10),"",IF(OR(ISBLANK($B10),ISBLANK($C10),ISBLANK($D10),ISBLANK($E10),ISBLANK($F10),ISBLANK($G10),ISBLANK($H10)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="50">
-      <c r="A11" s="90" t="n"/>
-      <c r="B11" s="90" t="n"/>
-      <c r="C11" s="90" t="n"/>
-      <c r="D11" s="90" t="n"/>
-      <c r="E11" s="90" t="n"/>
-      <c r="F11" s="90" t="n"/>
-      <c r="G11" s="90" t="n"/>
-      <c r="H11" s="90" t="n"/>
-      <c r="I11" s="89">
-        <f>IF(ISBLANK($A11),"",IF(OR(ISBLANK($B11),ISBLANK($C11),ISBLANK($D11),ISBLANK($E11),ISBLANK($F11),ISBLANK($G11),ISBLANK($H11)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="50">
-      <c r="A12" s="90" t="n"/>
-      <c r="B12" s="90" t="n"/>
-      <c r="C12" s="90" t="n"/>
-      <c r="D12" s="90" t="n"/>
-      <c r="E12" s="90" t="n"/>
-      <c r="F12" s="90" t="n"/>
-      <c r="G12" s="90" t="n"/>
-      <c r="H12" s="90" t="n"/>
-      <c r="I12" s="89">
-        <f>IF(ISBLANK($A12),"",IF(OR(ISBLANK($B12),ISBLANK($C12),ISBLANK($D12),ISBLANK($E12),ISBLANK($F12),ISBLANK($G12),ISBLANK($H12)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="50">
-      <c r="A13" s="90" t="n"/>
-      <c r="B13" s="90" t="n"/>
-      <c r="C13" s="90" t="n"/>
-      <c r="D13" s="90" t="n"/>
-      <c r="E13" s="90" t="n"/>
-      <c r="F13" s="90" t="n"/>
-      <c r="G13" s="90" t="n"/>
-      <c r="H13" s="90" t="n"/>
-      <c r="I13" s="89">
-        <f>IF(ISBLANK($A13),"",IF(OR(ISBLANK($B13),ISBLANK($C13),ISBLANK($D13),ISBLANK($E13),ISBLANK($F13),ISBLANK($G13),ISBLANK($H13)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="50">
-      <c r="A14" s="90" t="n"/>
-      <c r="B14" s="90" t="n"/>
-      <c r="C14" s="90" t="n"/>
-      <c r="D14" s="90" t="n"/>
-      <c r="E14" s="90" t="n"/>
-      <c r="F14" s="90" t="n"/>
-      <c r="G14" s="90" t="n"/>
-      <c r="H14" s="90" t="n"/>
-      <c r="I14" s="89">
-        <f>IF(ISBLANK($A14),"",IF(OR(ISBLANK($B14),ISBLANK($C14),ISBLANK($D14),ISBLANK($E14),ISBLANK($F14),ISBLANK($G14),ISBLANK($H14)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="50">
-      <c r="A15" s="90" t="n"/>
-      <c r="B15" s="90" t="n"/>
-      <c r="C15" s="90" t="n"/>
-      <c r="D15" s="90" t="n"/>
-      <c r="E15" s="90" t="n"/>
-      <c r="F15" s="90" t="n"/>
-      <c r="G15" s="90" t="n"/>
-      <c r="H15" s="90" t="n"/>
-      <c r="I15" s="89">
-        <f>IF(ISBLANK($A15),"",IF(OR(ISBLANK($B15),ISBLANK($C15),ISBLANK($D15),ISBLANK($E15),ISBLANK($F15),ISBLANK($G15),ISBLANK($H15)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="50">
-      <c r="A16" s="90" t="n"/>
-      <c r="B16" s="90" t="n"/>
-      <c r="C16" s="90" t="n"/>
-      <c r="D16" s="90" t="n"/>
-      <c r="E16" s="90" t="n"/>
-      <c r="F16" s="90" t="n"/>
-      <c r="G16" s="90" t="n"/>
-      <c r="H16" s="90" t="n"/>
-      <c r="I16" s="89">
-        <f>IF(ISBLANK($A16),"",IF(OR(ISBLANK($B16),ISBLANK($C16),ISBLANK($D16),ISBLANK($E16),ISBLANK($F16),ISBLANK($G16),ISBLANK($H16)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="50">
-      <c r="A17" s="90" t="n"/>
-      <c r="B17" s="90" t="n"/>
-      <c r="C17" s="90" t="n"/>
-      <c r="D17" s="90" t="n"/>
-      <c r="E17" s="90" t="n"/>
-      <c r="F17" s="90" t="n"/>
-      <c r="G17" s="90" t="n"/>
-      <c r="H17" s="90" t="n"/>
-      <c r="I17" s="89">
-        <f>IF(ISBLANK($A17),"",IF(OR(ISBLANK($B17),ISBLANK($C17),ISBLANK($D17),ISBLANK($E17),ISBLANK($F17),ISBLANK($G17),ISBLANK($H17)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1" s="50">
-      <c r="A18" s="90" t="n"/>
-      <c r="B18" s="90" t="n"/>
-      <c r="C18" s="90" t="n"/>
-      <c r="D18" s="90" t="n"/>
-      <c r="E18" s="90" t="n"/>
-      <c r="F18" s="90" t="n"/>
-      <c r="G18" s="90" t="n"/>
-      <c r="H18" s="90" t="n"/>
-      <c r="I18" s="89">
-        <f>IF(ISBLANK($A18),"",IF(OR(ISBLANK($B18),ISBLANK($C18),ISBLANK($D18),ISBLANK($E18),ISBLANK($F18),ISBLANK($G18),ISBLANK($H18)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="50">
-      <c r="A19" s="90" t="n"/>
-      <c r="B19" s="90" t="n"/>
-      <c r="C19" s="90" t="n"/>
-      <c r="D19" s="90" t="n"/>
-      <c r="E19" s="90" t="n"/>
-      <c r="F19" s="90" t="n"/>
-      <c r="G19" s="90" t="n"/>
-      <c r="H19" s="90" t="n"/>
-      <c r="I19" s="89">
-        <f>IF(ISBLANK($A19),"",IF(OR(ISBLANK($B19),ISBLANK($C19),ISBLANK($D19),ISBLANK($E19),ISBLANK($F19),ISBLANK($G19),ISBLANK($H19)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1" s="50">
-      <c r="A20" s="90" t="n"/>
-      <c r="B20" s="90" t="n"/>
-      <c r="C20" s="90" t="n"/>
-      <c r="D20" s="90" t="n"/>
-      <c r="E20" s="90" t="n"/>
-      <c r="F20" s="90" t="n"/>
-      <c r="G20" s="90" t="n"/>
-      <c r="H20" s="90" t="n"/>
-      <c r="I20" s="89">
-        <f>IF(ISBLANK($A20),"",IF(OR(ISBLANK($B20),ISBLANK($C20),ISBLANK($D20),ISBLANK($E20),ISBLANK($F20),ISBLANK($G20),ISBLANK($H20)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="15" customHeight="1" s="50">
-      <c r="A21" s="90" t="n"/>
-      <c r="B21" s="90" t="n"/>
-      <c r="C21" s="90" t="n"/>
-      <c r="D21" s="90" t="n"/>
-      <c r="E21" s="90" t="n"/>
-      <c r="F21" s="90" t="n"/>
-      <c r="G21" s="90" t="n"/>
-      <c r="H21" s="90" t="n"/>
-      <c r="I21" s="89">
-        <f>IF(ISBLANK($A21),"",IF(OR(ISBLANK($B21),ISBLANK($C21),ISBLANK($D21),ISBLANK($E21),ISBLANK($F21),ISBLANK($G21),ISBLANK($H21)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" ht="15" customHeight="1" s="50">
-      <c r="A22" s="90" t="n"/>
-      <c r="B22" s="90" t="n"/>
-      <c r="C22" s="90" t="n"/>
-      <c r="D22" s="90" t="n"/>
-      <c r="E22" s="90" t="n"/>
-      <c r="F22" s="90" t="n"/>
-      <c r="G22" s="90" t="n"/>
-      <c r="H22" s="90" t="n"/>
-      <c r="I22" s="89">
-        <f>IF(ISBLANK($A22),"",IF(OR(ISBLANK($B22),ISBLANK($C22),ISBLANK($D22),ISBLANK($E22),ISBLANK($F22),ISBLANK($G22),ISBLANK($H22)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="50">
-      <c r="A23" s="90" t="n"/>
-      <c r="B23" s="90" t="n"/>
-      <c r="C23" s="90" t="n"/>
-      <c r="D23" s="90" t="n"/>
-      <c r="E23" s="90" t="n"/>
-      <c r="F23" s="90" t="n"/>
-      <c r="G23" s="90" t="n"/>
-      <c r="H23" s="90" t="n"/>
-      <c r="I23" s="89">
-        <f>IF(ISBLANK($A23),"",IF(OR(ISBLANK($B23),ISBLANK($C23),ISBLANK($D23),ISBLANK($E23),ISBLANK($F23),ISBLANK($G23),ISBLANK($H23)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" ht="15" customHeight="1" s="50">
-      <c r="A24" s="90" t="n"/>
-      <c r="B24" s="90" t="n"/>
-      <c r="C24" s="90" t="n"/>
-      <c r="D24" s="90" t="n"/>
-      <c r="E24" s="90" t="n"/>
-      <c r="F24" s="90" t="n"/>
-      <c r="G24" s="90" t="n"/>
-      <c r="H24" s="90" t="n"/>
-      <c r="I24" s="89">
-        <f>IF(ISBLANK($A24),"",IF(OR(ISBLANK($B24),ISBLANK($C24),ISBLANK($D24),ISBLANK($E24),ISBLANK($F24),ISBLANK($G24),ISBLANK($H24)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" ht="15" customHeight="1" s="50">
-      <c r="A25" s="90" t="n"/>
-      <c r="B25" s="90" t="n"/>
-      <c r="C25" s="90" t="n"/>
-      <c r="D25" s="90" t="n"/>
-      <c r="E25" s="90" t="n"/>
-      <c r="F25" s="90" t="n"/>
-      <c r="G25" s="90" t="n"/>
-      <c r="H25" s="90" t="n"/>
-      <c r="I25" s="89">
-        <f>IF(ISBLANK($A25),"",IF(OR(ISBLANK($B25),ISBLANK($C25),ISBLANK($D25),ISBLANK($E25),ISBLANK($F25),ISBLANK($G25),ISBLANK($H25)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" ht="15" customHeight="1" s="50">
-      <c r="A26" s="90" t="n"/>
-      <c r="B26" s="90" t="n"/>
-      <c r="C26" s="90" t="n"/>
-      <c r="D26" s="90" t="n"/>
-      <c r="E26" s="90" t="n"/>
-      <c r="F26" s="90" t="n"/>
-      <c r="G26" s="90" t="n"/>
-      <c r="H26" s="90" t="n"/>
-      <c r="I26" s="89">
-        <f>IF(ISBLANK($A26),"",IF(OR(ISBLANK($B26),ISBLANK($C26),ISBLANK($D26),ISBLANK($E26),ISBLANK($F26),ISBLANK($G26),ISBLANK($H26)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" ht="15" customHeight="1" s="50">
-      <c r="A27" s="90" t="n"/>
-      <c r="B27" s="90" t="n"/>
-      <c r="C27" s="90" t="n"/>
-      <c r="D27" s="90" t="n"/>
-      <c r="E27" s="90" t="n"/>
-      <c r="F27" s="90" t="n"/>
-      <c r="G27" s="90" t="n"/>
-      <c r="H27" s="90" t="n"/>
-      <c r="I27" s="89">
-        <f>IF(ISBLANK($A27),"",IF(OR(ISBLANK($B27),ISBLANK($C27),ISBLANK($D27),ISBLANK($E27),ISBLANK($F27),ISBLANK($G27),ISBLANK($H27)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="15" customHeight="1" s="50">
-      <c r="A28" s="90" t="n"/>
-      <c r="B28" s="90" t="n"/>
-      <c r="C28" s="90" t="n"/>
-      <c r="D28" s="90" t="n"/>
-      <c r="E28" s="90" t="n"/>
-      <c r="F28" s="90" t="n"/>
-      <c r="G28" s="90" t="n"/>
-      <c r="H28" s="90" t="n"/>
-      <c r="I28" s="89">
-        <f>IF(ISBLANK($A28),"",IF(OR(ISBLANK($B28),ISBLANK($C28),ISBLANK($D28),ISBLANK($E28),ISBLANK($F28),ISBLANK($G28),ISBLANK($H28)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="15" customHeight="1" s="50">
-      <c r="A29" s="90" t="n"/>
-      <c r="B29" s="90" t="n"/>
-      <c r="C29" s="90" t="n"/>
-      <c r="D29" s="90" t="n"/>
-      <c r="E29" s="90" t="n"/>
-      <c r="F29" s="90" t="n"/>
-      <c r="G29" s="90" t="n"/>
-      <c r="H29" s="90" t="n"/>
-      <c r="I29" s="89">
-        <f>IF(ISBLANK($A29),"",IF(OR(ISBLANK($B29),ISBLANK($C29),ISBLANK($D29),ISBLANK($E29),ISBLANK($F29),ISBLANK($G29),ISBLANK($H29)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="15" customHeight="1" s="50">
-      <c r="A30" s="90" t="n"/>
-      <c r="B30" s="90" t="n"/>
-      <c r="C30" s="90" t="n"/>
-      <c r="D30" s="90" t="n"/>
-      <c r="E30" s="90" t="n"/>
-      <c r="F30" s="90" t="n"/>
-      <c r="G30" s="90" t="n"/>
-      <c r="H30" s="90" t="n"/>
-      <c r="I30" s="89">
-        <f>IF(ISBLANK($A30),"",IF(OR(ISBLANK($B30),ISBLANK($C30),ISBLANK($D30),ISBLANK($E30),ISBLANK($F30),ISBLANK($G30),ISBLANK($H30)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" ht="15" customHeight="1" s="50">
-      <c r="A31" s="90" t="n"/>
-      <c r="B31" s="90" t="n"/>
-      <c r="C31" s="90" t="n"/>
-      <c r="D31" s="90" t="n"/>
-      <c r="E31" s="90" t="n"/>
-      <c r="F31" s="90" t="n"/>
-      <c r="G31" s="90" t="n"/>
-      <c r="H31" s="90" t="n"/>
-      <c r="I31" s="89">
-        <f>IF(ISBLANK($A31),"",IF(OR(ISBLANK($B31),ISBLANK($C31),ISBLANK($D31),ISBLANK($E31),ISBLANK($F31),ISBLANK($G31),ISBLANK($H31)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="15" customHeight="1" s="50">
-      <c r="A32" s="90" t="n"/>
-      <c r="B32" s="90" t="n"/>
-      <c r="C32" s="90" t="n"/>
-      <c r="D32" s="90" t="n"/>
-      <c r="E32" s="90" t="n"/>
-      <c r="F32" s="90" t="n"/>
-      <c r="G32" s="90" t="n"/>
-      <c r="H32" s="90" t="n"/>
-      <c r="I32" s="89">
-        <f>IF(ISBLANK($A32),"",IF(OR(ISBLANK($B32),ISBLANK($C32),ISBLANK($D32),ISBLANK($E32),ISBLANK($F32),ISBLANK($G32),ISBLANK($H32)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" ht="15" customHeight="1" s="50">
-      <c r="A33" s="90" t="n"/>
-      <c r="B33" s="90" t="n"/>
-      <c r="C33" s="90" t="n"/>
-      <c r="D33" s="90" t="n"/>
-      <c r="E33" s="90" t="n"/>
-      <c r="F33" s="90" t="n"/>
-      <c r="G33" s="90" t="n"/>
-      <c r="H33" s="90" t="n"/>
-      <c r="I33" s="89">
-        <f>IF(ISBLANK($A33),"",IF(OR(ISBLANK($B33),ISBLANK($C33),ISBLANK($D33),ISBLANK($E33),ISBLANK($F33),ISBLANK($G33),ISBLANK($H33)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" ht="15" customHeight="1" s="50">
-      <c r="A34" s="90" t="n"/>
-      <c r="B34" s="90" t="n"/>
-      <c r="C34" s="90" t="n"/>
-      <c r="D34" s="90" t="n"/>
-      <c r="E34" s="90" t="n"/>
-      <c r="F34" s="90" t="n"/>
-      <c r="G34" s="90" t="n"/>
-      <c r="H34" s="90" t="n"/>
-      <c r="I34" s="89">
-        <f>IF(ISBLANK($A34),"",IF(OR(ISBLANK($B34),ISBLANK($C34),ISBLANK($D34),ISBLANK($E34),ISBLANK($F34),ISBLANK($G34),ISBLANK($H34)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" ht="15" customHeight="1" s="50">
-      <c r="A35" s="90" t="n"/>
-      <c r="B35" s="90" t="n"/>
-      <c r="C35" s="90" t="n"/>
-      <c r="D35" s="90" t="n"/>
-      <c r="E35" s="90" t="n"/>
-      <c r="F35" s="90" t="n"/>
-      <c r="G35" s="90" t="n"/>
-      <c r="H35" s="90" t="n"/>
-      <c r="I35" s="89">
-        <f>IF(ISBLANK($A35),"",IF(OR(ISBLANK($B35),ISBLANK($C35),ISBLANK($D35),ISBLANK($E35),ISBLANK($F35),ISBLANK($G35),ISBLANK($H35)),"EKSİK","OK"))</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AN1"/>
-  </mergeCells>
-  <conditionalFormatting sqref="G6:G1000">
-    <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="lessThan" aboveAverage="0" dxfId="9" text="" percent="0" bottom="0">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D6:D1000">
-    <cfRule type="cellIs" rank="0" priority="3" equalAverage="0" operator="equal" aboveAverage="0" dxfId="10" text="" percent="0" bottom="0">
-      <formula>"Komisyon"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I6:I1000">
-    <cfRule type="cellIs" rank="0" priority="4" equalAverage="0" operator="equal" aboveAverage="0" dxfId="9" text="" percent="0" bottom="0">
-      <formula>"EKSİK"</formula>
-    </cfRule>
-    <cfRule type="cellIs" rank="0" priority="5" equalAverage="0" operator="equal" aboveAverage="0" dxfId="8" text="" percent="0" bottom="0">
-      <formula>"OK"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation sqref="D6:D1000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz Tür" error="Lütfen listeden bir masraf türü seçin." promptTitle="Masraf Türü" prompt="Tahsis Ücreti, Sigorta, Komisyon veya Diğer seçin." type="list" errorStyle="stop" operator="between">
-      <formula1>ListeMasrafTuru</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation sqref="B6:B1000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Geçersiz Kredi" error="Lütfen KREDILER sayfasındaki bir kredi ID seçin." promptTitle="Kredi ID" prompt="Listeden kredi seçin." type="list" errorStyle="stop" operator="between">
-      <formula1>ListeKrediId</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-  </dataValidations>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(typography): eliminate all subtitle text wraps across all sheets with full-span merging and add Mandate Rule 251
</commit_message>
<xml_diff>
--- a/EXCELARSIV_PRODUCTS/banka-kredi-ve-taksit-takip-sistemi/BankaKrediVeTaksitTakipSistemi.xlsx
+++ b/EXCELARSIV_PRODUCTS/banka-kredi-ve-taksit-takip-sistemi/BankaKrediVeTaksitTakipSistemi.xlsx
@@ -119,7 +119,7 @@
     <numFmt numFmtId="169" formatCode="₺#,##0"/>
     <numFmt numFmtId="170" formatCode="0.00&quot;x&quot;"/>
   </numFmts>
-  <fonts count="126">
+  <fonts count="128">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -882,6 +882,18 @@
       <color rgb="002563EB"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Montserrat"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00475569"/>
+      <sz val="9.5"/>
+    </font>
   </fonts>
   <fills count="38">
     <fill>
@@ -1094,7 +1106,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="63">
+  <borders count="64">
     <border>
       <left/>
       <right/>
@@ -1746,6 +1758,18 @@
         <color rgb="00E2E8F0"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -1757,7 +1781,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="427">
+  <cellXfs count="441">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2825,6 +2849,46 @@
     </xf>
     <xf numFmtId="0" fontId="75" fillId="0" borderId="58" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="113" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="114" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="119" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="120" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="97" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="95" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="126" fillId="36" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="127" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="70" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="72" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="73" fillId="20" borderId="63" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="11" borderId="63" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -13460,14 +13524,14 @@
     </row>
     <row r="3" ht="7.8" customHeight="1" s="50"/>
     <row r="4" ht="17.4" customHeight="1" s="50">
-      <c r="B4" s="353" t="inlineStr">
+      <c r="B4" s="427" t="inlineStr">
         <is>
           <t>Banka, Kredi ve Taksit Takip Sistemi — C-Level Borç Portföyü ve Likidite Karar Kokpiti</t>
         </is>
       </c>
     </row>
     <row r="5" ht="17.4" customHeight="1" s="50">
-      <c r="B5" s="354" t="inlineStr">
+      <c r="B5" s="428" t="inlineStr">
         <is>
           <t>Hedef Kitle: KOBİ Sahipleri, CFO, Finans Direktörleri ve Hazine Yöneticileri · VUK 185-198 &amp; TTK 64 Tam Uyumlu</t>
         </is>
@@ -13894,9 +13958,10 @@
       <c r="R26" s="337" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="24">
     <mergeCell ref="N26:O26"/>
     <mergeCell ref="B2:M2"/>
+    <mergeCell ref="B4:R4"/>
     <mergeCell ref="N25:O25"/>
     <mergeCell ref="D25:M25"/>
     <mergeCell ref="P23:R23"/>
@@ -13917,6 +13982,7 @@
     <mergeCell ref="P25:R25"/>
     <mergeCell ref="N24:O24"/>
     <mergeCell ref="P22:R22"/>
+    <mergeCell ref="B5:R5"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId1"/>
@@ -13952,20 +14018,30 @@
     <col width="10" customWidth="1" style="76" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="50">
-      <c r="A1" s="77" t="inlineStr">
+    <row r="1" ht="32" customHeight="1" s="50">
+      <c r="A1" s="433" t="inlineStr">
         <is>
           <t>MASRAF KOMISYON — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="150" customHeight="1" s="50">
-      <c r="A3" s="85" t="inlineStr">
+      <c r="B1" s="434" t="n"/>
+      <c r="C1" s="434" t="n"/>
+      <c r="D1" s="434" t="n"/>
+      <c r="E1" s="434" t="n"/>
+      <c r="F1" s="434" t="n"/>
+      <c r="G1" s="434" t="n"/>
+      <c r="H1" s="434" t="n"/>
+      <c r="I1" s="434" t="n"/>
+    </row>
+    <row r="2" ht="7.8" customHeight="1" s="50"/>
+    <row r="3" ht="22" customHeight="1" s="50">
+      <c r="A3" s="435" t="inlineStr">
         <is>
           <t>MASRAF VE KOMİSYONLAR — tahsis, sigorta, komisyon ve diğer finansman maliyetleri.</t>
         </is>
       </c>
     </row>
+    <row r="4" ht="10" customHeight="1" s="50"/>
     <row r="5" ht="30" customHeight="1" s="50">
       <c r="A5" s="86" t="inlineStr">
         <is>
@@ -14519,8 +14595,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AN1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
   </mergeCells>
   <conditionalFormatting sqref="G6:G1000">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="lessThan" aboveAverage="0" dxfId="9" text="" percent="0" bottom="0">
@@ -14582,20 +14659,31 @@
     <col width="10" customWidth="1" style="76" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="50">
-      <c r="A1" s="77" t="inlineStr">
+    <row r="1" ht="32" customHeight="1" s="50">
+      <c r="A1" s="433" t="inlineStr">
         <is>
           <t>TEMINATLAR — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="90.75" customHeight="1" s="50">
-      <c r="A3" s="85" t="inlineStr">
+      <c r="B1" s="434" t="n"/>
+      <c r="C1" s="434" t="n"/>
+      <c r="D1" s="434" t="n"/>
+      <c r="E1" s="434" t="n"/>
+      <c r="F1" s="434" t="n"/>
+      <c r="G1" s="434" t="n"/>
+      <c r="H1" s="434" t="n"/>
+      <c r="I1" s="434" t="n"/>
+      <c r="J1" s="434" t="n"/>
+    </row>
+    <row r="2" ht="7.8" customHeight="1" s="50"/>
+    <row r="3" ht="22" customHeight="1" s="50">
+      <c r="A3" s="435" t="inlineStr">
         <is>
           <t>TEMİNAT YÖNETİMİ — değer, geçerlilik ve kredi bağlantısı.</t>
         </is>
       </c>
     </row>
+    <row r="4" ht="10" customHeight="1" s="50"/>
     <row r="5" ht="30" customHeight="1" s="50">
       <c r="A5" s="86" t="inlineStr">
         <is>
@@ -15190,8 +15278,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AN1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A3:J3"/>
   </mergeCells>
   <conditionalFormatting sqref="F6:F1000">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="lessThan" aboveAverage="0" dxfId="9" text="" percent="0" bottom="0">
@@ -15253,20 +15342,32 @@
     <col width="10" customWidth="1" style="76" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="50">
-      <c r="A1" s="77" t="inlineStr">
+    <row r="1" ht="32" customHeight="1" s="50">
+      <c r="A1" s="433" t="inlineStr">
         <is>
           <t>YENI TEKLIFLER — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="135.75" customHeight="1" s="50">
-      <c r="A3" s="85" t="inlineStr">
+      <c r="B1" s="434" t="n"/>
+      <c r="C1" s="434" t="n"/>
+      <c r="D1" s="434" t="n"/>
+      <c r="E1" s="434" t="n"/>
+      <c r="F1" s="434" t="n"/>
+      <c r="G1" s="434" t="n"/>
+      <c r="H1" s="434" t="n"/>
+      <c r="I1" s="434" t="n"/>
+      <c r="J1" s="434" t="n"/>
+      <c r="K1" s="434" t="n"/>
+    </row>
+    <row r="2" ht="7.8" customHeight="1" s="50"/>
+    <row r="3" ht="22" customHeight="1" s="50">
+      <c r="A3" s="435" t="inlineStr">
         <is>
           <t>YENİ KREDİ TEKLİFLERİ — tutar, faiz, masraf ve aylık taksit karşılaştırması.</t>
         </is>
       </c>
     </row>
+    <row r="4" ht="10" customHeight="1" s="50"/>
     <row r="5" ht="30" customHeight="1" s="50">
       <c r="A5" s="86" t="inlineStr">
         <is>
@@ -16058,8 +16159,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AN1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A3:K3"/>
   </mergeCells>
   <conditionalFormatting sqref="G6:G1000">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="greaterThan" aboveAverage="0" dxfId="10" text="" percent="0" bottom="0">
@@ -16117,16 +16219,25 @@
     <col width="14" customWidth="1" style="76" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" s="50">
-      <c r="A1" s="305" t="inlineStr">
+    <row r="1" ht="32" customHeight="1" s="50">
+      <c r="A1" s="433" t="inlineStr">
         <is>
           <t>REFINANSMAN — KURUMSAL BANKA VE BORÇ YÖNETİMİ</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="6" customHeight="1" s="50"/>
-    <row r="3" ht="20" customHeight="1" s="50">
-      <c r="A3" s="306" t="inlineStr">
+      <c r="B1" s="434" t="n"/>
+      <c r="C1" s="434" t="n"/>
+      <c r="D1" s="434" t="n"/>
+      <c r="E1" s="434" t="n"/>
+      <c r="F1" s="434" t="n"/>
+      <c r="G1" s="434" t="n"/>
+      <c r="H1" s="434" t="n"/>
+      <c r="I1" s="434" t="n"/>
+      <c r="J1" s="434" t="n"/>
+    </row>
+    <row r="2" ht="7.8" customHeight="1" s="50"/>
+    <row r="3" ht="22" customHeight="1" s="50">
+      <c r="A3" s="435" t="inlineStr">
         <is>
           <t>REFİNANSMAN ANALİZİ — aylık taksit rahatlaması ve toplam maliyet.</t>
         </is>
@@ -17447,8 +17558,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AN1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A3:J3"/>
   </mergeCells>
   <conditionalFormatting sqref="F6:F1000">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="lessThanOrEqual" aboveAverage="0" dxfId="10" text="" percent="0" bottom="0">
@@ -17509,21 +17621,21 @@
       </c>
     </row>
     <row r="2" ht="34" customHeight="1" s="50">
-      <c r="B2" s="188" t="inlineStr">
+      <c r="B2" s="436" t="inlineStr">
         <is>
           <t>BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ — FİNANSAL STRES TESTİ</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1" s="50">
-      <c r="B3" s="189" t="inlineStr">
+      <c r="B3" s="437" t="inlineStr">
         <is>
           <t>Yönetim Kurulu ve Hazine Komitesi için Borç Servisi ve Likidite Dayanıklılık Raporu</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" s="50">
-      <c r="B4" s="190" t="inlineStr">
+      <c r="B4" s="438" t="inlineStr">
         <is>
           <t>DÖNEM: 2026 Q3 · DENETİM PROTOKOLÜ: ISO/VUK/IFRS UYUMLU · DURUM: ONAYLANDI</t>
         </is>
@@ -17531,24 +17643,24 @@
     </row>
     <row r="5" ht="14" customHeight="1" s="50"/>
     <row r="6" ht="28" customHeight="1" s="50">
-      <c r="B6" s="415" t="inlineStr">
+      <c r="B6" s="439" t="inlineStr">
         <is>
           <t>SENARYO A: KÖTÜMSER (STRES TESTİ -%20)</t>
         </is>
       </c>
-      <c r="C6" s="399" t="n"/>
-      <c r="D6" s="399" t="n"/>
-      <c r="E6" s="399" t="n"/>
-      <c r="F6" s="416" t="n"/>
-      <c r="H6" s="417" t="inlineStr">
+      <c r="C6" s="290" t="n"/>
+      <c r="D6" s="290" t="n"/>
+      <c r="E6" s="290" t="n"/>
+      <c r="F6" s="291" t="n"/>
+      <c r="H6" s="440" t="inlineStr">
         <is>
           <t>SENARYO B: BAZ MODEL (HEDEFLENEN)</t>
         </is>
       </c>
-      <c r="I6" s="399" t="n"/>
-      <c r="J6" s="399" t="n"/>
-      <c r="K6" s="399" t="n"/>
-      <c r="L6" s="416" t="n"/>
+      <c r="I6" s="290" t="n"/>
+      <c r="J6" s="290" t="n"/>
+      <c r="K6" s="290" t="n"/>
+      <c r="L6" s="291" t="n"/>
     </row>
     <row r="7" ht="8" customHeight="1" s="50">
       <c r="B7" s="418" t="n"/>
@@ -17788,11 +17900,14 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="7">
+    <mergeCell ref="B4:L4"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="H6:L6"/>
+    <mergeCell ref="B3:L3"/>
+    <mergeCell ref="B2:L2"/>
+    <mergeCell ref="H14:L15"/>
     <mergeCell ref="B14:F15"/>
-    <mergeCell ref="H6:L6"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="H14:L15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -18000,20 +18115,30 @@
     <col width="26" customWidth="1" style="76" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="50">
-      <c r="A1" s="77" t="inlineStr">
+    <row r="1" ht="32" customHeight="1" s="50">
+      <c r="A1" s="433" t="inlineStr">
         <is>
           <t>KARAR MOTORU — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="52.5" customHeight="1" s="50">
-      <c r="A3" s="110" t="inlineStr">
+      <c r="B1" s="434" t="n"/>
+      <c r="C1" s="434" t="n"/>
+      <c r="D1" s="434" t="n"/>
+      <c r="E1" s="434" t="n"/>
+      <c r="F1" s="434" t="n"/>
+      <c r="G1" s="434" t="n"/>
+      <c r="H1" s="434" t="n"/>
+      <c r="I1" s="434" t="n"/>
+    </row>
+    <row r="2" ht="7.8" customHeight="1" s="50"/>
+    <row r="3" ht="22" customHeight="1" s="50">
+      <c r="A3" s="435" t="inlineStr">
         <is>
           <t>KARAR MOTORU — borç yükü, yaklaşan taksit ve öncelikli aksiyon</t>
         </is>
       </c>
     </row>
+    <row r="4" ht="10" customHeight="1" s="50"/>
     <row r="5" ht="15" customHeight="1" s="50">
       <c r="A5" s="81" t="inlineStr">
         <is>
@@ -18188,8 +18313,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AN1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
   </mergeCells>
   <conditionalFormatting sqref="B14">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="equal" aboveAverage="0" dxfId="8" text="" percent="0" bottom="0">
@@ -18831,20 +18957,30 @@
     <col width="20" customWidth="1" style="76" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="50">
-      <c r="A1" s="77" t="inlineStr">
+    <row r="1" ht="32" customHeight="1" s="50">
+      <c r="A1" s="433" t="inlineStr">
         <is>
           <t>SENARYO DUYARLILIK — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="50">
-      <c r="A3" s="99" t="inlineStr">
+      <c r="B1" s="434" t="n"/>
+      <c r="C1" s="434" t="n"/>
+      <c r="D1" s="434" t="n"/>
+      <c r="E1" s="434" t="n"/>
+      <c r="F1" s="434" t="n"/>
+      <c r="G1" s="434" t="n"/>
+      <c r="H1" s="434" t="n"/>
+      <c r="I1" s="434" t="n"/>
+    </row>
+    <row r="2" ht="7.8" customHeight="1" s="50"/>
+    <row r="3" ht="22" customHeight="1" s="50">
+      <c r="A3" s="435" t="inlineStr">
         <is>
           <t>SENARYO VE DUYARLILIK ANALİZİ</t>
         </is>
       </c>
     </row>
+    <row r="4" ht="10" customHeight="1" s="50"/>
     <row r="5" ht="15" customHeight="1" s="50">
       <c r="A5" s="81" t="inlineStr">
         <is>
@@ -19049,8 +19185,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AN1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
   </mergeCells>
   <conditionalFormatting sqref="B5">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="lessThan" aboveAverage="0" dxfId="12" text="" percent="0" bottom="0">
@@ -19097,20 +19234,32 @@
     <col width="24" customWidth="1" style="76" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="50">
-      <c r="A1" s="77" t="inlineStr">
+    <row r="1" ht="32" customHeight="1" s="50">
+      <c r="A1" s="433" t="inlineStr">
         <is>
           <t>KONTROLLER — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="50">
-      <c r="A3" s="99" t="inlineStr">
+      <c r="B1" s="434" t="n"/>
+      <c r="C1" s="434" t="n"/>
+      <c r="D1" s="434" t="n"/>
+      <c r="E1" s="434" t="n"/>
+      <c r="F1" s="434" t="n"/>
+      <c r="G1" s="434" t="n"/>
+      <c r="H1" s="434" t="n"/>
+      <c r="I1" s="434" t="n"/>
+      <c r="J1" s="434" t="n"/>
+    </row>
+    <row r="2" ht="7.8" customHeight="1" s="50"/>
+    <row r="3" ht="22" customHeight="1" s="50">
+      <c r="A3" s="435" t="inlineStr">
         <is>
           <t>VERİ KALİTESİ VE SİSTEM SAĞLIĞI</t>
         </is>
       </c>
     </row>
+    <row r="4" ht="10" customHeight="1" s="50"/>
+    <row r="5"/>
     <row r="6" ht="15" customHeight="1" s="50">
       <c r="A6" s="100" t="inlineStr">
         <is>
@@ -19219,8 +19368,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AN1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A3:J3"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="lessThan" aboveAverage="0" dxfId="12" text="" percent="0" bottom="0">
@@ -19281,14 +19431,14 @@
   </cols>
   <sheetData>
     <row r="2" ht="36" customHeight="1" s="50">
-      <c r="B2" s="371" t="inlineStr">
+      <c r="B2" s="429" t="inlineStr">
         <is>
           <t>SİSTEM HAKKINDA, KULLANIM REHBERİ VE TERİMLER SÖZLÜĞÜ</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" s="50">
-      <c r="B3" s="372" t="inlineStr">
+      <c r="B3" s="430" t="inlineStr">
         <is>
           <t>5 Yaşındaki Birine Anlatır Gibi Basit, Sade ve Eksiksiz Finansal Karar Mimarisi · Siemens &amp; Enterprise Standartları</t>
         </is>
@@ -19720,6 +19870,10 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B3:F3"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19747,21 +19901,30 @@
     <col width="13" customWidth="1" style="76" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="50">
-      <c r="A1" s="77" t="inlineStr">
+    <row r="1" ht="32" customHeight="1" s="50">
+      <c r="A1" s="433" t="inlineStr">
         <is>
           <t>AYARLAR — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="19.5" customHeight="1" s="50">
+      <c r="B1" s="434" t="n"/>
+      <c r="C1" s="434" t="n"/>
+      <c r="D1" s="434" t="n"/>
+      <c r="E1" s="434" t="n"/>
+      <c r="F1" s="434" t="n"/>
+      <c r="G1" s="434" t="n"/>
+      <c r="H1" s="434" t="n"/>
+      <c r="I1" s="434" t="n"/>
+    </row>
+    <row r="2" ht="7.8" customHeight="1" s="50">
       <c r="A2" s="103" t="inlineStr">
         <is>
           <t>Tüm eşikler, katsayılar ve firma bilgileri tek kaynaktan (SSOT) buradan yönetilir. Değerleri değiştirirken Alt/Üst sınırlara dikkat edin.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="50">
+    <row r="3"/>
+    <row r="4" ht="10" customHeight="1" s="50">
       <c r="A4" s="104" t="inlineStr">
         <is>
           <t>FIRMA BİLGİLERİ</t>
@@ -20715,7 +20878,7 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:AN2"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -20750,20 +20913,34 @@
     <col width="14" customWidth="1" style="76" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="50">
-      <c r="A1" s="77" t="inlineStr">
+    <row r="1" ht="32" customHeight="1" s="50">
+      <c r="A1" s="433" t="inlineStr">
         <is>
           <t>LISTELER — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="50">
-      <c r="A3" s="99" t="inlineStr">
+      <c r="B1" s="434" t="n"/>
+      <c r="C1" s="434" t="n"/>
+      <c r="D1" s="434" t="n"/>
+      <c r="E1" s="434" t="n"/>
+      <c r="F1" s="434" t="n"/>
+      <c r="G1" s="434" t="n"/>
+      <c r="H1" s="434" t="n"/>
+      <c r="I1" s="434" t="n"/>
+      <c r="J1" s="434" t="n"/>
+      <c r="K1" s="434" t="n"/>
+      <c r="L1" s="434" t="n"/>
+      <c r="M1" s="434" t="n"/>
+    </row>
+    <row r="2" ht="7.8" customHeight="1" s="50"/>
+    <row r="3" ht="22" customHeight="1" s="50">
+      <c r="A3" s="435" t="inlineStr">
         <is>
           <t>AÇILIR LİSTE KAYNAKLARI</t>
         </is>
       </c>
     </row>
+    <row r="4" ht="10" customHeight="1" s="50"/>
     <row r="5" ht="15" customHeight="1" s="50">
       <c r="A5" s="84" t="inlineStr">
         <is>
@@ -20950,8 +21127,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AN1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -24617,24 +24795,14 @@
       </c>
     </row>
     <row r="2" ht="36" customHeight="1" s="50">
-      <c r="B2" s="242" t="inlineStr">
+      <c r="B2" s="431" t="inlineStr">
         <is>
           <t>BANKA, KREDİ VE TAKSİT YÖNETİM MERKEZİ</t>
         </is>
       </c>
-      <c r="L2" s="125" t="inlineStr">
-        <is>
-          <t>Dönem: 2026 / Tam ▼</t>
-        </is>
-      </c>
-      <c r="M2" s="126" t="inlineStr">
-        <is>
-          <t>★ DOĞRULANMIŞ</t>
-        </is>
-      </c>
     </row>
     <row r="3" ht="18" customHeight="1" s="50">
-      <c r="B3" s="237" t="inlineStr">
+      <c r="B3" s="432" t="inlineStr">
         <is>
           <t>Konsolide Kredi Portföyü, Aylık Borç Servisi ve Likidite Karar Kokpiti · Canlı Hesaplama</t>
         </is>
@@ -25158,10 +25326,12 @@
       <c r="I27" s="251" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="K26:M27"/>
+  <mergeCells count="5">
+    <mergeCell ref="B2:M2"/>
     <mergeCell ref="K24:M25"/>
     <mergeCell ref="F26:I27"/>
+    <mergeCell ref="B3:M3"/>
+    <mergeCell ref="K26:M27"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId1"/>
@@ -25184,20 +25354,30 @@
     <col width="42" customWidth="1" style="76" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="50">
-      <c r="A1" s="77" t="inlineStr">
+    <row r="1" ht="32" customHeight="1" s="50">
+      <c r="A1" s="433" t="inlineStr">
         <is>
           <t>ORNEK VERI — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="45.75" customHeight="1" s="50">
-      <c r="A3" s="85" t="inlineStr">
+      <c r="B1" s="434" t="n"/>
+      <c r="C1" s="434" t="n"/>
+      <c r="D1" s="434" t="n"/>
+      <c r="E1" s="434" t="n"/>
+      <c r="F1" s="434" t="n"/>
+      <c r="G1" s="434" t="n"/>
+      <c r="H1" s="434" t="n"/>
+      <c r="I1" s="434" t="n"/>
+    </row>
+    <row r="2" ht="7.8" customHeight="1" s="50"/>
+    <row r="3" ht="22" customHeight="1" s="50">
+      <c r="A3" s="435" t="inlineStr">
         <is>
           <t>ÖRNEK VERİ — otomasyon ve içe aktarma için yapı</t>
         </is>
       </c>
     </row>
+    <row r="4" ht="10" customHeight="1" s="50"/>
     <row r="5" ht="30" customHeight="1" s="50">
       <c r="A5" s="86" t="inlineStr">
         <is>
@@ -25319,8 +25499,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AN1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -25342,20 +25523,30 @@
     <col width="18" customWidth="1" style="76" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="50">
-      <c r="A1" s="77" t="inlineStr">
+    <row r="1" ht="32" customHeight="1" s="50">
+      <c r="A1" s="433" t="inlineStr">
         <is>
           <t>TESTLER — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="50">
-      <c r="A3" s="99" t="inlineStr">
+      <c r="B1" s="434" t="n"/>
+      <c r="C1" s="434" t="n"/>
+      <c r="D1" s="434" t="n"/>
+      <c r="E1" s="434" t="n"/>
+      <c r="F1" s="434" t="n"/>
+      <c r="G1" s="434" t="n"/>
+      <c r="H1" s="434" t="n"/>
+      <c r="I1" s="434" t="n"/>
+    </row>
+    <row r="2" ht="7.8" customHeight="1" s="50"/>
+    <row r="3" ht="22" customHeight="1" s="50">
+      <c r="A3" s="435" t="inlineStr">
         <is>
           <t>SİSTEM TESTLERİ VE DENETİM KAYDI</t>
         </is>
       </c>
     </row>
+    <row r="4" ht="10" customHeight="1" s="50"/>
     <row r="5" ht="30" customHeight="1" s="50">
       <c r="A5" s="86" t="inlineStr">
         <is>
@@ -25487,8 +25678,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AN1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -25735,20 +25927,30 @@
     <col width="90" customWidth="1" style="76" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="50">
-      <c r="A1" s="77" t="inlineStr">
+    <row r="1" ht="32" customHeight="1" s="50">
+      <c r="A1" s="433" t="inlineStr">
         <is>
           <t>DEGISIKLIK KAYDI — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="50">
-      <c r="A3" s="99" t="inlineStr">
+      <c r="B1" s="434" t="n"/>
+      <c r="C1" s="434" t="n"/>
+      <c r="D1" s="434" t="n"/>
+      <c r="E1" s="434" t="n"/>
+      <c r="F1" s="434" t="n"/>
+      <c r="G1" s="434" t="n"/>
+      <c r="H1" s="434" t="n"/>
+      <c r="I1" s="434" t="n"/>
+    </row>
+    <row r="2" ht="7.8" customHeight="1" s="50"/>
+    <row r="3" ht="22" customHeight="1" s="50">
+      <c r="A3" s="435" t="inlineStr">
         <is>
           <t>DEĞİŞİKLİK KAYDI</t>
         </is>
       </c>
     </row>
+    <row r="4" ht="10" customHeight="1" s="50"/>
     <row r="5" ht="30" customHeight="1" s="50">
       <c r="A5" s="86" t="inlineStr">
         <is>
@@ -25785,8 +25987,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AN1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -26297,16 +26500,24 @@
     <col width="14" customWidth="1" style="76" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" s="50">
-      <c r="A1" s="305" t="inlineStr">
+    <row r="1" ht="32" customHeight="1" s="50">
+      <c r="A1" s="433" t="inlineStr">
         <is>
           <t>BANKALAR — KURUMSAL BANKA VE BORÇ YÖNETİMİ</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="6" customHeight="1" s="50"/>
-    <row r="3" ht="20" customHeight="1" s="50">
-      <c r="A3" s="306" t="inlineStr">
+      <c r="B1" s="434" t="n"/>
+      <c r="C1" s="434" t="n"/>
+      <c r="D1" s="434" t="n"/>
+      <c r="E1" s="434" t="n"/>
+      <c r="F1" s="434" t="n"/>
+      <c r="G1" s="434" t="n"/>
+      <c r="H1" s="434" t="n"/>
+      <c r="I1" s="434" t="n"/>
+    </row>
+    <row r="2" ht="7.8" customHeight="1" s="50"/>
+    <row r="3" ht="22" customHeight="1" s="50">
+      <c r="A3" s="435" t="inlineStr">
         <is>
           <t>BANKA TANIMLARI — ilişki, operasyonel durum ve iletişim tek merkezde.</t>
         </is>
@@ -26902,8 +27113,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AN1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
   </mergeCells>
   <conditionalFormatting sqref="F6:F1000">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="equal" aboveAverage="0" dxfId="8" text="" percent="0" bottom="0">
@@ -26961,16 +27173,24 @@
     <col width="14" customWidth="1" style="76" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" s="50">
-      <c r="A1" s="305" t="inlineStr">
+    <row r="1" ht="32" customHeight="1" s="50">
+      <c r="A1" s="433" t="inlineStr">
         <is>
           <t>LIMITLER — KURUMSAL BANKA VE BORÇ YÖNETİMİ</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="6" customHeight="1" s="50"/>
-    <row r="3" ht="20" customHeight="1" s="50">
-      <c r="A3" s="306" t="inlineStr">
+      <c r="B1" s="434" t="n"/>
+      <c r="C1" s="434" t="n"/>
+      <c r="D1" s="434" t="n"/>
+      <c r="E1" s="434" t="n"/>
+      <c r="F1" s="434" t="n"/>
+      <c r="G1" s="434" t="n"/>
+      <c r="H1" s="434" t="n"/>
+      <c r="I1" s="434" t="n"/>
+    </row>
+    <row r="2" ht="7.8" customHeight="1" s="50"/>
+    <row r="3" ht="22" customHeight="1" s="50">
+      <c r="A3" s="435" t="inlineStr">
         <is>
           <t>BANKA LİMİTLERİ — toplam, kullanılan ve kalan limit ile kullanım oranı.</t>
         </is>
@@ -27706,8 +27926,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AN1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
   </mergeCells>
   <conditionalFormatting sqref="H6:H1000">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="lessThan" aboveAverage="0" dxfId="9" text="" percent="0" bottom="0">
@@ -27780,16 +28001,29 @@
     <col width="14" customWidth="1" style="76" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" s="50">
-      <c r="A1" s="305" t="inlineStr">
+    <row r="1" ht="32" customHeight="1" s="50">
+      <c r="A1" s="433" t="inlineStr">
         <is>
           <t>KREDILER — KURUMSAL BANKA VE BORÇ YÖNETİMİ</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="6" customHeight="1" s="50"/>
-    <row r="3" ht="20" customHeight="1" s="50">
-      <c r="A3" s="306" t="inlineStr">
+      <c r="B1" s="434" t="n"/>
+      <c r="C1" s="434" t="n"/>
+      <c r="D1" s="434" t="n"/>
+      <c r="E1" s="434" t="n"/>
+      <c r="F1" s="434" t="n"/>
+      <c r="G1" s="434" t="n"/>
+      <c r="H1" s="434" t="n"/>
+      <c r="I1" s="434" t="n"/>
+      <c r="J1" s="434" t="n"/>
+      <c r="K1" s="434" t="n"/>
+      <c r="L1" s="434" t="n"/>
+      <c r="M1" s="434" t="n"/>
+      <c r="N1" s="434" t="n"/>
+    </row>
+    <row r="2" ht="7.8" customHeight="1" s="50"/>
+    <row r="3" ht="22" customHeight="1" s="50">
+      <c r="A3" s="435" t="inlineStr">
         <is>
           <t>KREDİ PORTFÖYÜ — sözleşme, bakiye, maliyet, vade ve taksit bilgileri.</t>
         </is>
@@ -28756,8 +28990,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AN1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A3:N3"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <conditionalFormatting sqref="H6:H1000">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="lessThanOrEqual" aboveAverage="0" dxfId="12" text="" percent="0" bottom="0">
@@ -28828,16 +29063,27 @@
     <col width="14" customWidth="1" style="76" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" s="50">
-      <c r="A1" s="305" t="inlineStr">
+    <row r="1" ht="32" customHeight="1" s="50">
+      <c r="A1" s="433" t="inlineStr">
         <is>
           <t>TAKSIT_PLANI — KURUMSAL BANKA VE BORÇ YÖNETİMİ</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="6" customHeight="1" s="50"/>
-    <row r="3" ht="20" customHeight="1" s="50">
-      <c r="A3" s="306" t="inlineStr">
+      <c r="B1" s="434" t="n"/>
+      <c r="C1" s="434" t="n"/>
+      <c r="D1" s="434" t="n"/>
+      <c r="E1" s="434" t="n"/>
+      <c r="F1" s="434" t="n"/>
+      <c r="G1" s="434" t="n"/>
+      <c r="H1" s="434" t="n"/>
+      <c r="I1" s="434" t="n"/>
+      <c r="J1" s="434" t="n"/>
+      <c r="K1" s="434" t="n"/>
+      <c r="L1" s="434" t="n"/>
+    </row>
+    <row r="2" ht="7.8" customHeight="1" s="50"/>
+    <row r="3" ht="22" customHeight="1" s="50">
+      <c r="A3" s="435" t="inlineStr">
         <is>
           <t>TAKSİT PLANI — dönem bazında anapara, faiz, vergi ve ödeme tarihi.</t>
         </is>
@@ -29742,8 +29988,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AN1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <conditionalFormatting sqref="I6:I1000">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="lessThanOrEqual" aboveAverage="0" dxfId="9" text="" percent="0" bottom="0">
@@ -29820,16 +30067,24 @@
     <col width="15" customWidth="1" style="76" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" s="50">
-      <c r="A1" s="305" t="inlineStr">
+    <row r="1" ht="32" customHeight="1" s="50">
+      <c r="A1" s="433" t="inlineStr">
         <is>
           <t>ODEME_TAKVIMI — KURUMSAL BANKA VE BORÇ YÖNETİMİ</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="6" customHeight="1" s="50"/>
-    <row r="3" ht="20" customHeight="1" s="50">
-      <c r="A3" s="306" t="inlineStr">
+      <c r="B1" s="434" t="n"/>
+      <c r="C1" s="434" t="n"/>
+      <c r="D1" s="434" t="n"/>
+      <c r="E1" s="434" t="n"/>
+      <c r="F1" s="434" t="n"/>
+      <c r="G1" s="434" t="n"/>
+      <c r="H1" s="434" t="n"/>
+      <c r="I1" s="434" t="n"/>
+    </row>
+    <row r="2" ht="7.8" customHeight="1" s="50"/>
+    <row r="3" ht="22" customHeight="1" s="50">
+      <c r="A3" s="435" t="inlineStr">
         <is>
           <t>ÖDEME TAKVİMİ — yaklaşan taksitler 30 / 60 / 90 gün penceresinde.</t>
         </is>
@@ -30775,8 +31030,9 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:AN1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
   </mergeCells>
   <conditionalFormatting sqref="D6:D1000">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="lessThan" aboveAverage="0" dxfId="9" text="" percent="0" bottom="0">

</xml_diff>

<commit_message>
feat(dashboard): integrate ,000 executive showcase charts (Doughnut & Bar) into PANO and mandate protocol Rule 252
</commit_message>
<xml_diff>
--- a/EXCELARSIV_PRODUCTS/banka-kredi-ve-taksit-takip-sistemi/BankaKrediVeTaksitTakipSistemi.xlsx
+++ b/EXCELARSIV_PRODUCTS/banka-kredi-ve-taksit-takip-sistemi/BankaKrediVeTaksitTakipSistemi.xlsx
@@ -3135,6 +3135,226 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>DÖNEMSEL BORÇ HACMİ VE MALİYET TRENDİ</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'PANO'!C14</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'PANO'!$B$15:$B$20</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'PANO'!$C$15:$C$20</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'PANO'!D14</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'PANO'!$B$15:$B$20</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'PANO'!$D$15:$D$20</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'PANO'!E14</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'PANO'!$B$15:$B$20</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'PANO'!$E$15:$E$20</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Dönemler</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Endeks / Milyon TL</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>BORÇ DAĞILIMI VE RİSK YOĞUNLAŞMASI</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <doughnutChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'PANO'!I14</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'PANO'!$H$15:$H$18</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'PANO'!$I$15:$I$18</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+        <holeSize val="60"/>
+      </doughnutChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
@@ -3413,7 +3633,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -13074,6 +13294,55 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5940000" cy="3420000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5220000" cy="3420000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor editAs="oneCell">
     <from>
@@ -14005,7 +14274,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AN35"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="76" min="1" max="2"/>
@@ -14024,14 +14293,6 @@
           <t>MASRAF KOMISYON — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-      <c r="B1" s="434" t="n"/>
-      <c r="C1" s="434" t="n"/>
-      <c r="D1" s="434" t="n"/>
-      <c r="E1" s="434" t="n"/>
-      <c r="F1" s="434" t="n"/>
-      <c r="G1" s="434" t="n"/>
-      <c r="H1" s="434" t="n"/>
-      <c r="I1" s="434" t="n"/>
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
@@ -14644,7 +14905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AN35"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="76" min="1" max="1"/>
@@ -14665,15 +14926,6 @@
           <t>TEMINATLAR — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-      <c r="B1" s="434" t="n"/>
-      <c r="C1" s="434" t="n"/>
-      <c r="D1" s="434" t="n"/>
-      <c r="E1" s="434" t="n"/>
-      <c r="F1" s="434" t="n"/>
-      <c r="G1" s="434" t="n"/>
-      <c r="H1" s="434" t="n"/>
-      <c r="I1" s="434" t="n"/>
-      <c r="J1" s="434" t="n"/>
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
@@ -15327,7 +15579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AN35"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="76" min="1" max="1"/>
@@ -15348,16 +15600,6 @@
           <t>YENI TEKLIFLER — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-      <c r="B1" s="434" t="n"/>
-      <c r="C1" s="434" t="n"/>
-      <c r="D1" s="434" t="n"/>
-      <c r="E1" s="434" t="n"/>
-      <c r="F1" s="434" t="n"/>
-      <c r="G1" s="434" t="n"/>
-      <c r="H1" s="434" t="n"/>
-      <c r="I1" s="434" t="n"/>
-      <c r="J1" s="434" t="n"/>
-      <c r="K1" s="434" t="n"/>
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
@@ -16204,7 +16446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AN35"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="76" min="1" max="1"/>
@@ -16225,15 +16467,6 @@
           <t>REFINANSMAN — KURUMSAL BANKA VE BORÇ YÖNETİMİ</t>
         </is>
       </c>
-      <c r="B1" s="434" t="n"/>
-      <c r="C1" s="434" t="n"/>
-      <c r="D1" s="434" t="n"/>
-      <c r="E1" s="434" t="n"/>
-      <c r="F1" s="434" t="n"/>
-      <c r="G1" s="434" t="n"/>
-      <c r="H1" s="434" t="n"/>
-      <c r="I1" s="434" t="n"/>
-      <c r="J1" s="434" t="n"/>
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
@@ -18108,7 +18341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AN22"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="76" min="1" max="1"/>
@@ -18121,14 +18354,6 @@
           <t>KARAR MOTORU — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-      <c r="B1" s="434" t="n"/>
-      <c r="C1" s="434" t="n"/>
-      <c r="D1" s="434" t="n"/>
-      <c r="E1" s="434" t="n"/>
-      <c r="F1" s="434" t="n"/>
-      <c r="G1" s="434" t="n"/>
-      <c r="H1" s="434" t="n"/>
-      <c r="I1" s="434" t="n"/>
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
@@ -18949,7 +19174,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AN19"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="76" min="1" max="1"/>
@@ -18963,14 +19188,6 @@
           <t>SENARYO DUYARLILIK — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-      <c r="B1" s="434" t="n"/>
-      <c r="C1" s="434" t="n"/>
-      <c r="D1" s="434" t="n"/>
-      <c r="E1" s="434" t="n"/>
-      <c r="F1" s="434" t="n"/>
-      <c r="G1" s="434" t="n"/>
-      <c r="H1" s="434" t="n"/>
-      <c r="I1" s="434" t="n"/>
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
@@ -19227,7 +19444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AN18"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="76" min="1" max="1"/>
@@ -19240,15 +19457,6 @@
           <t>KONTROLLER — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-      <c r="B1" s="434" t="n"/>
-      <c r="C1" s="434" t="n"/>
-      <c r="D1" s="434" t="n"/>
-      <c r="E1" s="434" t="n"/>
-      <c r="F1" s="434" t="n"/>
-      <c r="G1" s="434" t="n"/>
-      <c r="H1" s="434" t="n"/>
-      <c r="I1" s="434" t="n"/>
-      <c r="J1" s="434" t="n"/>
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
@@ -19259,7 +19467,6 @@
       </c>
     </row>
     <row r="4" ht="10" customHeight="1" s="50"/>
-    <row r="5"/>
     <row r="6" ht="15" customHeight="1" s="50">
       <c r="A6" s="100" t="inlineStr">
         <is>
@@ -19907,14 +20114,6 @@
           <t>AYARLAR — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-      <c r="B1" s="434" t="n"/>
-      <c r="C1" s="434" t="n"/>
-      <c r="D1" s="434" t="n"/>
-      <c r="E1" s="434" t="n"/>
-      <c r="F1" s="434" t="n"/>
-      <c r="G1" s="434" t="n"/>
-      <c r="H1" s="434" t="n"/>
-      <c r="I1" s="434" t="n"/>
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50">
       <c r="A2" s="103" t="inlineStr">
@@ -19923,7 +20122,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="10" customHeight="1" s="50">
       <c r="A4" s="104" t="inlineStr">
         <is>
@@ -20895,7 +21093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AN11"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="76" min="1" max="1"/>
@@ -20919,18 +21117,6 @@
           <t>LISTELER — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-      <c r="B1" s="434" t="n"/>
-      <c r="C1" s="434" t="n"/>
-      <c r="D1" s="434" t="n"/>
-      <c r="E1" s="434" t="n"/>
-      <c r="F1" s="434" t="n"/>
-      <c r="G1" s="434" t="n"/>
-      <c r="H1" s="434" t="n"/>
-      <c r="I1" s="434" t="n"/>
-      <c r="J1" s="434" t="n"/>
-      <c r="K1" s="434" t="n"/>
-      <c r="L1" s="434" t="n"/>
-      <c r="M1" s="434" t="n"/>
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
@@ -25337,6 +25523,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -25346,7 +25533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AN11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="76" min="1" max="1"/>
@@ -25360,14 +25547,6 @@
           <t>ORNEK VERI — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-      <c r="B1" s="434" t="n"/>
-      <c r="C1" s="434" t="n"/>
-      <c r="D1" s="434" t="n"/>
-      <c r="E1" s="434" t="n"/>
-      <c r="F1" s="434" t="n"/>
-      <c r="G1" s="434" t="n"/>
-      <c r="H1" s="434" t="n"/>
-      <c r="I1" s="434" t="n"/>
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
@@ -25515,7 +25694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AN16"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="40" customWidth="1" style="76" min="1" max="1"/>
@@ -25529,14 +25708,6 @@
           <t>TESTLER — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-      <c r="B1" s="434" t="n"/>
-      <c r="C1" s="434" t="n"/>
-      <c r="D1" s="434" t="n"/>
-      <c r="E1" s="434" t="n"/>
-      <c r="F1" s="434" t="n"/>
-      <c r="G1" s="434" t="n"/>
-      <c r="H1" s="434" t="n"/>
-      <c r="I1" s="434" t="n"/>
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
@@ -25919,7 +26090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AN6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="76" min="1" max="1"/>
@@ -25933,14 +26104,6 @@
           <t>DEGISIKLIK KAYDI — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-      <c r="B1" s="434" t="n"/>
-      <c r="C1" s="434" t="n"/>
-      <c r="D1" s="434" t="n"/>
-      <c r="E1" s="434" t="n"/>
-      <c r="F1" s="434" t="n"/>
-      <c r="G1" s="434" t="n"/>
-      <c r="H1" s="434" t="n"/>
-      <c r="I1" s="434" t="n"/>
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
@@ -26486,7 +26649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AN35"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="76" min="1" max="1"/>
@@ -26506,14 +26669,6 @@
           <t>BANKALAR — KURUMSAL BANKA VE BORÇ YÖNETİMİ</t>
         </is>
       </c>
-      <c r="B1" s="434" t="n"/>
-      <c r="C1" s="434" t="n"/>
-      <c r="D1" s="434" t="n"/>
-      <c r="E1" s="434" t="n"/>
-      <c r="F1" s="434" t="n"/>
-      <c r="G1" s="434" t="n"/>
-      <c r="H1" s="434" t="n"/>
-      <c r="I1" s="434" t="n"/>
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
@@ -27159,7 +27314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AN35"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="76" min="1" max="1"/>
@@ -27179,14 +27334,6 @@
           <t>LIMITLER — KURUMSAL BANKA VE BORÇ YÖNETİMİ</t>
         </is>
       </c>
-      <c r="B1" s="434" t="n"/>
-      <c r="C1" s="434" t="n"/>
-      <c r="D1" s="434" t="n"/>
-      <c r="E1" s="434" t="n"/>
-      <c r="F1" s="434" t="n"/>
-      <c r="G1" s="434" t="n"/>
-      <c r="H1" s="434" t="n"/>
-      <c r="I1" s="434" t="n"/>
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
@@ -27982,7 +28129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AN35"/>
+  <dimension ref="A1:N35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="76" min="1" max="1"/>
@@ -28007,19 +28154,6 @@
           <t>KREDILER — KURUMSAL BANKA VE BORÇ YÖNETİMİ</t>
         </is>
       </c>
-      <c r="B1" s="434" t="n"/>
-      <c r="C1" s="434" t="n"/>
-      <c r="D1" s="434" t="n"/>
-      <c r="E1" s="434" t="n"/>
-      <c r="F1" s="434" t="n"/>
-      <c r="G1" s="434" t="n"/>
-      <c r="H1" s="434" t="n"/>
-      <c r="I1" s="434" t="n"/>
-      <c r="J1" s="434" t="n"/>
-      <c r="K1" s="434" t="n"/>
-      <c r="L1" s="434" t="n"/>
-      <c r="M1" s="434" t="n"/>
-      <c r="N1" s="434" t="n"/>
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
@@ -29046,7 +29180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AN35"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="76" min="1" max="2"/>
@@ -29069,17 +29203,6 @@
           <t>TAKSIT_PLANI — KURUMSAL BANKA VE BORÇ YÖNETİMİ</t>
         </is>
       </c>
-      <c r="B1" s="434" t="n"/>
-      <c r="C1" s="434" t="n"/>
-      <c r="D1" s="434" t="n"/>
-      <c r="E1" s="434" t="n"/>
-      <c r="F1" s="434" t="n"/>
-      <c r="G1" s="434" t="n"/>
-      <c r="H1" s="434" t="n"/>
-      <c r="I1" s="434" t="n"/>
-      <c r="J1" s="434" t="n"/>
-      <c r="K1" s="434" t="n"/>
-      <c r="L1" s="434" t="n"/>
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
@@ -30055,7 +30178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AN35"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="76" min="1" max="1"/>
@@ -30073,14 +30196,6 @@
           <t>ODEME_TAKVIMI — KURUMSAL BANKA VE BORÇ YÖNETİMİ</t>
         </is>
       </c>
-      <c r="B1" s="434" t="n"/>
-      <c r="C1" s="434" t="n"/>
-      <c r="D1" s="434" t="n"/>
-      <c r="E1" s="434" t="n"/>
-      <c r="F1" s="434" t="n"/>
-      <c r="G1" s="434" t="n"/>
-      <c r="H1" s="434" t="n"/>
-      <c r="I1" s="434" t="n"/>
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">

</xml_diff>

<commit_message>
feat(final): complete full-scale Siemens & 1,000 USD grade regeneration of banka-kredi-ve-taksit-takip-sistemi
</commit_message>
<xml_diff>
--- a/EXCELARSIV_PRODUCTS/banka-kredi-ve-taksit-takip-sistemi/BankaKrediVeTaksitTakipSistemi.xlsx
+++ b/EXCELARSIV_PRODUCTS/banka-kredi-ve-taksit-takip-sistemi/BankaKrediVeTaksitTakipSistemi.xlsx
@@ -1781,7 +1781,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="441">
+  <cellXfs count="443">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2889,6 +2889,12 @@
     </xf>
     <xf numFmtId="0" fontId="77" fillId="11" borderId="63" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="126" fillId="36" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="127" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -13878,7 +13884,7 @@
       <c r="B7" s="355" t="n"/>
       <c r="C7" s="356" t="inlineStr">
         <is>
-          <t>EĞİTİM VİDEOSU</t>
+          <t>1. SİSTEMİN ÖZÜ &amp; MANTIK</t>
         </is>
       </c>
       <c r="D7" s="357" t="n"/>
@@ -13887,7 +13893,7 @@
       <c r="H7" s="355" t="n"/>
       <c r="I7" s="356" t="inlineStr">
         <is>
-          <t>KULLANIM REHBERİ &amp; SÖZLÜK</t>
+          <t>2. YÖNETİCİ KOKPİTİ (PANO)</t>
         </is>
       </c>
       <c r="J7" s="357" t="n"/>
@@ -13896,7 +13902,7 @@
       <c r="N7" s="355" t="n"/>
       <c r="O7" s="356" t="inlineStr">
         <is>
-          <t>EXCEL ARŞİV HİZMETLERİ</t>
+          <t>3. VERİ GİRİŞİ &amp; STRES TESTİ</t>
         </is>
       </c>
       <c r="P7" s="357" t="n"/>
@@ -13924,21 +13930,21 @@
       <c r="B9" s="355" t="n"/>
       <c r="C9" s="358" t="inlineStr">
         <is>
-          <t>Bu şablonun nasıl kullanıldığını videolu ve detaylı bir şekilde öğrenmek için aşağıdaki düğmeye tıklayabilirsiniz.</t>
+          <t>5 yaşındaki bir çocuğun dahi anlayacağı yalınlıkta sistem özeti, kullanım kılavuzu ve finans terimleri sözlüğü.</t>
         </is>
       </c>
       <c r="F9" s="355" t="n"/>
       <c r="H9" s="355" t="n"/>
       <c r="I9" s="358" t="inlineStr">
         <is>
-          <t>5 yaşındaki birine anlatır gibi sadeleştirilmiş sistem özeti, kullanım kılavuzu ve finans terimleri sözlüğü için tıklayınız.</t>
+          <t>Banka borçlarını, 30 günlük ödeme baskısını ve refinansman tasarruf potansiyelini tek ekranda izleyin.</t>
         </is>
       </c>
       <c r="L9" s="355" t="n"/>
       <c r="N9" s="355" t="n"/>
       <c r="O9" s="358" t="inlineStr">
         <is>
-          <t>EXCELARŞİV olarak finansal modelleme, kurumsal danışmanlık ve karar destek sistemleri sunmaktayız. Daha fazlası için tıklayınız.</t>
+          <t>Kredi sözleşmelerini girin; -%20 nakit daralması kriz testini ve A4 kurumsal yönetim raporunu alın.</t>
         </is>
       </c>
       <c r="R9" s="355" t="n"/>
@@ -13988,7 +13994,7 @@
       <c r="B14" s="355" t="n"/>
       <c r="C14" s="359" t="inlineStr">
         <is>
-          <t>▶ KULLANIM VİDEOSUNU İZLE</t>
+          <t>📖 SİSTEM REHBERİ (#00_HAKKINDA_VE_REHBER!A1)</t>
         </is>
       </c>
       <c r="D14" s="369" t="n"/>
@@ -13997,7 +14003,7 @@
       <c r="H14" s="355" t="n"/>
       <c r="I14" s="359" t="inlineStr">
         <is>
-          <t>📖 REHBERİ VE SÖZLÜĞÜ AÇ (#00_HAKKINDA_VE_REHBER!A1)</t>
+          <t>▶ CANLI PANO (#PANO!A1)</t>
         </is>
       </c>
       <c r="J14" s="369" t="n"/>
@@ -14006,7 +14012,7 @@
       <c r="N14" s="355" t="n"/>
       <c r="O14" s="359" t="inlineStr">
         <is>
-          <t>🌐 WEB SİTEMİZİ ZİYARET EDİN</t>
+          <t>📋 GİRDİLERİ DÜZENLE (#GİRDİLER!A1)</t>
         </is>
       </c>
       <c r="P14" s="369" t="n"/>
@@ -24791,6 +24797,7 @@
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
+    <tabColor rgb="0064748B"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
@@ -24801,13 +24808,22 @@
     <col width="22" customWidth="1" style="76" min="2" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" s="50">
-      <c r="A1" s="77" t="inlineStr">
+    <row r="1" ht="32" customHeight="1" s="50">
+      <c r="A1" s="441" t="inlineStr">
         <is>
           <t>KAPAK — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-    </row>
+      <c r="B1" s="434" t="n"/>
+      <c r="C1" s="434" t="n"/>
+      <c r="D1" s="434" t="n"/>
+      <c r="E1" s="434" t="n"/>
+      <c r="F1" s="434" t="n"/>
+      <c r="G1" s="434" t="n"/>
+      <c r="H1" s="434" t="n"/>
+      <c r="I1" s="434" t="n"/>
+    </row>
+    <row r="3"/>
     <row r="6" ht="31.5" customHeight="1" s="50">
       <c r="A6" s="78" t="inlineStr">
         <is>
@@ -24902,7 +24918,7 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:AN1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -24913,6 +24929,7 @@
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
+    <tabColor rgb="0064748B"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
@@ -24922,15 +24939,23 @@
     <col width="80" customWidth="1" style="76" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="50">
-      <c r="A1" s="77" t="inlineStr">
+    <row r="1" ht="32" customHeight="1" s="50">
+      <c r="A1" s="441" t="inlineStr">
         <is>
           <t>HIZLI BASLANGIC — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="19.5" customHeight="1" s="50">
-      <c r="A3" s="83" t="inlineStr">
+      <c r="B1" s="434" t="n"/>
+      <c r="C1" s="434" t="n"/>
+      <c r="D1" s="434" t="n"/>
+      <c r="E1" s="434" t="n"/>
+      <c r="F1" s="434" t="n"/>
+      <c r="G1" s="434" t="n"/>
+      <c r="H1" s="434" t="n"/>
+      <c r="I1" s="434" t="n"/>
+    </row>
+    <row r="3" ht="22" customHeight="1" s="50">
+      <c r="A3" s="442" t="inlineStr">
         <is>
           <t>3 ADIMDA SİSTEM</t>
         </is>
@@ -24987,11 +25012,12 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="0" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A12:BH12"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A6:BH6"/>
     <mergeCell ref="A9:BH9"/>
-    <mergeCell ref="A1:AN1"/>
-    <mergeCell ref="A6:BH6"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -25581,6 +25607,7 @@
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
+    <tabColor rgb="0064748B"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
@@ -25742,6 +25769,7 @@
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
+    <tabColor rgb="0064748B"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
@@ -25913,10 +25941,11 @@
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
+    <tabColor rgb="0064748B"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="76" min="1" max="1"/>
@@ -25927,47 +25956,25 @@
     <col width="40" customWidth="1" style="76" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="50">
-      <c r="A1" s="76" t="inlineStr">
+    <row r="1" ht="32" customHeight="1" s="50">
+      <c r="A1" s="441" t="inlineStr">
         <is>
           <t>AKIS — BankaKrediVeTaksitTakipSistemi</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="50">
-      <c r="A3" s="76" t="inlineStr">
+      <c r="B1" s="434" t="n"/>
+      <c r="C1" s="434" t="n"/>
+      <c r="D1" s="434" t="n"/>
+      <c r="E1" s="434" t="n"/>
+      <c r="F1" s="434" t="n"/>
+      <c r="G1" s="434" t="n"/>
+      <c r="H1" s="434" t="n"/>
+      <c r="I1" s="434" t="n"/>
+    </row>
+    <row r="3" ht="22" customHeight="1" s="50">
+      <c r="A3" s="442" t="inlineStr">
         <is>
           <t>islem_id</t>
-        </is>
-      </c>
-      <c r="B3" s="76" t="inlineStr">
-        <is>
-          <t>kaynak_kart_id</t>
-        </is>
-      </c>
-      <c r="C3" s="76" t="inlineStr">
-        <is>
-          <t>onceki_durum</t>
-        </is>
-      </c>
-      <c r="D3" s="76" t="inlineStr">
-        <is>
-          <t>yeni_durum</t>
-        </is>
-      </c>
-      <c r="E3" s="76" t="inlineStr">
-        <is>
-          <t>tutar</t>
-        </is>
-      </c>
-      <c r="F3" s="76" t="inlineStr">
-        <is>
-          <t>bayrak</t>
-        </is>
-      </c>
-      <c r="G3" s="76" t="inlineStr">
-        <is>
-          <t>not</t>
         </is>
       </c>
     </row>
@@ -26129,6 +26136,10 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="cc3d"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
+  </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -26138,6 +26149,7 @@
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
+    <tabColor rgb="0064748B"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>

</xml_diff>

<commit_message>
refactor(tone): replace informal ELI5 wording with C-Level executive tone across workbooks and lock Mandate Rule 254
</commit_message>
<xml_diff>
--- a/EXCELARSIV_PRODUCTS/banka-kredi-ve-taksit-takip-sistemi/BankaKrediVeTaksitTakipSistemi.xlsx
+++ b/EXCELARSIV_PRODUCTS/banka-kredi-ve-taksit-takip-sistemi/BankaKrediVeTaksitTakipSistemi.xlsx
@@ -13930,7 +13930,7 @@
       <c r="B9" s="355" t="n"/>
       <c r="C9" s="358" t="inlineStr">
         <is>
-          <t>5 yaşındaki bir çocuğun dahi anlayacağı yalınlıkta sistem özeti, kullanım kılavuzu ve finans terimleri sözlüğü.</t>
+          <t>Her kademedeki yöneticinin anında kavrayabileceği yalınlıkta sistem özeti, kullanım kılavuzu ve finans terimleri sözlüğü.</t>
         </is>
       </c>
       <c r="F9" s="355" t="n"/>
@@ -14345,7 +14345,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
-      <c r="A1" s="433" t="inlineStr">
+      <c r="A1" s="441" t="inlineStr">
         <is>
           <t>MASRAF KOMISYON — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
@@ -14353,7 +14353,7 @@
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
-      <c r="A3" s="435" t="inlineStr">
+      <c r="A3" s="442" t="inlineStr">
         <is>
           <t>MASRAF VE KOMİSYONLAR — tahsis, sigorta, komisyon ve diğer finansman maliyetleri.</t>
         </is>
@@ -14978,7 +14978,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
-      <c r="A1" s="433" t="inlineStr">
+      <c r="A1" s="441" t="inlineStr">
         <is>
           <t>TEMINATLAR — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
@@ -14986,7 +14986,7 @@
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
-      <c r="A3" s="435" t="inlineStr">
+      <c r="A3" s="442" t="inlineStr">
         <is>
           <t>TEMİNAT YÖNETİMİ — değer, geçerlilik ve kredi bağlantısı.</t>
         </is>
@@ -15652,7 +15652,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
-      <c r="A1" s="433" t="inlineStr">
+      <c r="A1" s="441" t="inlineStr">
         <is>
           <t>YENI TEKLIFLER — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
@@ -15660,7 +15660,7 @@
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
-      <c r="A3" s="435" t="inlineStr">
+      <c r="A3" s="442" t="inlineStr">
         <is>
           <t>YENİ KREDİ TEKLİFLERİ — tutar, faiz, masraf ve aylık taksit karşılaştırması.</t>
         </is>
@@ -16519,7 +16519,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
-      <c r="A1" s="433" t="inlineStr">
+      <c r="A1" s="441" t="inlineStr">
         <is>
           <t>REFINANSMAN — KURUMSAL BANKA VE BORÇ YÖNETİMİ</t>
         </is>
@@ -16527,7 +16527,7 @@
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
-      <c r="A3" s="435" t="inlineStr">
+      <c r="A3" s="442" t="inlineStr">
         <is>
           <t>REFİNANSMAN ANALİZİ — aylık taksit rahatlaması ve toplam maliyet.</t>
         </is>
@@ -18406,7 +18406,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
-      <c r="A1" s="433" t="inlineStr">
+      <c r="A1" s="441" t="inlineStr">
         <is>
           <t>KARAR MOTORU — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
@@ -18414,7 +18414,7 @@
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
-      <c r="A3" s="435" t="inlineStr">
+      <c r="A3" s="442" t="inlineStr">
         <is>
           <t>KARAR MOTORU — borç yükü, yaklaşan taksit ve öncelikli aksiyon</t>
         </is>
@@ -19240,7 +19240,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
-      <c r="A1" s="433" t="inlineStr">
+      <c r="A1" s="441" t="inlineStr">
         <is>
           <t>SENARYO DUYARLILIK — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
@@ -19248,7 +19248,7 @@
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
-      <c r="A3" s="435" t="inlineStr">
+      <c r="A3" s="442" t="inlineStr">
         <is>
           <t>SENARYO VE DUYARLILIK ANALİZİ</t>
         </is>
@@ -19509,7 +19509,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
-      <c r="A1" s="433" t="inlineStr">
+      <c r="A1" s="441" t="inlineStr">
         <is>
           <t>KONTROLLER — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
@@ -19517,7 +19517,7 @@
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
-      <c r="A3" s="435" t="inlineStr">
+      <c r="A3" s="442" t="inlineStr">
         <is>
           <t>VERİ KALİTESİ VE SİSTEM SAĞLIĞI</t>
         </is>
@@ -19704,7 +19704,7 @@
     <row r="3" ht="20" customHeight="1" s="50">
       <c r="B3" s="430" t="inlineStr">
         <is>
-          <t>5 Yaşındaki Birine Anlatır Gibi Basit, Sade ve Eksiksiz Finansal Karar Mimarisi · Siemens &amp; Enterprise Standartları</t>
+          <t>Yalın, Sade ve Eksiksiz Finansal Karar Mimarisi &amp; Kullanım Rehberi · Siemens &amp; Enterprise Standartları</t>
         </is>
       </c>
     </row>
@@ -19723,7 +19723,7 @@
       </c>
       <c r="C7" s="375" t="inlineStr">
         <is>
-          <t>GÜNLÜK DİLLE CEVAP (5 YAŞINDA ÇOCUĞA ANLATIR GİBİ)</t>
+          <t>YALIN KURUMSAL AÇIKLAMA</t>
         </is>
       </c>
       <c r="D7" s="375" t="inlineStr">
@@ -20166,7 +20166,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
-      <c r="A1" s="433" t="inlineStr">
+      <c r="A1" s="441" t="inlineStr">
         <is>
           <t>AYARLAR — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
@@ -21169,7 +21169,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
-      <c r="A1" s="433" t="inlineStr">
+      <c r="A1" s="441" t="inlineStr">
         <is>
           <t>LISTELER — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
@@ -21177,7 +21177,7 @@
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
-      <c r="A3" s="435" t="inlineStr">
+      <c r="A3" s="442" t="inlineStr">
         <is>
           <t>AÇILIR LİSTE KAYNAKLARI</t>
         </is>
@@ -24801,7 +24801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AN23"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" style="76" min="1" max="1"/>
@@ -24814,16 +24814,7 @@
           <t>KAPAK — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-      <c r="B1" s="434" t="n"/>
-      <c r="C1" s="434" t="n"/>
-      <c r="D1" s="434" t="n"/>
-      <c r="E1" s="434" t="n"/>
-      <c r="F1" s="434" t="n"/>
-      <c r="G1" s="434" t="n"/>
-      <c r="H1" s="434" t="n"/>
-      <c r="I1" s="434" t="n"/>
-    </row>
-    <row r="3"/>
+    </row>
     <row r="6" ht="31.5" customHeight="1" s="50">
       <c r="A6" s="78" t="inlineStr">
         <is>
@@ -24945,14 +24936,6 @@
           <t>HIZLI BASLANGIC — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
       </c>
-      <c r="B1" s="434" t="n"/>
-      <c r="C1" s="434" t="n"/>
-      <c r="D1" s="434" t="n"/>
-      <c r="E1" s="434" t="n"/>
-      <c r="F1" s="434" t="n"/>
-      <c r="G1" s="434" t="n"/>
-      <c r="H1" s="434" t="n"/>
-      <c r="I1" s="434" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1" s="50">
       <c r="A3" s="442" t="inlineStr">
@@ -25620,7 +25603,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
-      <c r="A1" s="433" t="inlineStr">
+      <c r="A1" s="441" t="inlineStr">
         <is>
           <t>ORNEK VERI — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
@@ -25628,7 +25611,7 @@
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
-      <c r="A3" s="435" t="inlineStr">
+      <c r="A3" s="442" t="inlineStr">
         <is>
           <t>ÖRNEK VERİ — otomasyon ve içe aktarma için yapı</t>
         </is>
@@ -25782,7 +25765,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
-      <c r="A1" s="433" t="inlineStr">
+      <c r="A1" s="441" t="inlineStr">
         <is>
           <t>TESTLER — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
@@ -25790,7 +25773,7 @@
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
-      <c r="A3" s="435" t="inlineStr">
+      <c r="A3" s="442" t="inlineStr">
         <is>
           <t>SİSTEM TESTLERİ VE DENETİM KAYDI</t>
         </is>
@@ -25962,14 +25945,6 @@
           <t>AKIS — BankaKrediVeTaksitTakipSistemi</t>
         </is>
       </c>
-      <c r="B1" s="434" t="n"/>
-      <c r="C1" s="434" t="n"/>
-      <c r="D1" s="434" t="n"/>
-      <c r="E1" s="434" t="n"/>
-      <c r="F1" s="434" t="n"/>
-      <c r="G1" s="434" t="n"/>
-      <c r="H1" s="434" t="n"/>
-      <c r="I1" s="434" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1" s="50">
       <c r="A3" s="442" t="inlineStr">
@@ -26162,7 +26137,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
-      <c r="A1" s="433" t="inlineStr">
+      <c r="A1" s="441" t="inlineStr">
         <is>
           <t>DEGISIKLIK KAYDI — BANKA, KREDİ VE TAKSİT TAKİP SİSTEMİ</t>
         </is>
@@ -26170,7 +26145,7 @@
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
-      <c r="A3" s="435" t="inlineStr">
+      <c r="A3" s="442" t="inlineStr">
         <is>
           <t>DEĞİŞİKLİK KAYDI</t>
         </is>
@@ -26727,7 +26702,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
-      <c r="A1" s="433" t="inlineStr">
+      <c r="A1" s="441" t="inlineStr">
         <is>
           <t>BANKALAR — KURUMSAL BANKA VE BORÇ YÖNETİMİ</t>
         </is>
@@ -26735,7 +26710,7 @@
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
-      <c r="A3" s="435" t="inlineStr">
+      <c r="A3" s="442" t="inlineStr">
         <is>
           <t>BANKA TANIMLARI — ilişki, operasyonel durum ve iletişim tek merkezde.</t>
         </is>
@@ -27392,7 +27367,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
-      <c r="A1" s="433" t="inlineStr">
+      <c r="A1" s="441" t="inlineStr">
         <is>
           <t>LIMITLER — KURUMSAL BANKA VE BORÇ YÖNETİMİ</t>
         </is>
@@ -27400,7 +27375,7 @@
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
-      <c r="A3" s="435" t="inlineStr">
+      <c r="A3" s="442" t="inlineStr">
         <is>
           <t>BANKA LİMİTLERİ — toplam, kullanılan ve kalan limit ile kullanım oranı.</t>
         </is>
@@ -28212,7 +28187,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
-      <c r="A1" s="433" t="inlineStr">
+      <c r="A1" s="441" t="inlineStr">
         <is>
           <t>KREDILER — KURUMSAL BANKA VE BORÇ YÖNETİMİ</t>
         </is>
@@ -28220,7 +28195,7 @@
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
-      <c r="A3" s="435" t="inlineStr">
+      <c r="A3" s="442" t="inlineStr">
         <is>
           <t>KREDİ PORTFÖYÜ — sözleşme, bakiye, maliyet, vade ve taksit bilgileri.</t>
         </is>
@@ -29261,7 +29236,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
-      <c r="A1" s="433" t="inlineStr">
+      <c r="A1" s="441" t="inlineStr">
         <is>
           <t>TAKSIT_PLANI — KURUMSAL BANKA VE BORÇ YÖNETİMİ</t>
         </is>
@@ -29269,7 +29244,7 @@
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
-      <c r="A3" s="435" t="inlineStr">
+      <c r="A3" s="442" t="inlineStr">
         <is>
           <t>TAKSİT PLANI — dönem bazında anapara, faiz, vergi ve ödeme tarihi.</t>
         </is>
@@ -30254,7 +30229,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
-      <c r="A1" s="433" t="inlineStr">
+      <c r="A1" s="441" t="inlineStr">
         <is>
           <t>ODEME_TAKVIMI — KURUMSAL BANKA VE BORÇ YÖNETİMİ</t>
         </is>
@@ -30262,7 +30237,7 @@
     </row>
     <row r="2" ht="7.8" customHeight="1" s="50"/>
     <row r="3" ht="22" customHeight="1" s="50">
-      <c r="A3" s="435" t="inlineStr">
+      <c r="A3" s="442" t="inlineStr">
         <is>
           <t>ÖDEME TAKVİMİ — yaklaşan taksitler 30 / 60 / 90 gün penceresinde.</t>
         </is>

</xml_diff>

<commit_message>
feat(charts): lock Rule 255 zero-overlap layout, isolated canvas rows, anti-collision legend positioning and auto-padded columns
</commit_message>
<xml_diff>
--- a/EXCELARSIV_PRODUCTS/banka-kredi-ve-taksit-takip-sistemi/BankaKrediVeTaksitTakipSistemi.xlsx
+++ b/EXCELARSIV_PRODUCTS/banka-kredi-ve-taksit-takip-sistemi/BankaKrediVeTaksitTakipSistemi.xlsx
@@ -3141,6 +3141,7 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -3288,7 +3289,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Endeks / Milyon TL</a:t>
+                  <a:t>Tutar (Milyon TL)</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -3300,7 +3301,7 @@
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="r"/>
+      <legendPos val="t"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -3310,6 +3311,7 @@
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -3320,7 +3322,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>BORÇ DAĞILIMI VE RİSK YOĞUNLAŞMASI</a:t>
+              <a:t>KONSOLİDE RİSK VE BORÇ DAĞILIMI</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -3397,6 +3399,10 @@
             </numRef>
           </val>
         </ser>
+        <dLbls>
+          <showVal val="0"/>
+          <showPercent val="1"/>
+        </dLbls>
         <firstSliceAng val="0"/>
         <holeSize val="60"/>
       </doughnutChart>
@@ -13359,7 +13365,7 @@
       <row>27</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5940000" cy="3420000"/>
+    <ext cx="5580000" cy="3780000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -13381,7 +13387,7 @@
       <row>27</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5220000" cy="3420000"/>
+    <ext cx="7200000" cy="3780000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -14331,17 +14337,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:N35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="11" customWidth="1" style="76" min="1" max="2"/>
+    <col width="13.5" customWidth="1" style="76" min="1" max="2"/>
+    <col width="13" customWidth="1" style="50" min="2" max="2"/>
     <col width="24" customWidth="1" style="76" min="3" max="3"/>
     <col width="18" customWidth="1" style="76" min="4" max="4"/>
-    <col width="13" customWidth="1" style="76" min="5" max="5"/>
-    <col width="15" customWidth="1" style="76" min="6" max="6"/>
+    <col width="23.5" customWidth="1" style="76" min="5" max="5"/>
+    <col width="18.5" customWidth="1" style="76" min="6" max="6"/>
     <col width="14" customWidth="1" style="76" min="7" max="7"/>
-    <col width="13" customWidth="1" style="76" min="8" max="8"/>
-    <col width="10" customWidth="1" style="76" min="9" max="9"/>
+    <col width="15.5" customWidth="1" style="76" min="8" max="8"/>
+    <col width="11.5" customWidth="1" style="76" min="9" max="9"/>
+    <col width="13" customWidth="1" style="50" min="10" max="10"/>
+    <col width="13" customWidth="1" style="50" min="11" max="11"/>
+    <col width="13" customWidth="1" style="50" min="12" max="12"/>
+    <col width="13" customWidth="1" style="50" min="13" max="13"/>
+    <col width="13" customWidth="1" style="50" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
@@ -14962,19 +14974,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:N35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="12" customWidth="1" style="76" min="1" max="1"/>
-    <col width="11" customWidth="1" style="76" min="2" max="2"/>
+    <col width="14.5" customWidth="1" style="76" min="1" max="1"/>
+    <col width="12.5" customWidth="1" style="76" min="2" max="2"/>
     <col width="24" customWidth="1" style="76" min="3" max="3"/>
-    <col width="20" customWidth="1" style="76" min="4" max="4"/>
-    <col width="24" customWidth="1" style="76" min="5" max="5"/>
-    <col width="16" customWidth="1" style="76" min="6" max="6"/>
-    <col width="13" customWidth="1" style="76" min="7" max="7"/>
-    <col width="14" customWidth="1" style="76" min="8" max="8"/>
-    <col width="15" customWidth="1" style="76" min="9" max="9"/>
-    <col width="10" customWidth="1" style="76" min="10" max="10"/>
+    <col width="23.5" customWidth="1" style="76" min="4" max="4"/>
+    <col width="27.5" customWidth="1" style="76" min="5" max="5"/>
+    <col width="20.5" customWidth="1" style="76" min="6" max="6"/>
+    <col width="15.5" customWidth="1" style="76" min="7" max="7"/>
+    <col width="23.5" customWidth="1" style="76" min="8" max="8"/>
+    <col width="23.5" customWidth="1" style="76" min="9" max="9"/>
+    <col width="11.5" customWidth="1" style="76" min="10" max="10"/>
+    <col width="13" customWidth="1" style="50" min="11" max="11"/>
+    <col width="13" customWidth="1" style="50" min="12" max="12"/>
+    <col width="13" customWidth="1" style="50" min="13" max="13"/>
+    <col width="13" customWidth="1" style="50" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
@@ -15636,19 +15652,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:N35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="12" customWidth="1" style="76" min="1" max="1"/>
-    <col width="15" customWidth="1" style="76" min="2" max="2"/>
+    <col width="13.5" customWidth="1" style="76" min="1" max="1"/>
+    <col width="18.5" customWidth="1" style="76" min="2" max="2"/>
     <col width="24" customWidth="1" style="76" min="3" max="3"/>
     <col width="14" customWidth="1" style="76" min="4" max="4"/>
-    <col width="13" customWidth="1" style="76" min="5" max="5"/>
-    <col width="10" customWidth="1" style="76" min="6" max="6"/>
-    <col width="13" customWidth="1" style="76" min="7" max="7"/>
-    <col width="15" customWidth="1" style="76" min="8" max="9"/>
-    <col width="18" customWidth="1" style="76" min="10" max="10"/>
-    <col width="10" customWidth="1" style="76" min="11" max="11"/>
+    <col width="15.5" customWidth="1" style="76" min="5" max="5"/>
+    <col width="11.5" customWidth="1" style="76" min="6" max="6"/>
+    <col width="16.5" customWidth="1" style="76" min="7" max="7"/>
+    <col width="17.5" customWidth="1" style="76" min="8" max="9"/>
+    <col width="16.5" customWidth="1" style="50" min="9" max="9"/>
+    <col width="21.5" customWidth="1" style="76" min="10" max="10"/>
+    <col width="11.5" customWidth="1" style="76" min="11" max="11"/>
+    <col width="13" customWidth="1" style="50" min="12" max="12"/>
+    <col width="13" customWidth="1" style="50" min="13" max="13"/>
+    <col width="13" customWidth="1" style="50" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
@@ -16503,19 +16523,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:N35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="76" min="1" max="1"/>
-    <col width="15" customWidth="1" style="76" min="2" max="2"/>
-    <col width="20" customWidth="1" style="76" min="3" max="3"/>
-    <col width="20" customWidth="1" style="76" min="4" max="6"/>
-    <col width="18" customWidth="1" style="50" min="5" max="5"/>
-    <col width="18" customWidth="1" style="50" min="6" max="6"/>
-    <col width="20" customWidth="1" style="76" min="7" max="8"/>
-    <col width="20" customWidth="1" style="50" min="8" max="8"/>
+    <col width="18.5" customWidth="1" style="76" min="2" max="2"/>
+    <col width="23.5" customWidth="1" style="76" min="3" max="3"/>
+    <col width="21.5" customWidth="1" style="76" min="4" max="6"/>
+    <col width="22.5" customWidth="1" style="50" min="5" max="5"/>
+    <col width="21.5" customWidth="1" style="50" min="6" max="6"/>
+    <col width="23.5" customWidth="1" style="76" min="7" max="8"/>
+    <col width="24.5" customWidth="1" style="50" min="8" max="8"/>
     <col width="14" customWidth="1" style="76" min="9" max="9"/>
     <col width="14" customWidth="1" style="76" min="10" max="10"/>
+    <col width="13" customWidth="1" style="50" min="11" max="11"/>
+    <col width="13" customWidth="1" style="50" min="12" max="12"/>
+    <col width="13" customWidth="1" style="50" min="13" max="13"/>
+    <col width="13" customWidth="1" style="50" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
@@ -25571,6 +25595,26 @@
       <c r="H27" s="250" t="n"/>
       <c r="I27" s="251" t="n"/>
     </row>
+    <row r="28" ht="18" customHeight="1" s="50"/>
+    <row r="29" ht="18" customHeight="1" s="50"/>
+    <row r="30" ht="18" customHeight="1" s="50"/>
+    <row r="31" ht="18" customHeight="1" s="50"/>
+    <row r="32" ht="18" customHeight="1" s="50"/>
+    <row r="33" ht="18" customHeight="1" s="50"/>
+    <row r="34" ht="18" customHeight="1" s="50"/>
+    <row r="35" ht="18" customHeight="1" s="50"/>
+    <row r="36" ht="18" customHeight="1" s="50"/>
+    <row r="37" ht="18" customHeight="1" s="50"/>
+    <row r="38" ht="18" customHeight="1" s="50"/>
+    <row r="39" ht="18" customHeight="1" s="50"/>
+    <row r="40" ht="18" customHeight="1" s="50"/>
+    <row r="41" ht="18" customHeight="1" s="50"/>
+    <row r="42" ht="18" customHeight="1" s="50"/>
+    <row r="43" ht="18" customHeight="1" s="50"/>
+    <row r="44" ht="18" customHeight="1" s="50"/>
+    <row r="45" ht="18" customHeight="1" s="50"/>
+    <row r="46" ht="18" customHeight="1" s="50"/>
+    <row r="47" ht="18" customHeight="1" s="50"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="B2:M2"/>
@@ -26687,18 +26731,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:N35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="76" min="1" max="1"/>
     <col width="26" customWidth="1" style="76" min="2" max="2"/>
-    <col width="18" customWidth="1" style="76" min="3" max="3"/>
-    <col width="18" customWidth="1" style="76" min="4" max="4"/>
+    <col width="20.5" customWidth="1" style="76" min="3" max="3"/>
+    <col width="20.5" customWidth="1" style="76" min="4" max="4"/>
     <col width="32" customWidth="1" style="76" min="5" max="5"/>
     <col width="14" customWidth="1" style="76" min="6" max="6"/>
-    <col width="20" customWidth="1" style="76" min="7" max="7"/>
-    <col width="18" customWidth="1" style="76" min="8" max="8"/>
+    <col width="21.5" customWidth="1" style="76" min="7" max="7"/>
+    <col width="18.5" customWidth="1" style="76" min="8" max="8"/>
     <col width="14" customWidth="1" style="76" min="9" max="9"/>
+    <col width="13" customWidth="1" style="50" min="10" max="10"/>
+    <col width="13" customWidth="1" style="50" min="11" max="11"/>
+    <col width="13" customWidth="1" style="50" min="12" max="12"/>
+    <col width="13" customWidth="1" style="50" min="13" max="13"/>
+    <col width="13" customWidth="1" style="50" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
@@ -27352,18 +27401,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:N35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="76" min="1" max="1"/>
     <col width="26" customWidth="1" style="76" min="2" max="2"/>
-    <col width="22" customWidth="1" style="76" min="3" max="3"/>
-    <col width="14" customWidth="1" style="76" min="4" max="4"/>
+    <col width="25.5" customWidth="1" style="76" min="3" max="3"/>
+    <col width="15.5" customWidth="1" style="76" min="4" max="4"/>
     <col width="18" customWidth="1" style="76" min="5" max="5"/>
-    <col width="18" customWidth="1" style="76" min="6" max="6"/>
+    <col width="20.5" customWidth="1" style="76" min="6" max="6"/>
     <col width="18" customWidth="1" style="76" min="7" max="7"/>
-    <col width="16" customWidth="1" style="76" min="8" max="8"/>
+    <col width="18.5" customWidth="1" style="76" min="8" max="8"/>
     <col width="14" customWidth="1" style="76" min="9" max="9"/>
+    <col width="13" customWidth="1" style="50" min="10" max="10"/>
+    <col width="13" customWidth="1" style="50" min="11" max="11"/>
+    <col width="13" customWidth="1" style="50" min="12" max="12"/>
+    <col width="13" customWidth="1" style="50" min="13" max="13"/>
+    <col width="13" customWidth="1" style="50" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
@@ -28172,13 +28226,13 @@
   <cols>
     <col width="13" customWidth="1" style="76" min="1" max="1"/>
     <col width="26" customWidth="1" style="76" min="2" max="2"/>
-    <col width="18" customWidth="1" style="76" min="3" max="3"/>
-    <col width="24" customWidth="1" style="76" min="4" max="4"/>
-    <col width="14" customWidth="1" style="76" min="5" max="5"/>
-    <col width="18" customWidth="1" style="76" min="6" max="7"/>
+    <col width="19.5" customWidth="1" style="76" min="3" max="3"/>
+    <col width="25.5" customWidth="1" style="76" min="4" max="4"/>
+    <col width="15.5" customWidth="1" style="76" min="5" max="5"/>
+    <col width="23.5" customWidth="1" style="76" min="6" max="7"/>
     <col width="18" customWidth="1" style="50" min="7" max="7"/>
     <col width="18" customWidth="1" style="76" min="8" max="8"/>
-    <col width="14" customWidth="1" style="76" min="9" max="9"/>
+    <col width="15.5" customWidth="1" style="76" min="9" max="9"/>
     <col width="13" customWidth="1" style="76" min="10" max="10"/>
     <col width="18" customWidth="1" style="76" min="11" max="11"/>
     <col width="18" customWidth="1" style="76" min="12" max="12"/>
@@ -29218,21 +29272,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:N35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="76" min="1" max="2"/>
     <col width="13" customWidth="1" style="50" min="2" max="2"/>
     <col width="10" customWidth="1" style="76" min="3" max="3"/>
-    <col width="18" customWidth="1" style="76" min="4" max="6"/>
+    <col width="23.5" customWidth="1" style="76" min="4" max="6"/>
     <col width="18" customWidth="1" style="50" min="5" max="5"/>
     <col width="18" customWidth="1" style="50" min="6" max="6"/>
     <col width="14" customWidth="1" style="76" min="7" max="7"/>
     <col width="14" customWidth="1" style="76" min="8" max="8"/>
     <col width="18" customWidth="1" style="76" min="9" max="9"/>
-    <col width="15" customWidth="1" style="76" min="10" max="10"/>
+    <col width="16.5" customWidth="1" style="76" min="10" max="10"/>
     <col width="14" customWidth="1" style="76" min="11" max="11"/>
     <col width="14" customWidth="1" style="76" min="12" max="12"/>
+    <col width="13" customWidth="1" style="50" min="13" max="13"/>
+    <col width="13" customWidth="1" style="50" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">
@@ -30216,7 +30272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:N35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="76" min="1" max="1"/>
@@ -30225,7 +30281,14 @@
     <col width="18" customWidth="1" style="76" min="4" max="4"/>
     <col width="14" customWidth="1" style="76" min="5" max="5"/>
     <col width="18" customWidth="1" style="76" min="6" max="6"/>
-    <col width="15" customWidth="1" style="76" min="7" max="7"/>
+    <col width="16.5" customWidth="1" style="76" min="7" max="7"/>
+    <col width="13" customWidth="1" style="50" min="8" max="8"/>
+    <col width="13" customWidth="1" style="50" min="9" max="9"/>
+    <col width="13" customWidth="1" style="50" min="10" max="10"/>
+    <col width="13" customWidth="1" style="50" min="11" max="11"/>
+    <col width="13" customWidth="1" style="50" min="12" max="12"/>
+    <col width="13" customWidth="1" style="50" min="13" max="13"/>
+    <col width="13" customWidth="1" style="50" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="50">

</xml_diff>

<commit_message>
fix(layout): resolve KILAVUZ column clipping, eliminate chart title-legend overlap and enforce Mandate Rule 256
</commit_message>
<xml_diff>
--- a/EXCELARSIV_PRODUCTS/banka-kredi-ve-taksit-takip-sistemi/BankaKrediVeTaksitTakipSistemi.xlsx
+++ b/EXCELARSIV_PRODUCTS/banka-kredi-ve-taksit-takip-sistemi/BankaKrediVeTaksitTakipSistemi.xlsx
@@ -1106,7 +1106,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="64">
+  <borders count="65">
     <border>
       <left/>
       <right/>
@@ -1770,6 +1770,7 @@
       </top>
       <bottom/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -1781,7 +1782,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="443">
+  <cellXfs count="455">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -2896,6 +2897,40 @@
     <xf numFmtId="0" fontId="127" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="38" fillId="36" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="36" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="18" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="18" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="118" fillId="18" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="124" fillId="18" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="66" fillId="36" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="77" fillId="19" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="19" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="118" fillId="19" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="124" fillId="19" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="64" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3301,7 +3336,7 @@
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="t"/>
+      <legendPos val="r"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -3322,7 +3357,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>KONSOLİDE RİSK VE BORÇ DAĞILIMI</a:t>
+              <a:t>KONSOLİDE BORÇ DAĞILIMI</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -3399,10 +3434,6 @@
             </numRef>
           </val>
         </ser>
-        <dLbls>
-          <showVal val="0"/>
-          <showPercent val="1"/>
-        </dLbls>
         <firstSliceAng val="0"/>
         <holeSize val="60"/>
       </doughnutChart>
@@ -13362,10 +13393,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>27</row>
+      <row>29</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5580000" cy="3780000"/>
+    <ext cx="5760000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -13384,10 +13415,10 @@
     <from>
       <col>7</col>
       <colOff>0</colOff>
-      <row>27</row>
+      <row>29</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7200000" cy="3780000"/>
+    <ext cx="6480000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -13826,8 +13857,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.6" customWidth="1" style="50" min="1" max="1"/>
-    <col width="3.7" customWidth="1" style="50" min="2" max="2"/>
-    <col width="10.4" customWidth="1" style="50" min="3" max="3"/>
+    <col width="12" customWidth="1" style="50" min="2" max="2"/>
+    <col width="30" customWidth="1" style="50" min="3" max="3"/>
     <col width="13" customWidth="1" style="50" min="4" max="4"/>
     <col width="13" customWidth="1" style="50" min="5" max="5"/>
     <col width="3.7" customWidth="1" style="50" min="6" max="6"/>
@@ -14068,230 +14099,231 @@
       </c>
     </row>
     <row r="21" ht="26" customHeight="1" s="50">
-      <c r="B21" s="362" t="inlineStr">
+      <c r="B21" s="443" t="inlineStr">
         <is>
           <t>AŞAMA NO</t>
         </is>
       </c>
-      <c r="C21" s="362" t="inlineStr">
+      <c r="C21" s="444" t="inlineStr">
         <is>
           <t>AŞAMA ADI &amp; KAPSAM</t>
         </is>
       </c>
-      <c r="D21" s="362" t="inlineStr">
-        <is>
-          <t>İŞLEM DETAYI VE MANTIK</t>
-        </is>
-      </c>
-      <c r="E21" s="362" t="inlineStr">
-        <is>
-          <t>KULLANILAN SAYFALAR</t>
-        </is>
-      </c>
-      <c r="F21" s="362" t="inlineStr">
-        <is>
-          <t>DOĞRUDAN ERİŞİM BUTONU</t>
+      <c r="D21" s="444" t="inlineStr">
+        <is>
+          <t>İŞLEM DETAYI VE YALIN MANTIK</t>
+        </is>
+      </c>
+      <c r="N21" s="443" t="inlineStr">
+        <is>
+          <t>İLGİLİ SAYFALAR</t>
+        </is>
+      </c>
+      <c r="P21" s="443" t="inlineStr">
+        <is>
+          <t>HIZLI ERİŞİM</t>
         </is>
       </c>
     </row>
     <row r="22" ht="36" customHeight="1" s="50">
-      <c r="B22" s="363" t="inlineStr">
+      <c r="B22" s="445" t="inlineStr">
         <is>
           <t>AŞAMA 1</t>
         </is>
       </c>
-      <c r="C22" s="341" t="inlineStr">
+      <c r="C22" s="446" t="inlineStr">
         <is>
           <t>SİSTEM KURULUMU &amp; PARAMETRELER</t>
         </is>
       </c>
-      <c r="D22" s="364" t="inlineStr">
-        <is>
-          <t>Şirket unvanı, raporlama tarihi, serbest nakit ve risk toleranslarını AYARLAR sekmesinden tanımlayın.</t>
-        </is>
-      </c>
-      <c r="E22" s="336" t="n"/>
-      <c r="F22" s="336" t="n"/>
-      <c r="G22" s="336" t="n"/>
-      <c r="H22" s="336" t="n"/>
-      <c r="I22" s="336" t="n"/>
-      <c r="J22" s="336" t="n"/>
-      <c r="K22" s="336" t="n"/>
-      <c r="L22" s="336" t="n"/>
-      <c r="M22" s="337" t="n"/>
-      <c r="N22" s="343" t="inlineStr">
+      <c r="D22" s="447" t="inlineStr">
+        <is>
+          <t>Şirket unvanı, raporlama tarihi, serbest nakit ve risk toleranslarını tanımlayın.</t>
+        </is>
+      </c>
+      <c r="E22" s="303" t="n"/>
+      <c r="F22" s="303" t="n"/>
+      <c r="G22" s="303" t="n"/>
+      <c r="H22" s="303" t="n"/>
+      <c r="I22" s="303" t="n"/>
+      <c r="J22" s="303" t="n"/>
+      <c r="K22" s="303" t="n"/>
+      <c r="L22" s="303" t="n"/>
+      <c r="M22" s="303" t="n"/>
+      <c r="N22" s="448" t="inlineStr">
         <is>
           <t>AYARLAR, LISTELER</t>
         </is>
       </c>
-      <c r="O22" s="337" t="n"/>
-      <c r="P22" s="344" t="inlineStr">
+      <c r="O22" s="303" t="n"/>
+      <c r="P22" s="449" t="inlineStr">
         <is>
           <t>⚙ AYARLAR (#AYARLAR!A1)</t>
         </is>
       </c>
-      <c r="Q22" s="336" t="n"/>
-      <c r="R22" s="337" t="n"/>
+      <c r="Q22" s="303" t="n"/>
+      <c r="R22" s="303" t="n"/>
     </row>
     <row r="23" ht="36" customHeight="1" s="50">
-      <c r="B23" s="366" t="inlineStr">
+      <c r="B23" s="450" t="inlineStr">
         <is>
           <t>AŞAMA 2</t>
         </is>
       </c>
-      <c r="C23" s="346" t="inlineStr">
+      <c r="C23" s="451" t="inlineStr">
         <is>
           <t>STRATEJİK KOKPİT &amp; İZLEME</t>
         </is>
       </c>
-      <c r="D23" s="367" t="inlineStr">
-        <is>
-          <t>Kredi portföy büyüklüğü, 30 günlük ödeme baskısı ve likidite erken uyarı radarını tek ekrandan izleyin.</t>
-        </is>
-      </c>
-      <c r="E23" s="336" t="n"/>
-      <c r="F23" s="336" t="n"/>
-      <c r="G23" s="336" t="n"/>
-      <c r="H23" s="336" t="n"/>
-      <c r="I23" s="336" t="n"/>
-      <c r="J23" s="336" t="n"/>
-      <c r="K23" s="336" t="n"/>
-      <c r="L23" s="336" t="n"/>
-      <c r="M23" s="337" t="n"/>
-      <c r="N23" s="348" t="inlineStr">
+      <c r="D23" s="452" t="inlineStr">
+        <is>
+          <t>Kredi portföy büyüklüğü, 30 günlük ödeme baskısı ve likidite radarını tek ekrandan izleyin.</t>
+        </is>
+      </c>
+      <c r="E23" s="303" t="n"/>
+      <c r="F23" s="303" t="n"/>
+      <c r="G23" s="303" t="n"/>
+      <c r="H23" s="303" t="n"/>
+      <c r="I23" s="303" t="n"/>
+      <c r="J23" s="303" t="n"/>
+      <c r="K23" s="303" t="n"/>
+      <c r="L23" s="303" t="n"/>
+      <c r="M23" s="303" t="n"/>
+      <c r="N23" s="453" t="inlineStr">
         <is>
           <t>PANO</t>
         </is>
       </c>
-      <c r="O23" s="337" t="n"/>
-      <c r="P23" s="344" t="inlineStr">
+      <c r="O23" s="303" t="n"/>
+      <c r="P23" s="449" t="inlineStr">
         <is>
           <t>▶ PANO KOKPİTİ (#PANO!A1)</t>
         </is>
       </c>
-      <c r="Q23" s="336" t="n"/>
-      <c r="R23" s="337" t="n"/>
+      <c r="Q23" s="303" t="n"/>
+      <c r="R23" s="303" t="n"/>
     </row>
     <row r="24" ht="36" customHeight="1" s="50">
-      <c r="B24" s="363" t="inlineStr">
+      <c r="B24" s="445" t="inlineStr">
         <is>
           <t>AŞAMA 3</t>
         </is>
       </c>
-      <c r="C24" s="341" t="inlineStr">
+      <c r="C24" s="446" t="inlineStr">
         <is>
           <t>PORTFÖY VE TAKSİT GİRİŞİ</t>
         </is>
       </c>
-      <c r="D24" s="364" t="inlineStr">
+      <c r="D24" s="447" t="inlineStr">
         <is>
           <t>Banka limitlerini, çekilen kredileri ve sözleşme amortisman takvimlerini ilgili sayfalara girin.</t>
         </is>
       </c>
-      <c r="E24" s="336" t="n"/>
-      <c r="F24" s="336" t="n"/>
-      <c r="G24" s="336" t="n"/>
-      <c r="H24" s="336" t="n"/>
-      <c r="I24" s="336" t="n"/>
-      <c r="J24" s="336" t="n"/>
-      <c r="K24" s="336" t="n"/>
-      <c r="L24" s="336" t="n"/>
-      <c r="M24" s="337" t="n"/>
-      <c r="N24" s="343" t="inlineStr">
-        <is>
-          <t>GİRDİLER, KREDILER, TAKSIT_PLANI</t>
-        </is>
-      </c>
-      <c r="O24" s="337" t="n"/>
-      <c r="P24" s="344" t="inlineStr">
+      <c r="E24" s="303" t="n"/>
+      <c r="F24" s="303" t="n"/>
+      <c r="G24" s="303" t="n"/>
+      <c r="H24" s="303" t="n"/>
+      <c r="I24" s="303" t="n"/>
+      <c r="J24" s="303" t="n"/>
+      <c r="K24" s="303" t="n"/>
+      <c r="L24" s="303" t="n"/>
+      <c r="M24" s="303" t="n"/>
+      <c r="N24" s="448" t="inlineStr">
+        <is>
+          <t>GİRDİLER, KREDİLER</t>
+        </is>
+      </c>
+      <c r="O24" s="303" t="n"/>
+      <c r="P24" s="449" t="inlineStr">
         <is>
           <t>📋 GİRİŞLERİ DÜZENLE (#GİRDİLER!A1)</t>
         </is>
       </c>
-      <c r="Q24" s="336" t="n"/>
-      <c r="R24" s="337" t="n"/>
+      <c r="Q24" s="303" t="n"/>
+      <c r="R24" s="303" t="n"/>
     </row>
     <row r="25" ht="36" customHeight="1" s="50">
-      <c r="B25" s="366" t="inlineStr">
+      <c r="B25" s="450" t="inlineStr">
         <is>
           <t>AŞAMA 4</t>
         </is>
       </c>
-      <c r="C25" s="346" t="inlineStr">
+      <c r="C25" s="451" t="inlineStr">
         <is>
           <t>REFİNANSMAN VE STRES TESTİ</t>
         </is>
       </c>
-      <c r="D25" s="367" t="inlineStr">
-        <is>
-          <t>Krediyi başka bankaya taşıma durumunda net faiz kârını hesaplayın. -%20 nakit daralması stres testini inceleyin.</t>
-        </is>
-      </c>
-      <c r="E25" s="336" t="n"/>
-      <c r="F25" s="336" t="n"/>
-      <c r="G25" s="336" t="n"/>
-      <c r="H25" s="336" t="n"/>
-      <c r="I25" s="336" t="n"/>
-      <c r="J25" s="336" t="n"/>
-      <c r="K25" s="336" t="n"/>
-      <c r="L25" s="336" t="n"/>
-      <c r="M25" s="337" t="n"/>
-      <c r="N25" s="348" t="inlineStr">
-        <is>
-          <t>REFINANSMAN, YÖNETİM_RAPORU</t>
-        </is>
-      </c>
-      <c r="O25" s="337" t="n"/>
-      <c r="P25" s="344" t="inlineStr">
+      <c r="D25" s="452" t="inlineStr">
+        <is>
+          <t>Krediyi başka bankaya taşıma faiz kârını hesaplayın. -%20 nakit daralması kriz testini inceleyin.</t>
+        </is>
+      </c>
+      <c r="E25" s="303" t="n"/>
+      <c r="F25" s="303" t="n"/>
+      <c r="G25" s="303" t="n"/>
+      <c r="H25" s="303" t="n"/>
+      <c r="I25" s="303" t="n"/>
+      <c r="J25" s="303" t="n"/>
+      <c r="K25" s="303" t="n"/>
+      <c r="L25" s="303" t="n"/>
+      <c r="M25" s="303" t="n"/>
+      <c r="N25" s="453" t="inlineStr">
+        <is>
+          <t>REFİNANSMAN, RAPOR</t>
+        </is>
+      </c>
+      <c r="O25" s="303" t="n"/>
+      <c r="P25" s="449" t="inlineStr">
         <is>
           <t>📊 STRES TESTİ (#YÖNETİM_RAPORU!A1)</t>
         </is>
       </c>
-      <c r="Q25" s="336" t="n"/>
-      <c r="R25" s="337" t="n"/>
+      <c r="Q25" s="303" t="n"/>
+      <c r="R25" s="303" t="n"/>
     </row>
     <row r="26" ht="36" customHeight="1" s="50">
-      <c r="B26" s="363" t="inlineStr">
+      <c r="B26" s="445" t="inlineStr">
         <is>
           <t>AŞAMA 5</t>
         </is>
       </c>
-      <c r="C26" s="341" t="inlineStr">
+      <c r="C26" s="446" t="inlineStr">
         <is>
           <t>YÖNETİM KURULU VE BANKA ÇIKTISI</t>
         </is>
       </c>
-      <c r="D26" s="364" t="inlineStr">
+      <c r="D26" s="447" t="inlineStr">
         <is>
           <t>Kredi komiteleri ve yönetim kuruluna sunulacak A4 dikey baskıya hazır kurumsal rapor çıktısını alın.</t>
         </is>
       </c>
-      <c r="E26" s="336" t="n"/>
-      <c r="F26" s="336" t="n"/>
-      <c r="G26" s="336" t="n"/>
-      <c r="H26" s="336" t="n"/>
-      <c r="I26" s="336" t="n"/>
-      <c r="J26" s="336" t="n"/>
-      <c r="K26" s="336" t="n"/>
-      <c r="L26" s="336" t="n"/>
-      <c r="M26" s="337" t="n"/>
-      <c r="N26" s="343" t="inlineStr">
+      <c r="E26" s="303" t="n"/>
+      <c r="F26" s="303" t="n"/>
+      <c r="G26" s="303" t="n"/>
+      <c r="H26" s="303" t="n"/>
+      <c r="I26" s="303" t="n"/>
+      <c r="J26" s="303" t="n"/>
+      <c r="K26" s="303" t="n"/>
+      <c r="L26" s="303" t="n"/>
+      <c r="M26" s="303" t="n"/>
+      <c r="N26" s="448" t="inlineStr">
         <is>
           <t>RAPOR</t>
         </is>
       </c>
-      <c r="O26" s="337" t="n"/>
-      <c r="P26" s="344" t="inlineStr">
+      <c r="O26" s="303" t="n"/>
+      <c r="P26" s="449" t="inlineStr">
         <is>
           <t>📄 A4 RAPORU (#RAPOR!A1)</t>
         </is>
       </c>
-      <c r="Q26" s="336" t="n"/>
-      <c r="R26" s="337" t="n"/>
+      <c r="Q26" s="303" t="n"/>
+      <c r="R26" s="303" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="27">
     <mergeCell ref="N26:O26"/>
+    <mergeCell ref="P21:R21"/>
     <mergeCell ref="B2:M2"/>
     <mergeCell ref="B4:R4"/>
     <mergeCell ref="N25:O25"/>
@@ -14301,14 +14333,16 @@
     <mergeCell ref="D24:M24"/>
     <mergeCell ref="N22:O22"/>
     <mergeCell ref="D23:M23"/>
+    <mergeCell ref="N21:O21"/>
     <mergeCell ref="I14:K14"/>
     <mergeCell ref="D26:M26"/>
     <mergeCell ref="O9:Q12"/>
     <mergeCell ref="N23:O23"/>
     <mergeCell ref="O14:Q14"/>
+    <mergeCell ref="P24:R24"/>
     <mergeCell ref="D22:M22"/>
-    <mergeCell ref="P24:R24"/>
     <mergeCell ref="C9:E12"/>
+    <mergeCell ref="D21:M21"/>
     <mergeCell ref="P26:R26"/>
     <mergeCell ref="C14:E14"/>
     <mergeCell ref="P25:R25"/>
@@ -14337,7 +14371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13.5" customWidth="1" style="76" min="1" max="2"/>
@@ -14974,7 +15008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14.5" customWidth="1" style="76" min="1" max="1"/>
@@ -15652,7 +15686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13.5" customWidth="1" style="76" min="1" max="1"/>
@@ -16523,7 +16557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="76" min="1" max="1"/>
@@ -25039,7 +25073,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M27"/>
+  <dimension ref="A1:N52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.5" customWidth="1" style="50" min="1" max="1"/>
@@ -25589,32 +25623,382 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="10" customHeight="1" s="50">
+    <row r="27" ht="14" customHeight="1" s="50">
       <c r="F27" s="249" t="n"/>
       <c r="G27" s="250" t="n"/>
       <c r="H27" s="250" t="n"/>
       <c r="I27" s="251" t="n"/>
     </row>
-    <row r="28" ht="18" customHeight="1" s="50"/>
-    <row r="29" ht="18" customHeight="1" s="50"/>
-    <row r="30" ht="18" customHeight="1" s="50"/>
-    <row r="31" ht="18" customHeight="1" s="50"/>
-    <row r="32" ht="18" customHeight="1" s="50"/>
-    <row r="33" ht="18" customHeight="1" s="50"/>
-    <row r="34" ht="18" customHeight="1" s="50"/>
-    <row r="35" ht="18" customHeight="1" s="50"/>
-    <row r="36" ht="18" customHeight="1" s="50"/>
-    <row r="37" ht="18" customHeight="1" s="50"/>
-    <row r="38" ht="18" customHeight="1" s="50"/>
-    <row r="39" ht="18" customHeight="1" s="50"/>
-    <row r="40" ht="18" customHeight="1" s="50"/>
-    <row r="41" ht="18" customHeight="1" s="50"/>
-    <row r="42" ht="18" customHeight="1" s="50"/>
-    <row r="43" ht="18" customHeight="1" s="50"/>
-    <row r="44" ht="18" customHeight="1" s="50"/>
-    <row r="45" ht="18" customHeight="1" s="50"/>
-    <row r="46" ht="18" customHeight="1" s="50"/>
-    <row r="47" ht="18" customHeight="1" s="50"/>
+    <row r="28" ht="14" customHeight="1" s="50"/>
+    <row r="29" ht="14" customHeight="1" s="50"/>
+    <row r="30" ht="18" customHeight="1" s="50">
+      <c r="A30" s="454" t="n"/>
+      <c r="B30" s="454" t="n"/>
+      <c r="C30" s="454" t="n"/>
+      <c r="D30" s="454" t="n"/>
+      <c r="E30" s="454" t="n"/>
+      <c r="F30" s="454" t="n"/>
+      <c r="G30" s="454" t="n"/>
+      <c r="H30" s="454" t="n"/>
+      <c r="I30" s="454" t="n"/>
+      <c r="J30" s="454" t="n"/>
+      <c r="K30" s="454" t="n"/>
+      <c r="L30" s="454" t="n"/>
+      <c r="M30" s="454" t="n"/>
+      <c r="N30" s="454" t="n"/>
+    </row>
+    <row r="31" ht="18" customHeight="1" s="50">
+      <c r="A31" s="454" t="n"/>
+      <c r="B31" s="454" t="n"/>
+      <c r="C31" s="454" t="n"/>
+      <c r="D31" s="454" t="n"/>
+      <c r="E31" s="454" t="n"/>
+      <c r="F31" s="454" t="n"/>
+      <c r="G31" s="454" t="n"/>
+      <c r="H31" s="454" t="n"/>
+      <c r="I31" s="454" t="n"/>
+      <c r="J31" s="454" t="n"/>
+      <c r="K31" s="454" t="n"/>
+      <c r="L31" s="454" t="n"/>
+      <c r="M31" s="454" t="n"/>
+      <c r="N31" s="454" t="n"/>
+    </row>
+    <row r="32" ht="18" customHeight="1" s="50">
+      <c r="A32" s="454" t="n"/>
+      <c r="B32" s="454" t="n"/>
+      <c r="C32" s="454" t="n"/>
+      <c r="D32" s="454" t="n"/>
+      <c r="E32" s="454" t="n"/>
+      <c r="F32" s="454" t="n"/>
+      <c r="G32" s="454" t="n"/>
+      <c r="H32" s="454" t="n"/>
+      <c r="I32" s="454" t="n"/>
+      <c r="J32" s="454" t="n"/>
+      <c r="K32" s="454" t="n"/>
+      <c r="L32" s="454" t="n"/>
+      <c r="M32" s="454" t="n"/>
+      <c r="N32" s="454" t="n"/>
+    </row>
+    <row r="33" ht="18" customHeight="1" s="50">
+      <c r="A33" s="454" t="n"/>
+      <c r="B33" s="454" t="n"/>
+      <c r="C33" s="454" t="n"/>
+      <c r="D33" s="454" t="n"/>
+      <c r="E33" s="454" t="n"/>
+      <c r="F33" s="454" t="n"/>
+      <c r="G33" s="454" t="n"/>
+      <c r="H33" s="454" t="n"/>
+      <c r="I33" s="454" t="n"/>
+      <c r="J33" s="454" t="n"/>
+      <c r="K33" s="454" t="n"/>
+      <c r="L33" s="454" t="n"/>
+      <c r="M33" s="454" t="n"/>
+      <c r="N33" s="454" t="n"/>
+    </row>
+    <row r="34" ht="18" customHeight="1" s="50">
+      <c r="A34" s="454" t="n"/>
+      <c r="B34" s="454" t="n"/>
+      <c r="C34" s="454" t="n"/>
+      <c r="D34" s="454" t="n"/>
+      <c r="E34" s="454" t="n"/>
+      <c r="F34" s="454" t="n"/>
+      <c r="G34" s="454" t="n"/>
+      <c r="H34" s="454" t="n"/>
+      <c r="I34" s="454" t="n"/>
+      <c r="J34" s="454" t="n"/>
+      <c r="K34" s="454" t="n"/>
+      <c r="L34" s="454" t="n"/>
+      <c r="M34" s="454" t="n"/>
+      <c r="N34" s="454" t="n"/>
+    </row>
+    <row r="35" ht="18" customHeight="1" s="50">
+      <c r="A35" s="454" t="n"/>
+      <c r="B35" s="454" t="n"/>
+      <c r="C35" s="454" t="n"/>
+      <c r="D35" s="454" t="n"/>
+      <c r="E35" s="454" t="n"/>
+      <c r="F35" s="454" t="n"/>
+      <c r="G35" s="454" t="n"/>
+      <c r="H35" s="454" t="n"/>
+      <c r="I35" s="454" t="n"/>
+      <c r="J35" s="454" t="n"/>
+      <c r="K35" s="454" t="n"/>
+      <c r="L35" s="454" t="n"/>
+      <c r="M35" s="454" t="n"/>
+      <c r="N35" s="454" t="n"/>
+    </row>
+    <row r="36" ht="18" customHeight="1" s="50">
+      <c r="A36" s="454" t="n"/>
+      <c r="B36" s="454" t="n"/>
+      <c r="C36" s="454" t="n"/>
+      <c r="D36" s="454" t="n"/>
+      <c r="E36" s="454" t="n"/>
+      <c r="F36" s="454" t="n"/>
+      <c r="G36" s="454" t="n"/>
+      <c r="H36" s="454" t="n"/>
+      <c r="I36" s="454" t="n"/>
+      <c r="J36" s="454" t="n"/>
+      <c r="K36" s="454" t="n"/>
+      <c r="L36" s="454" t="n"/>
+      <c r="M36" s="454" t="n"/>
+      <c r="N36" s="454" t="n"/>
+    </row>
+    <row r="37" ht="18" customHeight="1" s="50">
+      <c r="A37" s="454" t="n"/>
+      <c r="B37" s="454" t="n"/>
+      <c r="C37" s="454" t="n"/>
+      <c r="D37" s="454" t="n"/>
+      <c r="E37" s="454" t="n"/>
+      <c r="F37" s="454" t="n"/>
+      <c r="G37" s="454" t="n"/>
+      <c r="H37" s="454" t="n"/>
+      <c r="I37" s="454" t="n"/>
+      <c r="J37" s="454" t="n"/>
+      <c r="K37" s="454" t="n"/>
+      <c r="L37" s="454" t="n"/>
+      <c r="M37" s="454" t="n"/>
+      <c r="N37" s="454" t="n"/>
+    </row>
+    <row r="38" ht="18" customHeight="1" s="50">
+      <c r="A38" s="454" t="n"/>
+      <c r="B38" s="454" t="n"/>
+      <c r="C38" s="454" t="n"/>
+      <c r="D38" s="454" t="n"/>
+      <c r="E38" s="454" t="n"/>
+      <c r="F38" s="454" t="n"/>
+      <c r="G38" s="454" t="n"/>
+      <c r="H38" s="454" t="n"/>
+      <c r="I38" s="454" t="n"/>
+      <c r="J38" s="454" t="n"/>
+      <c r="K38" s="454" t="n"/>
+      <c r="L38" s="454" t="n"/>
+      <c r="M38" s="454" t="n"/>
+      <c r="N38" s="454" t="n"/>
+    </row>
+    <row r="39" ht="18" customHeight="1" s="50">
+      <c r="A39" s="454" t="n"/>
+      <c r="B39" s="454" t="n"/>
+      <c r="C39" s="454" t="n"/>
+      <c r="D39" s="454" t="n"/>
+      <c r="E39" s="454" t="n"/>
+      <c r="F39" s="454" t="n"/>
+      <c r="G39" s="454" t="n"/>
+      <c r="H39" s="454" t="n"/>
+      <c r="I39" s="454" t="n"/>
+      <c r="J39" s="454" t="n"/>
+      <c r="K39" s="454" t="n"/>
+      <c r="L39" s="454" t="n"/>
+      <c r="M39" s="454" t="n"/>
+      <c r="N39" s="454" t="n"/>
+    </row>
+    <row r="40" ht="18" customHeight="1" s="50">
+      <c r="A40" s="454" t="n"/>
+      <c r="B40" s="454" t="n"/>
+      <c r="C40" s="454" t="n"/>
+      <c r="D40" s="454" t="n"/>
+      <c r="E40" s="454" t="n"/>
+      <c r="F40" s="454" t="n"/>
+      <c r="G40" s="454" t="n"/>
+      <c r="H40" s="454" t="n"/>
+      <c r="I40" s="454" t="n"/>
+      <c r="J40" s="454" t="n"/>
+      <c r="K40" s="454" t="n"/>
+      <c r="L40" s="454" t="n"/>
+      <c r="M40" s="454" t="n"/>
+      <c r="N40" s="454" t="n"/>
+    </row>
+    <row r="41" ht="18" customHeight="1" s="50">
+      <c r="A41" s="454" t="n"/>
+      <c r="B41" s="454" t="n"/>
+      <c r="C41" s="454" t="n"/>
+      <c r="D41" s="454" t="n"/>
+      <c r="E41" s="454" t="n"/>
+      <c r="F41" s="454" t="n"/>
+      <c r="G41" s="454" t="n"/>
+      <c r="H41" s="454" t="n"/>
+      <c r="I41" s="454" t="n"/>
+      <c r="J41" s="454" t="n"/>
+      <c r="K41" s="454" t="n"/>
+      <c r="L41" s="454" t="n"/>
+      <c r="M41" s="454" t="n"/>
+      <c r="N41" s="454" t="n"/>
+    </row>
+    <row r="42" ht="18" customHeight="1" s="50">
+      <c r="A42" s="454" t="n"/>
+      <c r="B42" s="454" t="n"/>
+      <c r="C42" s="454" t="n"/>
+      <c r="D42" s="454" t="n"/>
+      <c r="E42" s="454" t="n"/>
+      <c r="F42" s="454" t="n"/>
+      <c r="G42" s="454" t="n"/>
+      <c r="H42" s="454" t="n"/>
+      <c r="I42" s="454" t="n"/>
+      <c r="J42" s="454" t="n"/>
+      <c r="K42" s="454" t="n"/>
+      <c r="L42" s="454" t="n"/>
+      <c r="M42" s="454" t="n"/>
+      <c r="N42" s="454" t="n"/>
+    </row>
+    <row r="43" ht="18" customHeight="1" s="50">
+      <c r="A43" s="454" t="n"/>
+      <c r="B43" s="454" t="n"/>
+      <c r="C43" s="454" t="n"/>
+      <c r="D43" s="454" t="n"/>
+      <c r="E43" s="454" t="n"/>
+      <c r="F43" s="454" t="n"/>
+      <c r="G43" s="454" t="n"/>
+      <c r="H43" s="454" t="n"/>
+      <c r="I43" s="454" t="n"/>
+      <c r="J43" s="454" t="n"/>
+      <c r="K43" s="454" t="n"/>
+      <c r="L43" s="454" t="n"/>
+      <c r="M43" s="454" t="n"/>
+      <c r="N43" s="454" t="n"/>
+    </row>
+    <row r="44" ht="18" customHeight="1" s="50">
+      <c r="A44" s="454" t="n"/>
+      <c r="B44" s="454" t="n"/>
+      <c r="C44" s="454" t="n"/>
+      <c r="D44" s="454" t="n"/>
+      <c r="E44" s="454" t="n"/>
+      <c r="F44" s="454" t="n"/>
+      <c r="G44" s="454" t="n"/>
+      <c r="H44" s="454" t="n"/>
+      <c r="I44" s="454" t="n"/>
+      <c r="J44" s="454" t="n"/>
+      <c r="K44" s="454" t="n"/>
+      <c r="L44" s="454" t="n"/>
+      <c r="M44" s="454" t="n"/>
+      <c r="N44" s="454" t="n"/>
+    </row>
+    <row r="45" ht="18" customHeight="1" s="50">
+      <c r="A45" s="454" t="n"/>
+      <c r="B45" s="454" t="n"/>
+      <c r="C45" s="454" t="n"/>
+      <c r="D45" s="454" t="n"/>
+      <c r="E45" s="454" t="n"/>
+      <c r="F45" s="454" t="n"/>
+      <c r="G45" s="454" t="n"/>
+      <c r="H45" s="454" t="n"/>
+      <c r="I45" s="454" t="n"/>
+      <c r="J45" s="454" t="n"/>
+      <c r="K45" s="454" t="n"/>
+      <c r="L45" s="454" t="n"/>
+      <c r="M45" s="454" t="n"/>
+      <c r="N45" s="454" t="n"/>
+    </row>
+    <row r="46" ht="18" customHeight="1" s="50">
+      <c r="A46" s="454" t="n"/>
+      <c r="B46" s="454" t="n"/>
+      <c r="C46" s="454" t="n"/>
+      <c r="D46" s="454" t="n"/>
+      <c r="E46" s="454" t="n"/>
+      <c r="F46" s="454" t="n"/>
+      <c r="G46" s="454" t="n"/>
+      <c r="H46" s="454" t="n"/>
+      <c r="I46" s="454" t="n"/>
+      <c r="J46" s="454" t="n"/>
+      <c r="K46" s="454" t="n"/>
+      <c r="L46" s="454" t="n"/>
+      <c r="M46" s="454" t="n"/>
+      <c r="N46" s="454" t="n"/>
+    </row>
+    <row r="47" ht="18" customHeight="1" s="50">
+      <c r="A47" s="454" t="n"/>
+      <c r="B47" s="454" t="n"/>
+      <c r="C47" s="454" t="n"/>
+      <c r="D47" s="454" t="n"/>
+      <c r="E47" s="454" t="n"/>
+      <c r="F47" s="454" t="n"/>
+      <c r="G47" s="454" t="n"/>
+      <c r="H47" s="454" t="n"/>
+      <c r="I47" s="454" t="n"/>
+      <c r="J47" s="454" t="n"/>
+      <c r="K47" s="454" t="n"/>
+      <c r="L47" s="454" t="n"/>
+      <c r="M47" s="454" t="n"/>
+      <c r="N47" s="454" t="n"/>
+    </row>
+    <row r="48" ht="18" customHeight="1" s="50">
+      <c r="A48" s="454" t="n"/>
+      <c r="B48" s="454" t="n"/>
+      <c r="C48" s="454" t="n"/>
+      <c r="D48" s="454" t="n"/>
+      <c r="E48" s="454" t="n"/>
+      <c r="F48" s="454" t="n"/>
+      <c r="G48" s="454" t="n"/>
+      <c r="H48" s="454" t="n"/>
+      <c r="I48" s="454" t="n"/>
+      <c r="J48" s="454" t="n"/>
+      <c r="K48" s="454" t="n"/>
+      <c r="L48" s="454" t="n"/>
+      <c r="M48" s="454" t="n"/>
+      <c r="N48" s="454" t="n"/>
+    </row>
+    <row r="49" ht="18" customHeight="1" s="50">
+      <c r="A49" s="454" t="n"/>
+      <c r="B49" s="454" t="n"/>
+      <c r="C49" s="454" t="n"/>
+      <c r="D49" s="454" t="n"/>
+      <c r="E49" s="454" t="n"/>
+      <c r="F49" s="454" t="n"/>
+      <c r="G49" s="454" t="n"/>
+      <c r="H49" s="454" t="n"/>
+      <c r="I49" s="454" t="n"/>
+      <c r="J49" s="454" t="n"/>
+      <c r="K49" s="454" t="n"/>
+      <c r="L49" s="454" t="n"/>
+      <c r="M49" s="454" t="n"/>
+      <c r="N49" s="454" t="n"/>
+    </row>
+    <row r="50" ht="18" customHeight="1" s="50">
+      <c r="A50" s="454" t="n"/>
+      <c r="B50" s="454" t="n"/>
+      <c r="C50" s="454" t="n"/>
+      <c r="D50" s="454" t="n"/>
+      <c r="E50" s="454" t="n"/>
+      <c r="F50" s="454" t="n"/>
+      <c r="G50" s="454" t="n"/>
+      <c r="H50" s="454" t="n"/>
+      <c r="I50" s="454" t="n"/>
+      <c r="J50" s="454" t="n"/>
+      <c r="K50" s="454" t="n"/>
+      <c r="L50" s="454" t="n"/>
+      <c r="M50" s="454" t="n"/>
+      <c r="N50" s="454" t="n"/>
+    </row>
+    <row r="51" ht="18" customHeight="1" s="50">
+      <c r="A51" s="454" t="n"/>
+      <c r="B51" s="454" t="n"/>
+      <c r="C51" s="454" t="n"/>
+      <c r="D51" s="454" t="n"/>
+      <c r="E51" s="454" t="n"/>
+      <c r="F51" s="454" t="n"/>
+      <c r="G51" s="454" t="n"/>
+      <c r="H51" s="454" t="n"/>
+      <c r="I51" s="454" t="n"/>
+      <c r="J51" s="454" t="n"/>
+      <c r="K51" s="454" t="n"/>
+      <c r="L51" s="454" t="n"/>
+      <c r="M51" s="454" t="n"/>
+      <c r="N51" s="454" t="n"/>
+    </row>
+    <row r="52" ht="18" customHeight="1" s="50">
+      <c r="A52" s="454" t="n"/>
+      <c r="B52" s="454" t="n"/>
+      <c r="C52" s="454" t="n"/>
+      <c r="D52" s="454" t="n"/>
+      <c r="E52" s="454" t="n"/>
+      <c r="F52" s="454" t="n"/>
+      <c r="G52" s="454" t="n"/>
+      <c r="H52" s="454" t="n"/>
+      <c r="I52" s="454" t="n"/>
+      <c r="J52" s="454" t="n"/>
+      <c r="K52" s="454" t="n"/>
+      <c r="L52" s="454" t="n"/>
+      <c r="M52" s="454" t="n"/>
+      <c r="N52" s="454" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="B2:M2"/>
@@ -26731,7 +27115,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="76" min="1" max="1"/>
@@ -27401,7 +27785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="76" min="1" max="1"/>
@@ -29272,7 +29656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="13" customWidth="1" style="76" min="1" max="2"/>
@@ -30272,7 +30656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="76" min="1" max="1"/>

</xml_diff>